<commit_message>
Update calibration reports after post-wiring audit test run
Auto-regenerated by running full test suite during Stack I audit.
No model logic changed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8W8EHSADMzvD3ufdXTkMr
</commit_message>
<xml_diff>
--- a/reports/phase10_calibration_reconciliation_pack.xlsx
+++ b/reports/phase10_calibration_reconciliation_pack.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export_Metadata" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workbook_Index" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Navigation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Dashboard" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Signoff" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Governance Timeline" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Readiness Matrix" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runtime Summary" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Reconciliation" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CO2 &amp; Balancing Reconciliation" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPEX Reconciliation" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Senior Debt Reconciliation" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SHL Reconciliation" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tax R35-R67-R69" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFADS Waterfall" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Distributions Sponsor" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns Reconciliation" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IRR Reconciliation" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calibration Residual Closeout" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Register" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Inventory" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accepted Conventions" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reviewer Notes" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Export_Metadata" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Workbook_Index" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cover" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Navigation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Executive Dashboard" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Executive Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Review Signoff" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Governance" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Governance Timeline" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Readiness Matrix" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Runtime Summary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Revenue Reconciliation" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="CO2 &amp; Balancing Reconciliation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="OPEX Reconciliation" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Senior Debt Reconciliation" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="SHL Reconciliation" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Tax R35-R67-R69" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="CFADS Waterfall" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Distributions Sponsor" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Returns Reconciliation" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="IRR Reconciliation" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Calibration Residual Closeout" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Gap Register" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Source Inventory" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Accepted Conventions" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Reviewer Notes" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Cover'!$1:$4</definedName>
@@ -907,7 +907,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09T07:39:19+00:00</t>
+          <t>2026-07-01T14:45:00+00:00</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-09T07:39:19+00:00</t>
+          <t>2026-07-01T14:45:00+00:00</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09T07:39:19+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="F6" s="21" t="inlineStr">
         <is>
-          <t>Factory-bound active project runtime output.</t>
+          <t>Template-based active project runtime output.</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t>0.09410162472306152</t>
+          <t>0.0941016247230615</t>
         </is>
       </c>
       <c r="C7" s="21" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>0.11149507555645398</t>
+          <t>0.11149507555645395</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>423843.61137671326</t>
+          <t>423843.6113767133</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>338435.33724222926</t>
+          <t>338435.3372422292</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>85408.27413448403</t>
+          <t>85408.27413448405</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>173572.2883697887</t>
+          <t>173572.28836978864</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -2087,7 +2087,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CRuntime Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-06-09T07:39:19+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-01T14:45:00+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5911,7 +5911,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09T07:39:19+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCO2 &amp; Balancing Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-06-09T07:39:19+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -7111,7 +7111,7 @@
         <v>0</v>
       </c>
       <c r="BL6" s="48" t="n">
-        <v>84674.77873934135</v>
+        <v>84674.77873934136</v>
       </c>
       <c r="BM6" s="49" t="inlineStr"/>
       <c r="BN6" s="49" t="inlineStr"/>
@@ -7148,7 +7148,7 @@
         <v>1029.640710136986</v>
       </c>
       <c r="G7" s="51" t="n">
-        <v>1038.364049027322</v>
+        <v>1038.364049027323</v>
       </c>
       <c r="H7" s="51" t="n">
         <v>1049.774642972678</v>
@@ -7172,7 +7172,7 @@
         <v>1125.396386130107</v>
       </c>
       <c r="O7" s="51" t="n">
-        <v>1135.335091961179</v>
+        <v>1135.33509196118</v>
       </c>
       <c r="P7" s="51" t="n">
         <v>1147.811301762951</v>
@@ -7190,7 +7190,7 @@
         <v>1204.182948412321</v>
       </c>
       <c r="U7" s="51" t="n">
-        <v>1211.8158571116</v>
+        <v>1211.815857111599</v>
       </c>
       <c r="V7" s="51" t="n">
         <v>1231.901202809582</v>
@@ -7208,7 +7208,7 @@
         <v>1289.683567404981</v>
       </c>
       <c r="AA7" s="51" t="n">
-        <v>1298.287522344152</v>
+        <v>1298.287522344153</v>
       </c>
       <c r="AB7" s="51" t="n">
         <v>1319.806100062564</v>
@@ -7265,7 +7265,7 @@
         <v>1607.362542211412</v>
       </c>
       <c r="AT7" s="51" t="n">
-        <v>1634.003910314363</v>
+        <v>1634.003910314364</v>
       </c>
       <c r="AU7" s="51" t="n">
         <v>1651.7106902768</v>
@@ -7274,7 +7274,7 @@
         <v>1669.861357202919</v>
       </c>
       <c r="AW7" s="51" t="n">
-        <v>1688.161932882021</v>
+        <v>1688.16193288202</v>
       </c>
       <c r="AX7" s="51" t="n">
         <v>1716.142517404927</v>
@@ -7283,7 +7283,7 @@
         <v>1730.493671654745</v>
       </c>
       <c r="AZ7" s="51" t="n">
-        <v>1759.175887207033</v>
+        <v>1759.175887207034</v>
       </c>
       <c r="BA7" s="51" t="n">
         <v>1774.186155209829</v>
@@ -7292,7 +7292,7 @@
         <v>1803.592555572423</v>
       </c>
       <c r="BC7" s="51" t="n">
-        <v>1824.350591344815</v>
+        <v>1824.350591344816</v>
       </c>
       <c r="BD7" s="51" t="n">
         <v>1844.398400040913</v>
@@ -7304,7 +7304,7 @@
         <v>1896.814945307277</v>
       </c>
       <c r="BG7" s="51" t="n">
-        <v>1914.023920947863</v>
+        <v>1914.023920947864</v>
       </c>
       <c r="BH7" s="51" t="n">
         <v>1945.74807433374</v>
@@ -7319,7 +7319,7 @@
         <v>0</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>85408.27413448403</v>
+        <v>85408.27413448405</v>
       </c>
       <c r="BM7" s="67" t="inlineStr">
         <is>
@@ -7354,16 +7354,16 @@
         <v>-0.01865205479464294</v>
       </c>
       <c r="E8" s="51" t="n">
-        <v>6.27826021917781</v>
+        <v>6.278260219177923</v>
       </c>
       <c r="F8" s="51" t="n">
         <v>6.382319780821945</v>
       </c>
       <c r="G8" s="51" t="n">
-        <v>-29.29726223169405</v>
+        <v>-29.29726223169382</v>
       </c>
       <c r="H8" s="51" t="n">
-        <v>-29.61921016830593</v>
+        <v>-29.6192101683057</v>
       </c>
       <c r="I8" s="51" t="n">
         <v>-22.38516998555588</v>
@@ -7384,10 +7384,10 @@
         <v>-73.38013122957932</v>
       </c>
       <c r="O8" s="51" t="n">
-        <v>-64.62289266058406</v>
+        <v>-64.62289266058383</v>
       </c>
       <c r="P8" s="51" t="n">
-        <v>-65.33303433817309</v>
+        <v>-65.33303433817287</v>
       </c>
       <c r="Q8" s="51" t="n">
         <v>-56.3691684365424</v>
@@ -7402,10 +7402,10 @@
         <v>-48.7366412214792</v>
       </c>
       <c r="U8" s="51" t="n">
-        <v>-39.14395528476871</v>
+        <v>-39.14395528476894</v>
       </c>
       <c r="V8" s="51" t="n">
-        <v>-39.79275012374296</v>
+        <v>-39.79275012374319</v>
       </c>
       <c r="W8" s="51" t="n">
         <v>-51.1227619524268</v>
@@ -7414,16 +7414,16 @@
         <v>-51.68455054531091</v>
       </c>
       <c r="Y8" s="51" t="n">
-        <v>-41.38144986158272</v>
+        <v>-41.3814498615825</v>
       </c>
       <c r="Z8" s="51" t="n">
-        <v>-42.0673302460284</v>
+        <v>-42.06733024602818</v>
       </c>
       <c r="AA8" s="51" t="n">
-        <v>-31.34871023446908</v>
+        <v>-31.34871023446885</v>
       </c>
       <c r="AB8" s="51" t="n">
-        <v>-31.86830211680831</v>
+        <v>-31.86830211680808</v>
       </c>
       <c r="AC8" s="51" t="n">
         <v>-20.85981889187292</v>
@@ -7444,10 +7444,10 @@
         <v>-9.653714532892081</v>
       </c>
       <c r="AI8" s="51" t="n">
-        <v>2.796444279981415</v>
+        <v>2.796444279981642</v>
       </c>
       <c r="AJ8" s="51" t="n">
-        <v>2.842794185174171</v>
+        <v>2.842794185174398</v>
       </c>
       <c r="AK8" s="51" t="n">
         <v>15.65761977772536</v>
@@ -7468,16 +7468,16 @@
         <v>43.92606212195642</v>
       </c>
       <c r="AQ8" s="51" t="n">
-        <v>15.91632630585104</v>
+        <v>15.91632630585059</v>
       </c>
       <c r="AR8" s="51" t="n">
-        <v>16.18013281920776</v>
+        <v>16.1801328192073</v>
       </c>
       <c r="AS8" s="51" t="n">
-        <v>31.3766655497775</v>
+        <v>31.37666554977773</v>
       </c>
       <c r="AT8" s="51" t="n">
-        <v>31.89672077988416</v>
+        <v>31.89672077988439</v>
       </c>
       <c r="AU8" s="51" t="n">
         <v>47.71001702913213</v>
@@ -7486,40 +7486,40 @@
         <v>48.23430293055117</v>
       </c>
       <c r="AW8" s="51" t="n">
-        <v>64.56065108818825</v>
+        <v>64.5606510881878</v>
       </c>
       <c r="AX8" s="51" t="n">
-        <v>65.63071712832357</v>
+        <v>65.63071712832311</v>
       </c>
       <c r="AY8" s="51" t="n">
-        <v>82.36809901955621</v>
+        <v>82.36809901955644</v>
       </c>
       <c r="AZ8" s="51" t="n">
-        <v>83.73331613037749</v>
+        <v>83.73331613037772</v>
       </c>
       <c r="BA8" s="51" t="n">
-        <v>63.19944975207341</v>
+        <v>63.19944975207363</v>
       </c>
       <c r="BB8" s="51" t="n">
-        <v>64.24695444409645</v>
+        <v>64.24695444409667</v>
       </c>
       <c r="BC8" s="51" t="n">
-        <v>83.02563452885852</v>
+        <v>83.02563452885897</v>
       </c>
       <c r="BD8" s="51" t="n">
-        <v>83.93800413906592</v>
+        <v>83.93800413906638</v>
       </c>
       <c r="BE8" s="51" t="n">
-        <v>103.3614633929906</v>
+        <v>103.3614633929908</v>
       </c>
       <c r="BF8" s="51" t="n">
-        <v>105.0746368193945</v>
+        <v>105.0746368193948</v>
       </c>
       <c r="BG8" s="51" t="n">
-        <v>124.9508885557098</v>
+        <v>124.95088855571</v>
       </c>
       <c r="BH8" s="51" t="n">
-        <v>127.0218977582904</v>
+        <v>127.0218977582906</v>
       </c>
       <c r="BI8" s="51" t="n">
         <v>147.621154260306</v>
@@ -8771,7 +8771,7 @@
         <v>0</v>
       </c>
       <c r="BL14" s="48" t="n">
-        <v>339112.7082112872</v>
+        <v>339112.7082112871</v>
       </c>
       <c r="BM14" s="49" t="inlineStr"/>
       <c r="BN14" s="49" t="inlineStr"/>
@@ -8804,7 +8804,7 @@
         <v>3156.84179835198</v>
       </c>
       <c r="G15" s="51" t="n">
-        <v>3150.433824560011</v>
+        <v>3150.43382456001</v>
       </c>
       <c r="H15" s="51" t="n">
         <v>3185.053976478251</v>
@@ -8831,7 +8831,7 @@
         <v>3341.229727547581</v>
       </c>
       <c r="P15" s="51" t="n">
-        <v>3377.946537740412</v>
+        <v>3377.946537740411</v>
       </c>
       <c r="Q15" s="51" t="n">
         <v>3396.588882121361</v>
@@ -8849,7 +8849,7 @@
         <v>3533.181191458345</v>
       </c>
       <c r="V15" s="51" t="n">
-        <v>3591.74220568141</v>
+        <v>3591.742205681411</v>
       </c>
       <c r="W15" s="51" t="n">
         <v>3607.952524064416</v>
@@ -8858,7 +8858,7 @@
         <v>3647.600353999189</v>
       </c>
       <c r="Y15" s="51" t="n">
-        <v>3667.635538833557</v>
+        <v>3667.635538833556</v>
       </c>
       <c r="Z15" s="51" t="n">
         <v>3728.425078151239</v>
@@ -8930,13 +8930,13 @@
         <v>7456.637704174131</v>
       </c>
       <c r="AW15" s="51" t="n">
-        <v>7485.204790953595</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX15" s="51" t="n">
-        <v>7609.268958759456</v>
+        <v>7609.268958759457</v>
       </c>
       <c r="AY15" s="51" t="n">
-        <v>7616.439250274022</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ15" s="51" t="n">
         <v>7742.678574864201</v>
@@ -8948,7 +8948,7 @@
         <v>7934.089829742647</v>
       </c>
       <c r="BC15" s="51" t="n">
-        <v>7951.805783737153</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD15" s="51" t="n">
         <v>8039.188264877119</v>
@@ -8960,7 +8960,7 @@
         <v>8149.943887963956</v>
       </c>
       <c r="BG15" s="51" t="n">
-        <v>8093.726742854876</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH15" s="51" t="n">
         <v>8227.876909863522</v>
@@ -8975,7 +8975,7 @@
         <v>56.12442601729508</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>338435.3372422293</v>
+        <v>338435.3372422292</v>
       </c>
       <c r="BM15" s="53" t="inlineStr">
         <is>
@@ -9012,7 +9012,7 @@
         <v>-6.382319796672618</v>
       </c>
       <c r="G16" s="51" t="n">
-        <v>29.29726226411412</v>
+        <v>29.29726226411367</v>
       </c>
       <c r="H16" s="51" t="n">
         <v>29.61921020108139</v>
@@ -9039,7 +9039,7 @@
         <v>64.62289266058451</v>
       </c>
       <c r="P16" s="51" t="n">
-        <v>65.33303433817309</v>
+        <v>65.33303433817264</v>
       </c>
       <c r="Q16" s="51" t="n">
         <v>56.36916843654308</v>
@@ -9054,10 +9054,10 @@
         <v>48.73664122147966</v>
       </c>
       <c r="U16" s="51" t="n">
-        <v>39.14395528476916</v>
+        <v>39.14395528476962</v>
       </c>
       <c r="V16" s="51" t="n">
-        <v>39.79275012374364</v>
+        <v>39.7927501237441</v>
       </c>
       <c r="W16" s="51" t="n">
         <v>51.12276195242794</v>
@@ -9066,7 +9066,7 @@
         <v>51.68455054531159</v>
       </c>
       <c r="Y16" s="51" t="n">
-        <v>41.38144986158568</v>
+        <v>41.38144986158522</v>
       </c>
       <c r="Z16" s="51" t="n">
         <v>42.06733024603</v>
@@ -9138,13 +9138,13 @@
         <v>-48.23430293055117</v>
       </c>
       <c r="AW16" s="51" t="n">
-        <v>-64.56065108818802</v>
+        <v>-64.56065108818711</v>
       </c>
       <c r="AX16" s="51" t="n">
-        <v>-65.63071712832425</v>
+        <v>-65.63071712832334</v>
       </c>
       <c r="AY16" s="51" t="n">
-        <v>-82.36809901955621</v>
+        <v>-82.36809901955712</v>
       </c>
       <c r="AZ16" s="51" t="n">
         <v>-83.73331613037772</v>
@@ -9156,7 +9156,7 @@
         <v>-64.24695444409645</v>
       </c>
       <c r="BC16" s="51" t="n">
-        <v>-83.02563452885988</v>
+        <v>-83.02563452886079</v>
       </c>
       <c r="BD16" s="51" t="n">
         <v>-83.93800413906956</v>
@@ -9168,7 +9168,7 @@
         <v>-105.074636819395</v>
       </c>
       <c r="BG16" s="51" t="n">
-        <v>-124.9508885557088</v>
+        <v>-124.9508885557098</v>
       </c>
       <c r="BH16" s="51" t="n">
         <v>-127.0218977582899</v>
@@ -9888,7 +9888,7 @@
         <v>0</v>
       </c>
       <c r="BL6" s="48" t="n">
-        <v>756328.0823817673</v>
+        <v>756328.0823817672</v>
       </c>
       <c r="BM6" s="49" t="inlineStr"/>
       <c r="BN6" s="49" t="inlineStr"/>
@@ -10194,7 +10194,7 @@
         <v>1733.916326884588</v>
       </c>
       <c r="Z8" s="51" t="n">
-        <v>1874.767353856139</v>
+        <v>1874.767353856141</v>
       </c>
       <c r="AA8" s="51" t="n">
         <v>2017.495329935953</v>
@@ -10308,7 +10308,7 @@
         <v>0</v>
       </c>
       <c r="BL8" s="68" t="n">
-        <v>25146.29258193518</v>
+        <v>25146.2925819353</v>
       </c>
       <c r="BM8" s="67" t="inlineStr">
         <is>
@@ -10744,7 +10744,7 @@
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>22467.38828020644</v>
+        <v>22467.38828020645</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -10956,7 +10956,7 @@
         <v>0</v>
       </c>
       <c r="BL12" s="68" t="n">
-        <v>-355.4283885138502</v>
+        <v>-355.4283885138393</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -11263,7 +11263,7 @@
         <v>1562.92793164969</v>
       </c>
       <c r="U15" s="51" t="n">
-        <v>1614.127408287924</v>
+        <v>1614.127408287925</v>
       </c>
       <c r="V15" s="51" t="n">
         <v>1698.473876792322</v>
@@ -11275,7 +11275,7 @@
         <v>1834.031142387474</v>
       </c>
       <c r="Y15" s="51" t="n">
-        <v>1899.739863358543</v>
+        <v>1899.739863358542</v>
       </c>
       <c r="Z15" s="51" t="n">
         <v>1993.741499006938</v>
@@ -11460,7 +11460,7 @@
         <v>-60.40387274817022</v>
       </c>
       <c r="P16" s="51" t="n">
-        <v>-54.90965235037061</v>
+        <v>-54.90965235037106</v>
       </c>
       <c r="Q16" s="51" t="n">
         <v>-80.61471705150598</v>
@@ -11475,7 +11475,7 @@
         <v>-92.33355388440941</v>
       </c>
       <c r="U16" s="51" t="n">
-        <v>-116.6522892320186</v>
+        <v>-116.6522892320181</v>
       </c>
       <c r="V16" s="51" t="n">
         <v>-113.6277107302412</v>
@@ -11487,7 +11487,7 @@
         <v>-118.0128330985194</v>
       </c>
       <c r="Y16" s="51" t="n">
-        <v>-140.851026971548</v>
+        <v>-140.8510269715484</v>
       </c>
       <c r="Z16" s="51" t="n">
         <v>-142.7279760798131</v>
@@ -11604,7 +11604,7 @@
         <v>0</v>
       </c>
       <c r="BL16" s="68" t="n">
-        <v>0.4694318841065979</v>
+        <v>0.4694318841138738</v>
       </c>
       <c r="BM16" s="67" t="inlineStr">
         <is>
@@ -12480,7 +12480,7 @@
         <v>0</v>
       </c>
       <c r="BL22" s="48" t="n">
-        <v>712969.5518136515</v>
+        <v>712969.5518136513</v>
       </c>
       <c r="BM22" s="49" t="inlineStr"/>
       <c r="BN22" s="49" t="inlineStr"/>
@@ -12688,7 +12688,7 @@
         <v>0</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>738115.3749637025</v>
+        <v>738115.3749637026</v>
       </c>
       <c r="BM23" s="67" t="inlineStr">
         <is>
@@ -12783,7 +12783,7 @@
         <v>1733.916326884588</v>
       </c>
       <c r="Y24" s="51" t="n">
-        <v>1874.767353856139</v>
+        <v>1874.767353856141</v>
       </c>
       <c r="Z24" s="51" t="n">
         <v>2017.495329935953</v>
@@ -12900,7 +12900,7 @@
         <v>0</v>
       </c>
       <c r="BL24" s="68" t="n">
-        <v>25145.82315005106</v>
+        <v>25145.82315005129</v>
       </c>
       <c r="BM24" s="67" t="inlineStr">
         <is>
@@ -13281,7 +13281,7 @@
         <v>0.2552278573021478</v>
       </c>
       <c r="G28" s="75" t="n">
-        <v>0.2352910460430022</v>
+        <v>0.235291046043002</v>
       </c>
       <c r="H28" s="75" t="n">
         <v>0.2544170039600802</v>
@@ -13308,7 +13308,7 @@
         <v>-0.03798532063051097</v>
       </c>
       <c r="P28" s="75" t="n">
-        <v>-0.006115312196259826</v>
+        <v>-0.006115312196260048</v>
       </c>
       <c r="Q28" s="59" t="inlineStr">
         <is>
@@ -14223,7 +14223,7 @@
         <v>36259.81258005062</v>
       </c>
       <c r="V7" s="51" t="n">
-        <v>36441.58133164083</v>
+        <v>36441.58133164084</v>
       </c>
       <c r="W7" s="51" t="n">
         <v>36633.62919266382</v>
@@ -15121,7 +15121,7 @@
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>46045.27529548419</v>
+        <v>46045.27529548418</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -15333,7 +15333,7 @@
         <v>0</v>
       </c>
       <c r="BL12" s="68" t="n">
-        <v>7289.895295484188</v>
+        <v>7289.895295484173</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -16610,7 +16610,7 @@
         <v>212.1157355378084</v>
       </c>
       <c r="G19" s="51" t="n">
-        <v>204.7709771115667</v>
+        <v>204.7709771115672</v>
       </c>
       <c r="H19" s="51" t="n">
         <v>215.1847439167914</v>
@@ -16655,7 +16655,7 @@
         <v>181.7687515902151</v>
       </c>
       <c r="V19" s="51" t="n">
-        <v>192.0478610229875</v>
+        <v>192.047861022987</v>
       </c>
       <c r="W19" s="51" t="n">
         <v>174.1412765880596</v>
@@ -18969,7 +18969,7 @@
         <v>0</v>
       </c>
       <c r="BL31" s="52" t="n">
-        <v>77462.92180595815</v>
+        <v>77462.92180595813</v>
       </c>
       <c r="BM31" s="58" t="inlineStr">
         <is>
@@ -20350,7 +20350,7 @@
         <v>0</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>70691.54000000001</v>
+        <v>70691.53999999998</v>
       </c>
       <c r="BM7" s="58" t="inlineStr">
         <is>
@@ -21242,7 +21242,7 @@
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>70691.54000000001</v>
+        <v>70691.53999999998</v>
       </c>
       <c r="BM11" s="58" t="inlineStr">
         <is>
@@ -21963,7 +21963,7 @@
         <v>789.9273535381026</v>
       </c>
       <c r="G15" s="51" t="n">
-        <v>824.5447644261719</v>
+        <v>824.5447644261715</v>
       </c>
       <c r="H15" s="51" t="n">
         <v>871.7885150300467</v>
@@ -22005,10 +22005,10 @@
         <v>1615.762702699066</v>
       </c>
       <c r="U15" s="51" t="n">
-        <v>1689.734939543117</v>
+        <v>1689.734939543118</v>
       </c>
       <c r="V15" s="51" t="n">
-        <v>1775.334571548981</v>
+        <v>1775.334571548982</v>
       </c>
       <c r="W15" s="51" t="n">
         <v>1856.497995964273</v>
@@ -22089,13 +22089,13 @@
         <v>6272.007161369031</v>
       </c>
       <c r="AW15" s="51" t="n">
-        <v>6316.696230223001</v>
+        <v>6316.696230223002</v>
       </c>
       <c r="AX15" s="51" t="n">
-        <v>6421.392852823383</v>
+        <v>6421.392852823384</v>
       </c>
       <c r="AY15" s="51" t="n">
-        <v>6447.930689543428</v>
+        <v>6447.930689543427</v>
       </c>
       <c r="AZ15" s="51" t="n">
         <v>6554.802468928128</v>
@@ -22107,7 +22107,7 @@
         <v>6746.213723806573</v>
       </c>
       <c r="BC15" s="51" t="n">
-        <v>6780.051659875586</v>
+        <v>6780.051659875585</v>
       </c>
       <c r="BD15" s="51" t="n">
         <v>6854.557722072019</v>
@@ -22119,7 +22119,7 @@
         <v>6962.067782027882</v>
       </c>
       <c r="BG15" s="51" t="n">
-        <v>6925.218182124282</v>
+        <v>6925.218182124281</v>
       </c>
       <c r="BH15" s="51" t="n">
         <v>7040.000803927449</v>
@@ -22906,7 +22906,7 @@
         <v>0</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>296.3409163432356</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y19" s="51" t="n">
         <v>0</v>
@@ -23795,10 +23795,10 @@
         <v>3919.300509790613</v>
       </c>
       <c r="W23" s="51" t="n">
-        <v>2143.965938241632</v>
+        <v>2143.965938241631</v>
       </c>
       <c r="X23" s="51" t="n">
-        <v>287.4679422773593</v>
+        <v>287.4679422773584</v>
       </c>
       <c r="Y23" s="51" t="n">
         <v>0</v>
@@ -23918,7 +23918,7 @@
         <v>0</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>323990.5146440844</v>
+        <v>323990.5146440843</v>
       </c>
       <c r="BM23" s="58" t="inlineStr">
         <is>
@@ -24639,7 +24639,7 @@
         <v>789.9273535381026</v>
       </c>
       <c r="G27" s="51" t="n">
-        <v>824.5447644261719</v>
+        <v>824.5447644261715</v>
       </c>
       <c r="H27" s="51" t="n">
         <v>871.7885150300467</v>
@@ -24681,16 +24681,16 @@
         <v>1615.762702699066</v>
       </c>
       <c r="U27" s="51" t="n">
-        <v>1689.734939543117</v>
+        <v>1689.734939543118</v>
       </c>
       <c r="V27" s="51" t="n">
-        <v>1775.334571548981</v>
+        <v>1775.334571548982</v>
       </c>
       <c r="W27" s="51" t="n">
         <v>1856.497995964273</v>
       </c>
       <c r="X27" s="51" t="n">
-        <v>287.4679422773593</v>
+        <v>287.4679422773584</v>
       </c>
       <c r="Y27" s="51" t="n">
         <v>0</v>
@@ -24810,7 +24810,7 @@
         <v>0</v>
       </c>
       <c r="BL27" s="52" t="n">
-        <v>24999.99999999999</v>
+        <v>25000</v>
       </c>
       <c r="BM27" s="58" t="inlineStr">
         <is>
@@ -25576,10 +25576,10 @@
         <v>3919.300509790613</v>
       </c>
       <c r="V31" s="51" t="n">
-        <v>2143.965938241632</v>
+        <v>2143.965938241631</v>
       </c>
       <c r="W31" s="51" t="n">
-        <v>287.4679422773593</v>
+        <v>287.4679422773584</v>
       </c>
       <c r="X31" s="51" t="n">
         <v>0</v>
@@ -25702,7 +25702,7 @@
         <v>0</v>
       </c>
       <c r="BL31" s="52" t="n">
-        <v>298990.5146440844</v>
+        <v>298990.5146440843</v>
       </c>
       <c r="BM31" s="58" t="inlineStr">
         <is>
@@ -26474,7 +26474,7 @@
         <v>0</v>
       </c>
       <c r="X35" s="51" t="n">
-        <v>1646.338424129086</v>
+        <v>1646.338424129087</v>
       </c>
       <c r="Y35" s="51" t="n">
         <v>2022.69192865896</v>
@@ -26549,13 +26549,13 @@
         <v>6272.007161369031</v>
       </c>
       <c r="AW35" s="51" t="n">
-        <v>6316.696230223001</v>
+        <v>6316.696230223002</v>
       </c>
       <c r="AX35" s="51" t="n">
-        <v>6421.392852823383</v>
+        <v>6421.392852823384</v>
       </c>
       <c r="AY35" s="51" t="n">
-        <v>6447.930689543428</v>
+        <v>6447.930689543427</v>
       </c>
       <c r="AZ35" s="51" t="n">
         <v>6554.802468928128</v>
@@ -26567,7 +26567,7 @@
         <v>6746.213723806573</v>
       </c>
       <c r="BC35" s="51" t="n">
-        <v>6780.051659875586</v>
+        <v>6780.051659875585</v>
       </c>
       <c r="BD35" s="51" t="n">
         <v>6854.557722072019</v>
@@ -26579,7 +26579,7 @@
         <v>6962.067782027882</v>
       </c>
       <c r="BG35" s="51" t="n">
-        <v>6925.218182124282</v>
+        <v>6925.218182124281</v>
       </c>
       <c r="BH35" s="51" t="n">
         <v>7040.000803927449</v>
@@ -27366,10 +27366,10 @@
         <v>0</v>
       </c>
       <c r="X39" s="51" t="n">
-        <v>296.3409163432356</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y39" s="51" t="n">
-        <v>364.0845471586128</v>
+        <v>364.0845471586127</v>
       </c>
       <c r="Z39" s="51" t="n">
         <v>381.3716598916898</v>
@@ -27486,7 +27486,7 @@
         <v>10.10239668311311</v>
       </c>
       <c r="BL39" s="52" t="n">
-        <v>39649.7536131641</v>
+        <v>39649.75361316411</v>
       </c>
       <c r="BM39" s="58" t="inlineStr">
         <is>
@@ -28258,7 +28258,7 @@
         <v>0</v>
       </c>
       <c r="X43" s="51" t="n">
-        <v>296.3409163432356</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y43" s="51" t="n">
         <v>0</v>
@@ -29431,7 +29431,7 @@
         <v>0</v>
       </c>
       <c r="BL6" s="48" t="n">
-        <v>339112.7082112872</v>
+        <v>339112.7082112871</v>
       </c>
       <c r="BM6" s="49" t="inlineStr"/>
       <c r="BN6" s="49" t="inlineStr"/>
@@ -29464,7 +29464,7 @@
         <v>3156.84179835198</v>
       </c>
       <c r="G7" s="51" t="n">
-        <v>3150.433824560011</v>
+        <v>3150.43382456001</v>
       </c>
       <c r="H7" s="51" t="n">
         <v>3185.053976478251</v>
@@ -29491,7 +29491,7 @@
         <v>3341.229727547581</v>
       </c>
       <c r="P7" s="51" t="n">
-        <v>3377.946537740412</v>
+        <v>3377.946537740411</v>
       </c>
       <c r="Q7" s="51" t="n">
         <v>3396.588882121361</v>
@@ -29509,7 +29509,7 @@
         <v>3533.181191458345</v>
       </c>
       <c r="V7" s="51" t="n">
-        <v>3591.74220568141</v>
+        <v>3591.742205681411</v>
       </c>
       <c r="W7" s="51" t="n">
         <v>3607.952524064416</v>
@@ -29518,7 +29518,7 @@
         <v>3647.600353999189</v>
       </c>
       <c r="Y7" s="51" t="n">
-        <v>3667.635538833557</v>
+        <v>3667.635538833556</v>
       </c>
       <c r="Z7" s="51" t="n">
         <v>3728.425078151239</v>
@@ -29590,13 +29590,13 @@
         <v>7456.637704174131</v>
       </c>
       <c r="AW7" s="51" t="n">
-        <v>7485.204790953595</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX7" s="51" t="n">
-        <v>7609.268958759456</v>
+        <v>7609.268958759457</v>
       </c>
       <c r="AY7" s="51" t="n">
-        <v>7616.439250274022</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ7" s="51" t="n">
         <v>7742.678574864201</v>
@@ -29608,7 +29608,7 @@
         <v>7934.089829742647</v>
       </c>
       <c r="BC7" s="51" t="n">
-        <v>7951.805783737153</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD7" s="51" t="n">
         <v>8039.188264877119</v>
@@ -29620,7 +29620,7 @@
         <v>8149.943887963956</v>
       </c>
       <c r="BG7" s="51" t="n">
-        <v>8093.726742854876</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH7" s="51" t="n">
         <v>8227.876909863522</v>
@@ -29635,7 +29635,7 @@
         <v>56.12442601729508</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>338435.3372422293</v>
+        <v>338435.3372422292</v>
       </c>
       <c r="BM7" s="53" t="inlineStr">
         <is>
@@ -29672,7 +29672,7 @@
         <v>-6.382319796672618</v>
       </c>
       <c r="G8" s="51" t="n">
-        <v>29.29726226411412</v>
+        <v>29.29726226411367</v>
       </c>
       <c r="H8" s="51" t="n">
         <v>29.61921020108139</v>
@@ -29699,7 +29699,7 @@
         <v>64.62289266058451</v>
       </c>
       <c r="P8" s="51" t="n">
-        <v>65.33303433817309</v>
+        <v>65.33303433817264</v>
       </c>
       <c r="Q8" s="51" t="n">
         <v>56.36916843654308</v>
@@ -29714,10 +29714,10 @@
         <v>48.73664122147966</v>
       </c>
       <c r="U8" s="51" t="n">
-        <v>39.14395528476916</v>
+        <v>39.14395528476962</v>
       </c>
       <c r="V8" s="51" t="n">
-        <v>39.79275012374364</v>
+        <v>39.7927501237441</v>
       </c>
       <c r="W8" s="51" t="n">
         <v>51.12276195242794</v>
@@ -29726,7 +29726,7 @@
         <v>51.68455054531159</v>
       </c>
       <c r="Y8" s="51" t="n">
-        <v>41.38144986158568</v>
+        <v>41.38144986158522</v>
       </c>
       <c r="Z8" s="51" t="n">
         <v>42.06733024603</v>
@@ -29798,13 +29798,13 @@
         <v>-48.23430293055117</v>
       </c>
       <c r="AW8" s="51" t="n">
-        <v>-64.56065108818802</v>
+        <v>-64.56065108818711</v>
       </c>
       <c r="AX8" s="51" t="n">
-        <v>-65.63071712832425</v>
+        <v>-65.63071712832334</v>
       </c>
       <c r="AY8" s="51" t="n">
-        <v>-82.36809901955621</v>
+        <v>-82.36809901955712</v>
       </c>
       <c r="AZ8" s="51" t="n">
         <v>-83.73331613037772</v>
@@ -29816,7 +29816,7 @@
         <v>-64.24695444409645</v>
       </c>
       <c r="BC8" s="51" t="n">
-        <v>-83.02563452885988</v>
+        <v>-83.02563452886079</v>
       </c>
       <c r="BD8" s="51" t="n">
         <v>-83.93800413906956</v>
@@ -29828,7 +29828,7 @@
         <v>-105.074636819395</v>
       </c>
       <c r="BG8" s="51" t="n">
-        <v>-124.9508885557088</v>
+        <v>-124.9508885557098</v>
       </c>
       <c r="BH8" s="51" t="n">
         <v>-127.0218977582899</v>
@@ -30267,7 +30267,7 @@
         <v>0</v>
       </c>
       <c r="X11" s="51" t="n">
-        <v>296.3409163432356</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y11" s="51" t="n">
         <v>0</v>
@@ -31108,7 +31108,7 @@
         <v>3156.84179835198</v>
       </c>
       <c r="G15" s="51" t="n">
-        <v>3150.433824560011</v>
+        <v>3150.43382456001</v>
       </c>
       <c r="H15" s="51" t="n">
         <v>3185.053976478251</v>
@@ -31135,7 +31135,7 @@
         <v>3341.229727547581</v>
       </c>
       <c r="P15" s="51" t="n">
-        <v>3377.946537740412</v>
+        <v>3377.946537740411</v>
       </c>
       <c r="Q15" s="51" t="n">
         <v>3396.588882121361</v>
@@ -31153,7 +31153,7 @@
         <v>3533.181191458345</v>
       </c>
       <c r="V15" s="51" t="n">
-        <v>3591.74220568141</v>
+        <v>3591.742205681411</v>
       </c>
       <c r="W15" s="51" t="n">
         <v>3607.952524064416</v>
@@ -31162,7 +31162,7 @@
         <v>3351.259437655953</v>
       </c>
       <c r="Y15" s="51" t="n">
-        <v>3667.635538833557</v>
+        <v>3667.635538833556</v>
       </c>
       <c r="Z15" s="51" t="n">
         <v>3347.053418259549</v>
@@ -31234,13 +31234,13 @@
         <v>6327.676415127706</v>
       </c>
       <c r="AW15" s="51" t="n">
-        <v>7485.204790953595</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX15" s="51" t="n">
-        <v>6453.418245251247</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY15" s="51" t="n">
-        <v>7616.439250274022</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ15" s="51" t="n">
         <v>6562.814130457138</v>
@@ -31252,7 +31252,7 @@
         <v>6719.771359457463</v>
       </c>
       <c r="BC15" s="51" t="n">
-        <v>7951.805783737153</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD15" s="51" t="n">
         <v>6805.367874904156</v>
@@ -31264,7 +31264,7 @@
         <v>6896.771687198937</v>
       </c>
       <c r="BG15" s="51" t="n">
-        <v>8093.726742854876</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH15" s="51" t="n">
         <v>6960.676765156581</v>
@@ -31279,7 +31279,7 @@
         <v>56.12442601729508</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>318295.1130998205</v>
+        <v>318295.1130998204</v>
       </c>
       <c r="BM15" s="58" t="inlineStr">
         <is>
@@ -31882,13 +31882,13 @@
         <v>6327.676415127706</v>
       </c>
       <c r="AW19" s="51" t="n">
-        <v>7485.204790953595</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX19" s="51" t="n">
-        <v>6453.418245251247</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY19" s="51" t="n">
-        <v>7616.439250274022</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ19" s="51" t="n">
         <v>6562.814130457138</v>
@@ -31900,7 +31900,7 @@
         <v>6719.771359457463</v>
       </c>
       <c r="BC19" s="51" t="n">
-        <v>7951.805783737153</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD19" s="51" t="n">
         <v>6805.367874904156</v>
@@ -31912,7 +31912,7 @@
         <v>6896.771687198937</v>
       </c>
       <c r="BG19" s="51" t="n">
-        <v>8093.726742854876</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH19" s="51" t="n">
         <v>6960.676765156581</v>
@@ -32530,13 +32530,13 @@
         <v>6327.676415127706</v>
       </c>
       <c r="AW23" s="51" t="n">
-        <v>7485.204790953595</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX23" s="51" t="n">
-        <v>6453.418245251247</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY23" s="51" t="n">
-        <v>7616.439250274022</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ23" s="51" t="n">
         <v>6562.814130457138</v>
@@ -32548,7 +32548,7 @@
         <v>6719.771359457463</v>
       </c>
       <c r="BC23" s="51" t="n">
-        <v>7951.805783737153</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD23" s="51" t="n">
         <v>6805.367874904156</v>
@@ -32560,7 +32560,7 @@
         <v>6896.771687198937</v>
       </c>
       <c r="BG23" s="51" t="n">
-        <v>8093.726742854876</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH23" s="51" t="n">
         <v>6960.676765156581</v>
@@ -33791,13 +33791,13 @@
         <v>6327.676415127706</v>
       </c>
       <c r="AW7" s="51" t="n">
-        <v>7485.204790953595</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX7" s="51" t="n">
-        <v>6453.418245251247</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY7" s="51" t="n">
-        <v>7616.439250274022</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ7" s="51" t="n">
         <v>6562.814130457138</v>
@@ -33809,7 +33809,7 @@
         <v>6719.771359457463</v>
       </c>
       <c r="BC7" s="51" t="n">
-        <v>7951.805783737153</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD7" s="51" t="n">
         <v>6805.367874904156</v>
@@ -33821,7 +33821,7 @@
         <v>6896.771687198937</v>
       </c>
       <c r="BG7" s="51" t="n">
-        <v>8093.726742854876</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH7" s="51" t="n">
         <v>6960.676765156581</v>
@@ -33836,7 +33836,7 @@
         <v>56.12442601729508</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>173572.2883697887</v>
+        <v>173572.2883697886</v>
       </c>
       <c r="BM7" s="79" t="inlineStr">
         <is>
@@ -34003,13 +34003,13 @@
         <v>-1083.746844591877</v>
       </c>
       <c r="AW8" s="51" t="n">
-        <v>2650.095104931562</v>
+        <v>2650.095104931563</v>
       </c>
       <c r="AX8" s="51" t="n">
-        <v>-1084.175519478923</v>
+        <v>-1084.175519478922</v>
       </c>
       <c r="AY8" s="51" t="n">
-        <v>2664.474182350283</v>
+        <v>2664.474182350282</v>
       </c>
       <c r="AZ8" s="51" t="n">
         <v>-1123.527521187737</v>
@@ -34021,7 +34021,7 @@
         <v>-1135.358429515777</v>
       </c>
       <c r="BC8" s="51" t="n">
-        <v>2791.409369359827</v>
+        <v>2791.409369359826</v>
       </c>
       <c r="BD8" s="51" t="n">
         <v>-1216.386437867111</v>
@@ -34033,7 +34033,7 @@
         <v>-1210.356704635606</v>
       </c>
       <c r="BG8" s="51" t="n">
-        <v>2767.937934958466</v>
+        <v>2767.937934958465</v>
       </c>
       <c r="BH8" s="51" t="n">
         <v>-1244.509601780442</v>
@@ -34048,7 +34048,7 @@
         <v>-5316.083126731314</v>
       </c>
       <c r="BL8" s="80" t="n">
-        <v>21862.8947830672</v>
+        <v>21862.89478306711</v>
       </c>
       <c r="BM8" s="79" t="inlineStr">
         <is>
@@ -37112,7 +37112,7 @@
       <c r="BJ7" s="70" t="inlineStr"/>
       <c r="BK7" s="70" t="inlineStr"/>
       <c r="BL7" s="83" t="n">
-        <v>0.09410162472306152</v>
+        <v>0.09410162472306149</v>
       </c>
       <c r="BM7" s="53" t="inlineStr">
         <is>
@@ -37446,7 +37446,7 @@
         </is>
       </c>
       <c r="BL8" s="84" t="n">
-        <v>-0.0005983752769384842</v>
+        <v>-0.000598375276938512</v>
       </c>
       <c r="BM8" s="53" t="inlineStr">
         <is>
@@ -37972,7 +37972,7 @@
         </is>
       </c>
       <c r="BL12" s="85" t="n">
-        <v>-0.004604924443546016</v>
+        <v>-0.004604924443546043</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -40917,7 +40917,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09T07:39:19+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -41360,7 +41360,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CIRR Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-06-09T07:39:19+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -41412,7 +41412,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09T07:39:19+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -42376,7 +42376,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCalibration Residual Closeout&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-06-09T07:39:19+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -42532,7 +42532,7 @@
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>252468.72481961406</t>
+          <t>252468.7248196141</t>
         </is>
       </c>
       <c r="E6" s="21" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>252468.72481961406</t>
+          <t>252468.7248196141</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
@@ -42835,7 +42835,7 @@
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>756328.0823817673</t>
+          <t>756328.0823817672</t>
         </is>
       </c>
       <c r="D10" s="21" t="inlineStr">
@@ -42845,7 +42845,7 @@
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>25146.29258193518</t>
+          <t>25146.292581935297</t>
         </is>
       </c>
       <c r="F10" s="21" t="inlineStr">
@@ -42912,17 +42912,17 @@
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>712969.5518136515</t>
+          <t>712969.5518136513</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>738115.3749637025</t>
+          <t>738115.3749637026</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>25145.82315005106</t>
+          <t>25145.823150051292</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
@@ -43066,17 +43066,17 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>38755.38</t>
+          <t>38755.380000000005</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>46045.275295484185</t>
+          <t>46045.27529548418</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>7289.895295484188</t>
+          <t>7289.895295484173</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -43143,12 +43143,12 @@
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>84674.77873934135</t>
+          <t>84674.77873934136</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>85408.27413448403</t>
+          <t>85408.27413448405</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">
@@ -43220,17 +43220,17 @@
       </c>
       <c r="C15" s="21" t="inlineStr">
         <is>
-          <t>22822.816668720294</t>
+          <t>22822.816668720287</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>22467.388280206444</t>
+          <t>22467.388280206447</t>
         </is>
       </c>
       <c r="E15" s="21" t="inlineStr">
         <is>
-          <t>-355.4283885138502</t>
+          <t>-355.4283885138393</t>
         </is>
       </c>
       <c r="F15" s="21" t="inlineStr">
@@ -43302,12 +43302,12 @@
       </c>
       <c r="D16" s="21" t="inlineStr">
         <is>
-          <t>43358.999999999985</t>
+          <t>43358.99999999999</t>
         </is>
       </c>
       <c r="E16" s="21" t="inlineStr">
         <is>
-          <t>0.46943188410659786</t>
+          <t>0.4694318841138738</t>
         </is>
       </c>
       <c r="F16" s="21" t="inlineStr">
@@ -43456,12 +43456,12 @@
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>0.11149507555645398</t>
+          <t>0.11149507555645395</t>
         </is>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>-0.004604924443546016</t>
+          <t>-0.0046049244435460435</t>
         </is>
       </c>
       <c r="F18" s="21" t="inlineStr">
@@ -44303,7 +44303,7 @@
       </c>
       <c r="D29" s="21" t="inlineStr">
         <is>
-          <t>318295.1130998205</t>
+          <t>318295.11309982045</t>
         </is>
       </c>
       <c r="E29" s="21" t="inlineStr">
@@ -44380,7 +44380,7 @@
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
-          <t>20140.22414240874</t>
+          <t>20140.224142408744</t>
         </is>
       </c>
       <c r="E30" s="21" t="inlineStr">
@@ -44996,7 +44996,7 @@
       </c>
       <c r="D38" s="21" t="inlineStr">
         <is>
-          <t>39434.911711302164</t>
+          <t>39434.91171130216</t>
         </is>
       </c>
       <c r="E38" s="21" t="inlineStr">
@@ -45073,7 +45073,7 @@
       </c>
       <c r="D39" s="21" t="inlineStr">
         <is>
-          <t>1128738.031373649</t>
+          <t>1128738.0313736491</t>
         </is>
       </c>
       <c r="E39" s="21" t="inlineStr">
@@ -45150,7 +45150,7 @@
       </c>
       <c r="D40" s="21" t="inlineStr">
         <is>
-          <t>1161441.7213736488</t>
+          <t>1161441.721373649</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
@@ -45304,7 +45304,7 @@
       </c>
       <c r="D42" s="21" t="inlineStr">
         <is>
-          <t>77462.92180595815</t>
+          <t>77462.92180595813</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr">
@@ -45381,7 +45381,7 @@
       </c>
       <c r="D43" s="21" t="inlineStr">
         <is>
-          <t>70691.54000000001</t>
+          <t>70691.53999999998</t>
         </is>
       </c>
       <c r="E43" s="21" t="inlineStr">
@@ -45458,7 +45458,7 @@
       </c>
       <c r="D44" s="21" t="inlineStr">
         <is>
-          <t>39649.7536131641</t>
+          <t>39649.75361316411</t>
         </is>
       </c>
       <c r="E44" s="21" t="inlineStr">
@@ -45535,7 +45535,7 @@
       </c>
       <c r="D45" s="21" t="inlineStr">
         <is>
-          <t>20140.22414240874</t>
+          <t>20140.224142408744</t>
         </is>
       </c>
       <c r="E45" s="21" t="inlineStr">
@@ -45612,7 +45612,7 @@
       </c>
       <c r="D46" s="21" t="inlineStr">
         <is>
-          <t>298990.5146440844</t>
+          <t>298990.5146440843</t>
         </is>
       </c>
       <c r="E46" s="21" t="inlineStr">
@@ -45689,7 +45689,7 @@
       </c>
       <c r="D47" s="21" t="inlineStr">
         <is>
-          <t>323990.5146440844</t>
+          <t>323990.5146440843</t>
         </is>
       </c>
       <c r="E47" s="21" t="inlineStr">
@@ -45766,7 +45766,7 @@
       </c>
       <c r="D48" s="21" t="inlineStr">
         <is>
-          <t>24999.999999999993</t>
+          <t>24999.999999999996</t>
         </is>
       </c>
       <c r="E48" s="21" t="inlineStr">
@@ -45843,7 +45843,7 @@
       </c>
       <c r="D49" s="21" t="inlineStr">
         <is>
-          <t>20140.22414240874</t>
+          <t>20140.224142408744</t>
         </is>
       </c>
       <c r="E49" s="21" t="inlineStr">
@@ -45920,7 +45920,7 @@
       </c>
       <c r="D50" s="21" t="inlineStr">
         <is>
-          <t>70691.54000000001</t>
+          <t>70691.53999999998</t>
         </is>
       </c>
       <c r="E50" s="21" t="inlineStr">
@@ -45997,7 +45997,7 @@
       </c>
       <c r="D51" s="21" t="inlineStr">
         <is>
-          <t>220276.4089620228</t>
+          <t>220276.40896202278</t>
         </is>
       </c>
       <c r="E51" s="21" t="inlineStr">
@@ -46069,17 +46069,17 @@
       </c>
       <c r="C52" s="21" t="inlineStr">
         <is>
-          <t>151709.3935867215</t>
+          <t>151709.39358672153</t>
         </is>
       </c>
       <c r="D52" s="21" t="inlineStr">
         <is>
-          <t>173572.2883697887</t>
+          <t>173572.28836978864</t>
         </is>
       </c>
       <c r="E52" s="21" t="inlineStr">
         <is>
-          <t>21862.894783067197</t>
+          <t>21862.89478306711</t>
         </is>
       </c>
       <c r="F52" s="21" t="inlineStr">
@@ -46377,12 +46377,12 @@
       </c>
       <c r="C56" s="21" t="inlineStr">
         <is>
-          <t>339112.70821128716</t>
+          <t>339112.7082112871</t>
         </is>
       </c>
       <c r="D56" s="21" t="inlineStr">
         <is>
-          <t>338435.33724222926</t>
+          <t>338435.3372422292</t>
         </is>
       </c>
       <c r="E56" s="21" t="inlineStr">
@@ -46442,12 +46442,12 @@
       </c>
       <c r="C57" s="21" t="inlineStr">
         <is>
-          <t>339112.70821128716</t>
+          <t>339112.7082112871</t>
         </is>
       </c>
       <c r="D57" s="21" t="inlineStr">
         <is>
-          <t>338435.33724222926</t>
+          <t>338435.3372422292</t>
         </is>
       </c>
       <c r="E57" s="21" t="inlineStr">
@@ -46507,12 +46507,12 @@
       </c>
       <c r="C58" s="21" t="inlineStr">
         <is>
-          <t>423787.48695062846</t>
+          <t>423787.4869506285</t>
         </is>
       </c>
       <c r="D58" s="21" t="inlineStr">
         <is>
-          <t>423843.61137671326</t>
+          <t>423843.6113767133</t>
         </is>
       </c>
       <c r="E58" s="21" t="inlineStr">
@@ -46572,12 +46572,12 @@
       </c>
       <c r="C59" s="21" t="inlineStr">
         <is>
-          <t>423787.48695062846</t>
+          <t>423787.4869506285</t>
         </is>
       </c>
       <c r="D59" s="21" t="inlineStr">
         <is>
-          <t>423843.61137671326</t>
+          <t>423843.6113767133</t>
         </is>
       </c>
       <c r="E59" s="21" t="inlineStr">
@@ -46715,12 +46715,12 @@
       </c>
       <c r="D61" s="21" t="inlineStr">
         <is>
-          <t>0.09410162472306152</t>
+          <t>0.0941016247230615</t>
         </is>
       </c>
       <c r="E61" s="21" t="inlineStr">
         <is>
-          <t>-0.0005983752769384842</t>
+          <t>-0.000598375276938512</t>
         </is>
       </c>
       <c r="F61" s="21" t="inlineStr">
@@ -48100,7 +48100,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>2026-06-09T07:39:19+00:00</t>
+          <t>2026-07-01T14:45:00+00:00</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -48134,7 +48134,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>233981e40e69f48736ea89ac5322f52c924703cf</t>
+          <t>9a0ba27f424473368d929fd676903b9565603069</t>
         </is>
       </c>
     </row>
@@ -48146,7 +48146,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-06-09T07:39:19+00:00</t>
+          <t>2026-07-01T14:45:00+00:00</t>
         </is>
       </c>
     </row>
@@ -48194,7 +48194,7 @@
       </c>
       <c r="B17" s="24" t="inlineStr">
         <is>
-          <t>0.09410162472306152</t>
+          <t>0.0941016247230615</t>
         </is>
       </c>
       <c r="D17" s="20" t="inlineStr">
@@ -48214,7 +48214,7 @@
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>0.11149507555645398</t>
+          <t>0.11149507555645395</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -48254,7 +48254,7 @@
       </c>
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>423843.61137671326</t>
+          <t>423843.6113767133</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -48274,7 +48274,7 @@
       </c>
       <c r="B21" s="24" t="inlineStr">
         <is>
-          <t>338435.33724222926</t>
+          <t>338435.3372422292</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
@@ -48294,7 +48294,7 @@
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>173572.2883697887</t>
+          <t>173572.28836978864</t>
         </is>
       </c>
     </row>
@@ -48386,7 +48386,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09T07:39:19+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49382,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CNavigation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-06-09T07:39:19+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -49432,7 +49432,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09T07:39:19+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49990,7 +49990,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Dashboard&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-06-09T07:39:19+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -50039,7 +50039,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-09T07:39:19+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -50104,7 +50104,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.09410162472306152</t>
+          <t>0.0941016247230615</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -50129,7 +50129,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.11149507555645398</t>
+          <t>0.11149507555645395</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -50154,7 +50154,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>423843.61137671326</t>
+          <t>423843.6113767133</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -50179,7 +50179,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>338435.33724222926</t>
+          <t>338435.3372422292</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -50204,7 +50204,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>85408.27413448403</t>
+          <t>85408.27413448405</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -50638,7 +50638,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-06-09T07:39:19+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Update calibration reconciliation pack (auto-regenerated artifact)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8W8EHSADMzvD3ufdXTkMr
</commit_message>
<xml_diff>
--- a/reports/phase10_calibration_reconciliation_pack.xlsx
+++ b/reports/phase10_calibration_reconciliation_pack.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01T14:45:00+00:00</t>
+          <t>2026-07-01T14:57:16+00:00</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01T14:45:00+00:00</t>
+          <t>2026-07-01T14:57:16+00:00</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CRuntime Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-01T14:45:00+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-01T14:57:16+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5911,7 +5911,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCO2 &amp; Balancing Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -40917,7 +40917,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -41360,7 +41360,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CIRR Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -41412,7 +41412,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -42376,7 +42376,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCalibration Residual Closeout&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -48100,7 +48100,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>2026-07-01T14:45:00+00:00</t>
+          <t>2026-07-01T14:57:16+00:00</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -48134,7 +48134,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>9a0ba27f424473368d929fd676903b9565603069</t>
+          <t>927f114e566dce1b03290efc6c7e2e366b6c3673</t>
         </is>
       </c>
     </row>
@@ -48146,7 +48146,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-07-01T14:45:00+00:00</t>
+          <t>2026-07-01T14:57:16+00:00</t>
         </is>
       </c>
     </row>
@@ -48386,7 +48386,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49382,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CNavigation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -49432,7 +49432,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49990,7 +49990,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Dashboard&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -50039,7 +50039,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:45:00+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -50638,7 +50638,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:45:00+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Stack P: update calibration reports to reflect Stack K–O parity results
Auto-regenerated reports now reflect the final Sprint K–O model state:
TUHO equity IRR 11.59% (−2 bps vs golden), Oborovo equity IRR 10.66%
(+6 bps vs golden). IRR reconciliation summary updated accordingly.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8W8EHSADMzvD3ufdXTkMr
</commit_message>
<xml_diff>
--- a/reports/phase10_calibration_reconciliation_pack.xlsx
+++ b/reports/phase10_calibration_reconciliation_pack.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01T14:57:16+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01T14:57:16+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>0.11149507555645395</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>1.554228403104244</t>
+          <t>1.3785647255425093</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>1.3856226986474167</t>
+          <t>1.162014679369489</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>173572.28836978864</t>
+          <t>180089.48366015987</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>77462.92180595815</t>
+          <t>76153.89091893201</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
@@ -2087,7 +2087,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CRuntime Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-01T14:57:16+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5911,7 +5911,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCO2 &amp; Balancing Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -14250,28 +14250,28 @@
         <v>38028.01009465598</v>
       </c>
       <c r="AE7" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>34219.39256116209</v>
       </c>
       <c r="AF7" s="51" t="n">
-        <v>33339.73575126298</v>
+        <v>29380.93173303165</v>
       </c>
       <c r="AG7" s="51" t="n">
-        <v>29325.85443333631</v>
+        <v>25209.22609491149</v>
       </c>
       <c r="AH7" s="51" t="n">
-        <v>24257.27807523225</v>
+        <v>19978.76699288986</v>
       </c>
       <c r="AI7" s="51" t="n">
-        <v>19826.73796185821</v>
+        <v>15377.18958936602</v>
       </c>
       <c r="AJ7" s="51" t="n">
-        <v>14186.92079596805</v>
+        <v>9562.397895654238</v>
       </c>
       <c r="AK7" s="51" t="n">
-        <v>9189.011119904026</v>
+        <v>4379.618798924304</v>
       </c>
       <c r="AL7" s="51" t="n">
-        <v>2980.071929073079</v>
+        <v>0</v>
       </c>
       <c r="AM7" s="51" t="n">
         <v>0</v>
@@ -14349,7 +14349,7 @@
         <v>0</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>1161441.721373649</v>
+        <v>1128415.624878298</v>
       </c>
       <c r="BM7" s="58" t="inlineStr">
         <is>
@@ -15022,28 +15022,28 @@
         <v>1520.203564090807</v>
       </c>
       <c r="AE11" s="51" t="n">
-        <v>1499.571198065934</v>
+        <v>1349.384713328492</v>
       </c>
       <c r="AF11" s="51" t="n">
-        <v>1329.144131950351</v>
+        <v>1171.319811756862</v>
       </c>
       <c r="AG11" s="51" t="n">
-        <v>1153.213113528784</v>
+        <v>991.3303696112138</v>
       </c>
       <c r="AH11" s="51" t="n">
-        <v>969.7062900036407</v>
+        <v>798.6689998538479</v>
       </c>
       <c r="AI11" s="51" t="n">
-        <v>779.6688164053136</v>
+        <v>604.6942885836913</v>
       </c>
       <c r="AJ11" s="51" t="n">
-        <v>567.1347910085725</v>
+        <v>382.2653703426579</v>
       </c>
       <c r="AK11" s="51" t="n">
-        <v>361.3496802940232</v>
+        <v>172.2246096071239</v>
       </c>
       <c r="AL11" s="51" t="n">
-        <v>119.1310288534003</v>
+        <v>0</v>
       </c>
       <c r="AM11" s="51" t="n">
         <v>0</v>
@@ -15121,7 +15121,7 @@
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>46045.27529548418</v>
+        <v>44736.24440845805</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -15234,28 +15234,28 @@
         <v>-96.75643590919344</v>
       </c>
       <c r="AE12" s="51" t="n">
-        <v>-77.91880193406564</v>
+        <v>-228.1052866715081</v>
       </c>
       <c r="AF12" s="51" t="n">
-        <v>-197.7258680496491</v>
+        <v>-355.5501882431381</v>
       </c>
       <c r="AG12" s="51" t="n">
-        <v>-202.5368864712163</v>
+        <v>-364.4196303887862</v>
       </c>
       <c r="AH12" s="51" t="n">
-        <v>-212.1637099963592</v>
+        <v>-383.201000146152</v>
       </c>
       <c r="AI12" s="51" t="n">
-        <v>-219.1911835946864</v>
+        <v>-394.1657114163087</v>
       </c>
       <c r="AJ12" s="51" t="n">
-        <v>-252.7952089914274</v>
+        <v>-437.6646296573421</v>
       </c>
       <c r="AK12" s="51" t="n">
-        <v>-246.5503197059768</v>
+        <v>-435.6753903928761</v>
       </c>
       <c r="AL12" s="51" t="n">
-        <v>-300.6089711465997</v>
+        <v>-419.74</v>
       </c>
       <c r="AM12" s="51" t="n">
         <v>-178.47</v>
@@ -15333,7 +15333,7 @@
         <v>0</v>
       </c>
       <c r="BL12" s="68" t="n">
-        <v>7289.895295484173</v>
+        <v>5980.864408458045</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -15790,28 +15790,28 @@
         <v>1520.203564090807</v>
       </c>
       <c r="AE15" s="51" t="n">
-        <v>1499.571198065934</v>
+        <v>1349.384713328492</v>
       </c>
       <c r="AF15" s="51" t="n">
-        <v>1329.144131950351</v>
+        <v>1171.319811756862</v>
       </c>
       <c r="AG15" s="51" t="n">
-        <v>1153.213113528784</v>
+        <v>991.3303696112138</v>
       </c>
       <c r="AH15" s="51" t="n">
-        <v>969.7062900036407</v>
+        <v>798.6689998538479</v>
       </c>
       <c r="AI15" s="51" t="n">
-        <v>779.6688164053136</v>
+        <v>604.6942885836913</v>
       </c>
       <c r="AJ15" s="51" t="n">
-        <v>567.1347910085725</v>
+        <v>382.2653703426579</v>
       </c>
       <c r="AK15" s="51" t="n">
-        <v>361.3496802940232</v>
+        <v>172.2246096071239</v>
       </c>
       <c r="AL15" s="51" t="n">
-        <v>119.1310288534003</v>
+        <v>0</v>
       </c>
       <c r="AM15" s="51" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>39434.91171130216</v>
+        <v>38125.88082427603</v>
       </c>
       <c r="BM15" s="58" t="inlineStr">
         <is>
@@ -17451,31 +17451,31 @@
         <v>0</v>
       </c>
       <c r="AD23" s="51" t="n">
-        <v>0</v>
+        <v>3808.617533493891</v>
       </c>
       <c r="AE23" s="51" t="n">
-        <v>4688.274343393</v>
+        <v>4838.460828130443</v>
       </c>
       <c r="AF23" s="51" t="n">
-        <v>4013.881317926676</v>
+        <v>4171.705638120166</v>
       </c>
       <c r="AG23" s="51" t="n">
-        <v>5068.576358104057</v>
+        <v>5230.459102021628</v>
       </c>
       <c r="AH23" s="51" t="n">
-        <v>4430.540113374041</v>
+        <v>4601.577403523834</v>
       </c>
       <c r="AI23" s="51" t="n">
-        <v>5639.817165890164</v>
+        <v>5814.791693711786</v>
       </c>
       <c r="AJ23" s="51" t="n">
-        <v>4997.90967606402</v>
+        <v>5182.779096729934</v>
       </c>
       <c r="AK23" s="51" t="n">
-        <v>6208.939190830946</v>
+        <v>4379.618798924304</v>
       </c>
       <c r="AL23" s="51" t="n">
-        <v>2980.071929073079</v>
+        <v>0</v>
       </c>
       <c r="AM23" s="51" t="n">
         <v>0</v>
@@ -17663,31 +17663,31 @@
         <v>-1465.03</v>
       </c>
       <c r="AD24" s="51" t="n">
-        <v>-1643.29</v>
+        <v>2165.327533493891</v>
       </c>
       <c r="AE24" s="51" t="n">
-        <v>3849.174343393</v>
+        <v>3999.360828130443</v>
       </c>
       <c r="AF24" s="51" t="n">
-        <v>-645.1986820733237</v>
+        <v>-487.3743618798344</v>
       </c>
       <c r="AG24" s="51" t="n">
-        <v>1242.796358104057</v>
+        <v>1404.679102021627</v>
       </c>
       <c r="AH24" s="51" t="n">
-        <v>-593.2298866259598</v>
+        <v>-422.1925964761667</v>
       </c>
       <c r="AI24" s="51" t="n">
-        <v>1540.107165890164</v>
+        <v>1715.081693711786</v>
       </c>
       <c r="AJ24" s="51" t="n">
-        <v>-596.6303239359804</v>
+        <v>-411.7609032700657</v>
       </c>
       <c r="AK24" s="51" t="n">
-        <v>1715.609190830946</v>
+        <v>-113.7112010756964</v>
       </c>
       <c r="AL24" s="51" t="n">
-        <v>-3174.90807092692</v>
+        <v>-6154.98</v>
       </c>
       <c r="AM24" s="51" t="n">
         <v>-4425.36</v>
@@ -17975,28 +17975,28 @@
         <v>38028.01009465598</v>
       </c>
       <c r="AD27" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>34219.39256116209</v>
       </c>
       <c r="AE27" s="51" t="n">
-        <v>33339.73575126298</v>
+        <v>29380.93173303165</v>
       </c>
       <c r="AF27" s="51" t="n">
-        <v>29325.85443333631</v>
+        <v>25209.22609491149</v>
       </c>
       <c r="AG27" s="51" t="n">
-        <v>24257.27807523225</v>
+        <v>19978.76699288986</v>
       </c>
       <c r="AH27" s="51" t="n">
-        <v>19826.73796185821</v>
+        <v>15377.18958936602</v>
       </c>
       <c r="AI27" s="51" t="n">
-        <v>14186.92079596805</v>
+        <v>9562.397895654238</v>
       </c>
       <c r="AJ27" s="51" t="n">
-        <v>9189.011119904026</v>
+        <v>4379.618798924304</v>
       </c>
       <c r="AK27" s="51" t="n">
-        <v>2980.071929073079</v>
+        <v>0</v>
       </c>
       <c r="AL27" s="51" t="n">
         <v>0</v>
@@ -18077,7 +18077,7 @@
         <v>0</v>
       </c>
       <c r="BL27" s="52" t="n">
-        <v>1128738.031373649</v>
+        <v>1095711.934878298</v>
       </c>
       <c r="BM27" s="58" t="inlineStr">
         <is>
@@ -18867,7 +18867,7 @@
         <v>1495.417636415413</v>
       </c>
       <c r="AD31" s="51" t="n">
-        <v>1520.203564090807</v>
+        <v>5328.821097584698</v>
       </c>
       <c r="AE31" s="51" t="n">
         <v>6187.845541458934</v>
@@ -18888,10 +18888,10 @@
         <v>5565.044467072592</v>
       </c>
       <c r="AK31" s="51" t="n">
-        <v>6570.28887112497</v>
+        <v>4551.843408531427</v>
       </c>
       <c r="AL31" s="51" t="n">
-        <v>3099.20295792648</v>
+        <v>0</v>
       </c>
       <c r="AM31" s="51" t="n">
         <v>0</v>
@@ -18969,7 +18969,7 @@
         <v>0</v>
       </c>
       <c r="BL31" s="52" t="n">
-        <v>77462.92180595813</v>
+        <v>76153.89091893201</v>
       </c>
       <c r="BM31" s="58" t="inlineStr">
         <is>
@@ -33755,10 +33755,10 @@
         <v>0</v>
       </c>
       <c r="AK7" s="51" t="n">
-        <v>0</v>
+        <v>6398.064261517846</v>
       </c>
       <c r="AL7" s="51" t="n">
-        <v>5571.621393283242</v>
+        <v>5690.752422136643</v>
       </c>
       <c r="AM7" s="51" t="n">
         <v>6735.889890096291</v>
@@ -33836,7 +33836,7 @@
         <v>56.12442601729508</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>173572.2883697886</v>
+        <v>180089.4836601599</v>
       </c>
       <c r="BM7" s="79" t="inlineStr">
         <is>
@@ -33967,10 +33967,10 @@
         <v>0</v>
       </c>
       <c r="AK8" s="51" t="n">
-        <v>0</v>
+        <v>6398.064261517846</v>
       </c>
       <c r="AL8" s="51" t="n">
-        <v>5569.332351252046</v>
+        <v>5688.463380105447</v>
       </c>
       <c r="AM8" s="51" t="n">
         <v>6279.82438136977</v>
@@ -34048,7 +34048,7 @@
         <v>-5316.083126731314</v>
       </c>
       <c r="BL8" s="80" t="n">
-        <v>21862.89478306711</v>
+        <v>28380.09007343833</v>
       </c>
       <c r="BM8" s="79" t="inlineStr">
         <is>
@@ -37638,7 +37638,7 @@
       <c r="BJ11" s="70" t="inlineStr"/>
       <c r="BK11" s="70" t="inlineStr"/>
       <c r="BL11" s="83" t="n">
-        <v>0.111495075556454</v>
+        <v>0.1158773428956301</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -37972,7 +37972,7 @@
         </is>
       </c>
       <c r="BL12" s="85" t="n">
-        <v>-0.004604924443546043</v>
+        <v>-0.0002226571043698472</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -39716,7 +39716,7 @@
       <c r="BJ23" s="70" t="inlineStr"/>
       <c r="BK23" s="70" t="inlineStr"/>
       <c r="BL23" s="86" t="n">
-        <v>1.554228403104244</v>
+        <v>1.378564725542509</v>
       </c>
       <c r="BM23" s="67" t="inlineStr">
         <is>
@@ -40050,7 +40050,7 @@
         </is>
       </c>
       <c r="BL24" s="87" t="n">
-        <v>0.1032284031042439</v>
+        <v>-0.07243527445749076</v>
       </c>
       <c r="BM24" s="67" t="inlineStr">
         <is>
@@ -40488,7 +40488,7 @@
       <c r="BJ27" s="70" t="inlineStr"/>
       <c r="BK27" s="70" t="inlineStr"/>
       <c r="BL27" s="86" t="n">
-        <v>1.385622698647417</v>
+        <v>1.162014679369489</v>
       </c>
       <c r="BM27" s="58" t="inlineStr">
         <is>
@@ -40917,7 +40917,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -41035,7 +41035,7 @@
       </c>
       <c r="B9" s="89" t="inlineStr">
         <is>
-          <t>0.111495</t>
+          <t>0.115877</t>
         </is>
       </c>
       <c r="C9" s="89" t="inlineStr">
@@ -41045,7 +41045,7 @@
       </c>
       <c r="D9" s="89" t="inlineStr">
         <is>
-          <t>-0.004605</t>
+          <t>-0.000223</t>
         </is>
       </c>
       <c r="E9" s="90" t="inlineStr">
@@ -41360,7 +41360,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CIRR Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -41412,7 +41412,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -42376,7 +42376,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCalibration Residual Closeout&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -43071,12 +43071,12 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>46045.27529548418</t>
+          <t>44736.24440845805</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>7289.895295484173</t>
+          <t>5980.864408458045</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -43379,12 +43379,12 @@
       </c>
       <c r="D17" s="21" t="inlineStr">
         <is>
-          <t>1.554228403104244</t>
+          <t>1.3785647255425093</t>
         </is>
       </c>
       <c r="E17" s="21" t="inlineStr">
         <is>
-          <t>0.10322840310424386</t>
+          <t>-0.07243527445749076</t>
         </is>
       </c>
       <c r="F17" s="21" t="inlineStr">
@@ -43456,12 +43456,12 @@
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>0.11149507555645395</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>-0.0046049244435460435</t>
+          <t>-0.0002226571043698472</t>
         </is>
       </c>
       <c r="F18" s="21" t="inlineStr">
@@ -43687,12 +43687,12 @@
       </c>
       <c r="D21" s="21" t="inlineStr">
         <is>
-          <t>0.111495</t>
+          <t>0.115877</t>
         </is>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
-          <t>-0.004605</t>
+          <t>-0.000223</t>
         </is>
       </c>
       <c r="F21" s="21" t="inlineStr">
@@ -44688,7 +44688,7 @@
       </c>
       <c r="D34" s="21" t="inlineStr">
         <is>
-          <t>1.3856226986474167</t>
+          <t>1.162014679369489</t>
         </is>
       </c>
       <c r="E34" s="21" t="inlineStr">
@@ -44996,7 +44996,7 @@
       </c>
       <c r="D38" s="21" t="inlineStr">
         <is>
-          <t>39434.91171130216</t>
+          <t>38125.88082427603</t>
         </is>
       </c>
       <c r="E38" s="21" t="inlineStr">
@@ -45073,7 +45073,7 @@
       </c>
       <c r="D39" s="21" t="inlineStr">
         <is>
-          <t>1128738.0313736491</t>
+          <t>1095711.9348782978</t>
         </is>
       </c>
       <c r="E39" s="21" t="inlineStr">
@@ -45150,7 +45150,7 @@
       </c>
       <c r="D40" s="21" t="inlineStr">
         <is>
-          <t>1161441.721373649</t>
+          <t>1128415.624878298</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
@@ -45304,7 +45304,7 @@
       </c>
       <c r="D42" s="21" t="inlineStr">
         <is>
-          <t>77462.92180595813</t>
+          <t>76153.89091893201</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr">
@@ -46074,12 +46074,12 @@
       </c>
       <c r="D52" s="21" t="inlineStr">
         <is>
-          <t>173572.28836978864</t>
+          <t>180089.48366015987</t>
         </is>
       </c>
       <c r="E52" s="21" t="inlineStr">
         <is>
-          <t>21862.89478306711</t>
+          <t>28380.090073438332</t>
         </is>
       </c>
       <c r="F52" s="21" t="inlineStr">
@@ -48100,7 +48100,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>2026-07-01T14:57:16+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -48134,7 +48134,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>927f114e566dce1b03290efc6c7e2e366b6c3673</t>
+          <t>dd4f044670c5062e420f95ef114df3f9b594e621</t>
         </is>
       </c>
     </row>
@@ -48146,7 +48146,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-07-01T14:57:16+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -48214,7 +48214,7 @@
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>0.11149507555645395</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -48234,7 +48234,7 @@
       </c>
       <c r="B19" s="24" t="inlineStr">
         <is>
-          <t>1.554228403104244</t>
+          <t>1.3785647255425093</t>
         </is>
       </c>
       <c r="D19" s="20" t="inlineStr">
@@ -48294,7 +48294,7 @@
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>173572.28836978864</t>
+          <t>180089.48366015987</t>
         </is>
       </c>
     </row>
@@ -48386,7 +48386,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49382,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CNavigation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -49432,7 +49432,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49990,7 +49990,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Dashboard&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -50039,7 +50039,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-01T14:57:16+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -50129,7 +50129,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.11149507555645395</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -50229,7 +50229,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.554228403104244</t>
+          <t>1.3785647255425093</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -50254,7 +50254,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3856226986474167</t>
+          <t>1.162014679369489</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -50638,7 +50638,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-01T14:57:16+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
chore: update generated reports after Stack S test run
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8W8EHSADMzvD3ufdXTkMr
</commit_message>
<xml_diff>
--- a/reports/phase10_calibration_reconciliation_pack.xlsx
+++ b/reports/phase10_calibration_reconciliation_pack.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-02T20:20:08+00:00</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-02T20:20:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CRuntime Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-02T20:20:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5911,7 +5911,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCO2 &amp; Balancing Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -40917,7 +40917,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -41360,7 +41360,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CIRR Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -41412,7 +41412,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -42376,7 +42376,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCalibration Residual Closeout&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -48100,7 +48100,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-02T20:20:08+00:00</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -48134,7 +48134,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>dd4f044670c5062e420f95ef114df3f9b594e621</t>
+          <t>a5febc6e24417592aac1269d87ce14f32f388870</t>
         </is>
       </c>
     </row>
@@ -48146,7 +48146,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-02T20:20:08+00:00</t>
         </is>
       </c>
     </row>
@@ -48386,7 +48386,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49382,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CNavigation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -49432,7 +49432,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49990,7 +49990,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Dashboard&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -50039,7 +50039,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -50638,7 +50638,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
chore: revert generated reports to main baseline (out of Stack S scope)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8W8EHSADMzvD3ufdXTkMr
</commit_message>
<xml_diff>
--- a/reports/phase10_calibration_reconciliation_pack.xlsx
+++ b/reports/phase10_calibration_reconciliation_pack.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T20:20:08+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T20:20:08+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CRuntime Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-02T20:20:08+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5911,7 +5911,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCO2 &amp; Balancing Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -40917,7 +40917,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -41360,7 +41360,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CIRR Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -41412,7 +41412,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -42376,7 +42376,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCalibration Residual Closeout&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -48100,7 +48100,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>2026-07-02T20:20:08+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -48134,7 +48134,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>a5febc6e24417592aac1269d87ce14f32f388870</t>
+          <t>dd4f044670c5062e420f95ef114df3f9b594e621</t>
         </is>
       </c>
     </row>
@@ -48146,7 +48146,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-07-02T20:20:08+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -48386,7 +48386,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49382,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CNavigation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -49432,7 +49432,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49990,7 +49990,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Dashboard&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -50039,7 +50039,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T20:20:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -50638,7 +50638,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T20:20:08+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
chore: restore generated report artifacts to main state
Remove auto-generated calibration reports from PR diff — out of scope for
Phase 0 hotfix. Restored to main baseline.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8W8EHSADMzvD3ufdXTkMr
</commit_message>
<xml_diff>
--- a/reports/phase10_calibration_reconciliation_pack.xlsx
+++ b/reports/phase10_calibration_reconciliation_pack.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03T20:06:50+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03T20:06:50+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03T20:06:50+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>0.11321363695747841</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>165471.11047208743</t>
+          <t>180089.48366015987</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>75486.60520011785</t>
+          <t>76153.89091893201</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
@@ -2087,7 +2087,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CRuntime Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-03T20:06:50+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5911,7 +5911,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03T20:06:50+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCO2 &amp; Balancing Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-03T20:06:50+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -11857,88 +11857,88 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>1989.106693769401</v>
+        <v>2116.361416666667</v>
       </c>
       <c r="D19" s="51" t="n">
-        <v>2022.075313003147</v>
+        <v>2144.69175</v>
       </c>
       <c r="E19" s="51" t="n">
-        <v>2011.897283088215</v>
+        <v>2144.914083333334</v>
       </c>
       <c r="F19" s="51" t="n">
-        <v>2045.243646896307</v>
+        <v>2169.311</v>
       </c>
       <c r="G19" s="51" t="n">
-        <v>2041.09207119988</v>
+        <v>2194.979083333334</v>
       </c>
       <c r="H19" s="51" t="n">
-        <v>2063.521654399878</v>
+        <v>2189.918</v>
       </c>
       <c r="I19" s="51" t="n">
-        <v>2059.740388389284</v>
+        <v>2243.1435</v>
       </c>
       <c r="J19" s="51" t="n">
-        <v>2093.87973184325</v>
+        <v>2287.658</v>
       </c>
       <c r="K19" s="51" t="n">
-        <v>2079.711488155402</v>
+        <v>2342.122833333333</v>
       </c>
       <c r="L19" s="51" t="n">
-        <v>2114.181844312673</v>
+        <v>2395.111416666667</v>
       </c>
       <c r="M19" s="51" t="n">
-        <v>2119.985981148247</v>
+        <v>2435.872083333333</v>
       </c>
       <c r="N19" s="51" t="n">
-        <v>2155.123870338549</v>
+        <v>2484.465916666667</v>
       </c>
       <c r="O19" s="51" t="n">
-        <v>2164.704254947222</v>
+        <v>2875.376522231662</v>
       </c>
       <c r="P19" s="51" t="n">
-        <v>2188.492213792796</v>
+        <v>2829.374203596205</v>
       </c>
       <c r="Q19" s="51" t="n">
-        <v>2200.570150808295</v>
+        <v>0</v>
       </c>
       <c r="R19" s="51" t="n">
-        <v>2237.043689219482</v>
+        <v>0</v>
       </c>
       <c r="S19" s="51" t="n">
-        <v>2245.580238898558</v>
+        <v>0</v>
       </c>
       <c r="T19" s="51" t="n">
-        <v>2282.799800869252</v>
+        <v>0</v>
       </c>
       <c r="U19" s="51" t="n">
-        <v>2289.065099472558</v>
+        <v>0</v>
       </c>
       <c r="V19" s="51" t="n">
-        <v>2327.005404988678</v>
+        <v>0</v>
       </c>
       <c r="W19" s="51" t="n">
-        <v>2337.507689488432</v>
+        <v>0</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>2363.194587175117</v>
+        <v>0</v>
       </c>
       <c r="Y19" s="51" t="n">
-        <v>2376.174912802545</v>
+        <v>0</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>2415.559027379383</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="51" t="n">
-        <v>3379.663922072882</v>
+        <v>0</v>
       </c>
       <c r="AB19" s="51" t="n">
-        <v>3435.680451168012</v>
+        <v>0</v>
       </c>
       <c r="AC19" s="51" t="n">
-        <v>3365.998420752923</v>
+        <v>0</v>
       </c>
       <c r="AD19" s="51" t="n">
-        <v>3421.788449826067</v>
+        <v>0</v>
       </c>
       <c r="AE19" s="51" t="n">
         <v>0</v>
@@ -12040,7 +12040,7 @@
         <v>0</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>65826.38828020645</v>
+        <v>32853.2998091612</v>
       </c>
       <c r="BM19" s="67" t="inlineStr">
         <is>
@@ -12069,88 +12069,88 @@
       </c>
       <c r="B20" s="50" t="inlineStr"/>
       <c r="C20" s="51" t="n">
-        <v>-127.2547003226625</v>
+        <v>2.257460346299922e-05</v>
       </c>
       <c r="D20" s="51" t="n">
-        <v>-129.3638942506627</v>
+        <v>-6.747457253809444</v>
       </c>
       <c r="E20" s="51" t="n">
-        <v>-132.7944419476889</v>
+        <v>0.2223582974293095</v>
       </c>
       <c r="F20" s="51" t="n">
-        <v>-134.9954547976515</v>
+        <v>-10.92810169395852</v>
       </c>
       <c r="G20" s="51" t="n">
-        <v>-103.8219942392489</v>
+        <v>50.06501789420463</v>
       </c>
       <c r="H20" s="51" t="n">
-        <v>-104.9628952748462</v>
+        <v>21.43345032527623</v>
       </c>
       <c r="I20" s="51" t="n">
-        <v>-109.5705885445132</v>
+        <v>73.83252306620261</v>
       </c>
       <c r="J20" s="51" t="n">
-        <v>-111.3866756474617</v>
+        <v>82.39159250928833</v>
       </c>
       <c r="K20" s="51" t="n">
-        <v>-115.2676361454241</v>
+        <v>147.1437090325076</v>
       </c>
       <c r="L20" s="51" t="n">
-        <v>-117.1781494517013</v>
+        <v>163.7514229022922</v>
       </c>
       <c r="M20" s="51" t="n">
-        <v>-69.9319859582306</v>
+        <v>245.9541162268556</v>
       </c>
       <c r="N20" s="51" t="n">
-        <v>-71.09107964814484</v>
+        <v>258.2509666799729</v>
       </c>
       <c r="O20" s="51" t="n">
-        <v>-78.43927664433613</v>
+        <v>632.2329906401042</v>
       </c>
       <c r="P20" s="51" t="n">
-        <v>-79.30124671734939</v>
+        <v>561.5807430860605</v>
       </c>
       <c r="Q20" s="51" t="n">
-        <v>-87.08788978115626</v>
+        <v>-2287.658040589451</v>
       </c>
       <c r="R20" s="51" t="n">
-        <v>-88.53133546813615</v>
+        <v>-2325.575024687618</v>
       </c>
       <c r="S20" s="51" t="n">
-        <v>-96.54259994560471</v>
+        <v>-2342.122838844162</v>
       </c>
       <c r="T20" s="51" t="n">
-        <v>-98.1427535358639</v>
+        <v>-2380.942554405116</v>
       </c>
       <c r="U20" s="51" t="n">
-        <v>-106.0463032261123</v>
+        <v>-2395.111402698671</v>
       </c>
       <c r="V20" s="51" t="n">
-        <v>-107.8039767602477</v>
+        <v>-2434.809381748925</v>
       </c>
       <c r="W20" s="51" t="n">
-        <v>-98.36437314777368</v>
+        <v>-2435.872062636206</v>
       </c>
       <c r="X20" s="51" t="n">
-        <v>-99.44530032522243</v>
+        <v>-2462.63988750034</v>
       </c>
       <c r="Y20" s="51" t="n">
-        <v>-108.2910184327302</v>
+        <v>-2484.465931235276</v>
       </c>
       <c r="Z20" s="51" t="n">
-        <v>-110.0858971912849</v>
+        <v>-2525.644924570668</v>
       </c>
       <c r="AA20" s="51" t="n">
-        <v>504.3609086899392</v>
+        <v>-2875.303013382943</v>
       </c>
       <c r="AB20" s="51" t="n">
-        <v>512.7204817621459</v>
+        <v>-2922.959969405866</v>
       </c>
       <c r="AC20" s="51" t="n">
-        <v>536.6659621780268</v>
+        <v>-2829.332458574896</v>
       </c>
       <c r="AD20" s="51" t="n">
-        <v>576.9951581442028</v>
+        <v>-2844.793291681864</v>
       </c>
       <c r="AE20" s="51" t="n">
         <v>0</v>
@@ -12252,7 +12252,7 @@
         <v>0</v>
       </c>
       <c r="BL20" s="68" t="n">
-        <v>-354.9589566297218</v>
+        <v>-33328.04742767497</v>
       </c>
       <c r="BM20" s="67" t="inlineStr">
         <is>
@@ -13194,48 +13194,20 @@
       <c r="P27" s="75" t="n">
         <v>1.19388468780374</v>
       </c>
-      <c r="Q27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="R27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="S27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="T27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="U27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="V27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="W27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="X27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="Y27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="Z27" s="75" t="n">
-        <v>1.543504023661211</v>
-      </c>
-      <c r="AA27" s="75" t="n">
-        <v>1.816832861184551</v>
-      </c>
-      <c r="AB27" s="75" t="n">
-        <v>1.816832861184551</v>
-      </c>
-      <c r="AC27" s="75" t="n">
-        <v>1.816832861184551</v>
-      </c>
-      <c r="AD27" s="75" t="n">
-        <v>1.816832861184609</v>
-      </c>
+      <c r="Q27" s="70" t="n"/>
+      <c r="R27" s="70" t="n"/>
+      <c r="S27" s="70" t="n"/>
+      <c r="T27" s="70" t="n"/>
+      <c r="U27" s="70" t="n"/>
+      <c r="V27" s="70" t="n"/>
+      <c r="W27" s="70" t="n"/>
+      <c r="X27" s="70" t="n"/>
+      <c r="Y27" s="70" t="n"/>
+      <c r="Z27" s="70" t="n"/>
+      <c r="AA27" s="70" t="n"/>
+      <c r="AB27" s="70" t="n"/>
+      <c r="AC27" s="70" t="n"/>
+      <c r="AD27" s="70" t="n"/>
       <c r="AE27" s="70" t="n"/>
       <c r="AF27" s="70" t="n"/>
       <c r="AG27" s="70" t="n"/>
@@ -13338,47 +13310,75 @@
       <c r="P28" s="75" t="n">
         <v>-0.006115312196260048</v>
       </c>
-      <c r="Q28" s="75" t="n">
-        <v>0.3435040236612112</v>
-      </c>
-      <c r="R28" s="75" t="n">
-        <v>0.343504023661211</v>
-      </c>
-      <c r="S28" s="75" t="n">
-        <v>0.3435040236612112</v>
-      </c>
-      <c r="T28" s="75" t="n">
-        <v>0.3435040236612112</v>
-      </c>
-      <c r="U28" s="75" t="n">
-        <v>0.3435040236612115</v>
-      </c>
-      <c r="V28" s="75" t="n">
-        <v>0.3435040236612115</v>
-      </c>
-      <c r="W28" s="75" t="n">
-        <v>0.3435040236612112</v>
-      </c>
-      <c r="X28" s="75" t="n">
-        <v>0.3435040236612115</v>
-      </c>
-      <c r="Y28" s="75" t="n">
-        <v>0.3435040236612112</v>
-      </c>
-      <c r="Z28" s="75" t="n">
-        <v>0.3435040236612112</v>
-      </c>
-      <c r="AA28" s="75" t="n">
-        <v>0.4043967420309842</v>
-      </c>
-      <c r="AB28" s="75" t="n">
-        <v>0.4043967420309844</v>
-      </c>
-      <c r="AC28" s="75" t="n">
-        <v>0.4042120165976311</v>
-      </c>
-      <c r="AD28" s="75" t="n">
-        <v>0.404212016597689</v>
+      <c r="Q28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="R28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="S28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="T28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="U28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="V28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="W28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="X28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Y28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="Z28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AA28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AB28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AC28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="AD28" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="AE28" s="59" t="inlineStr">
         <is>
@@ -14232,43 +14232,43 @@
         <v>36807.77046925188</v>
       </c>
       <c r="Y7" s="51" t="n">
-        <v>36990.76781846865</v>
+        <v>37287.10873481189</v>
       </c>
       <c r="Z7" s="51" t="n">
-        <v>37153.93619991388</v>
+        <v>37461.93045892712</v>
       </c>
       <c r="AA7" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AB7" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AC7" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AD7" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AE7" s="51" t="n">
-        <v>32601.66748205897</v>
+        <v>34219.39256116209</v>
       </c>
       <c r="AF7" s="51" t="n">
-        <v>27699.41436164256</v>
+        <v>29380.93173303165</v>
       </c>
       <c r="AG7" s="51" t="n">
-        <v>22832.10451072115</v>
+        <v>25209.22609491149</v>
       </c>
       <c r="AH7" s="51" t="n">
-        <v>17508.16721901635</v>
+        <v>19978.76699288986</v>
       </c>
       <c r="AI7" s="51" t="n">
-        <v>13429.81973793022</v>
+        <v>15377.18958936602</v>
       </c>
       <c r="AJ7" s="51" t="n">
-        <v>7538.449458770179</v>
+        <v>9562.397895654238</v>
       </c>
       <c r="AK7" s="51" t="n">
-        <v>3070.632209149414</v>
+        <v>4379.618798924304</v>
       </c>
       <c r="AL7" s="51" t="n">
         <v>0</v>
@@ -14349,7 +14349,7 @@
         <v>0</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>1111577.307961688</v>
+        <v>1128415.624878298</v>
       </c>
       <c r="BM7" s="58" t="inlineStr">
         <is>
@@ -15004,43 +15004,43 @@
         <v>1467.403116040841</v>
       </c>
       <c r="Y11" s="51" t="n">
-        <v>1454.629007476236</v>
+        <v>1466.282350146234</v>
       </c>
       <c r="Z11" s="51" t="n">
-        <v>1485.261681863516</v>
+        <v>1497.574026609034</v>
       </c>
       <c r="AA11" s="51" t="n">
-        <v>1467.824763479375</v>
+        <v>1495.417636415413</v>
       </c>
       <c r="AB11" s="51" t="n">
-        <v>1492.153350719365</v>
+        <v>1520.203564090807</v>
       </c>
       <c r="AC11" s="51" t="n">
-        <v>1467.824763479375</v>
+        <v>1495.417636415413</v>
       </c>
       <c r="AD11" s="51" t="n">
-        <v>1492.153350719365</v>
+        <v>1520.203564090807</v>
       </c>
       <c r="AE11" s="51" t="n">
-        <v>1285.592421042525</v>
+        <v>1349.384713328492</v>
       </c>
       <c r="AF11" s="51" t="n">
-        <v>1104.283319217483</v>
+        <v>1171.319811756862</v>
       </c>
       <c r="AG11" s="51" t="n">
-        <v>897.8521799280383</v>
+        <v>991.3303696112138</v>
       </c>
       <c r="AH11" s="51" t="n">
-        <v>699.9045740441409</v>
+        <v>798.6689998538479</v>
       </c>
       <c r="AI11" s="51" t="n">
-        <v>528.1157031354352</v>
+        <v>604.6942885836913</v>
       </c>
       <c r="AJ11" s="51" t="n">
-        <v>301.3562294323492</v>
+        <v>382.2653703426579</v>
       </c>
       <c r="AK11" s="51" t="n">
-        <v>120.7498775002309</v>
+        <v>172.2246096071239</v>
       </c>
       <c r="AL11" s="51" t="n">
         <v>0</v>
@@ -15121,7 +15121,7 @@
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>44068.95868964389</v>
+        <v>44736.24440845805</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -15216,43 +15216,43 @@
         <v>346.4431160408415</v>
       </c>
       <c r="Y12" s="51" t="n">
-        <v>321.1990074762359</v>
+        <v>332.8523501462341</v>
       </c>
       <c r="Z12" s="51" t="n">
-        <v>343.4716818635161</v>
+        <v>355.7840266090338</v>
       </c>
       <c r="AA12" s="51" t="n">
-        <v>303.8347634793749</v>
+        <v>331.427636415413</v>
       </c>
       <c r="AB12" s="51" t="n">
-        <v>-242.3666492806353</v>
+        <v>-214.3164359091934</v>
       </c>
       <c r="AC12" s="51" t="n">
-        <v>-235.015236520625</v>
+        <v>-207.4223635845869</v>
       </c>
       <c r="AD12" s="51" t="n">
-        <v>-124.8066492806354</v>
+        <v>-96.75643590919344</v>
       </c>
       <c r="AE12" s="51" t="n">
-        <v>-291.8975789574747</v>
+        <v>-228.1052866715081</v>
       </c>
       <c r="AF12" s="51" t="n">
-        <v>-422.5866807825169</v>
+        <v>-355.5501882431381</v>
       </c>
       <c r="AG12" s="51" t="n">
-        <v>-457.8978200719617</v>
+        <v>-364.4196303887862</v>
       </c>
       <c r="AH12" s="51" t="n">
-        <v>-481.965425955859</v>
+        <v>-383.201000146152</v>
       </c>
       <c r="AI12" s="51" t="n">
-        <v>-470.7442968645648</v>
+        <v>-394.1657114163087</v>
       </c>
       <c r="AJ12" s="51" t="n">
-        <v>-518.5737705676509</v>
+        <v>-437.6646296573421</v>
       </c>
       <c r="AK12" s="51" t="n">
-        <v>-487.1501224997691</v>
+        <v>-435.6753903928761</v>
       </c>
       <c r="AL12" s="51" t="n">
         <v>-419.74</v>
@@ -15333,7 +15333,7 @@
         <v>0</v>
       </c>
       <c r="BL12" s="68" t="n">
-        <v>5313.578689643888</v>
+        <v>5980.864408458045</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -15769,46 +15769,46 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X15" s="51" t="n">
-        <v>1284.405766824072</v>
+        <v>988.064850480836</v>
       </c>
       <c r="Y15" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z15" s="51" t="n">
-        <v>1312.866050771856</v>
+        <v>931.4943908801665</v>
       </c>
       <c r="AA15" s="51" t="n">
-        <v>1467.824763479375</v>
+        <v>1495.417636415413</v>
       </c>
       <c r="AB15" s="51" t="n">
-        <v>1492.153350719365</v>
+        <v>1520.203564090807</v>
       </c>
       <c r="AC15" s="51" t="n">
-        <v>1467.824763479375</v>
+        <v>1495.417636415413</v>
       </c>
       <c r="AD15" s="51" t="n">
-        <v>1492.153350719365</v>
+        <v>1520.203564090807</v>
       </c>
       <c r="AE15" s="51" t="n">
-        <v>1285.592421042525</v>
+        <v>1349.384713328492</v>
       </c>
       <c r="AF15" s="51" t="n">
-        <v>1104.283319217483</v>
+        <v>1171.319811756862</v>
       </c>
       <c r="AG15" s="51" t="n">
-        <v>897.8521799280383</v>
+        <v>991.3303696112138</v>
       </c>
       <c r="AH15" s="51" t="n">
-        <v>699.9045740441409</v>
+        <v>798.6689998538479</v>
       </c>
       <c r="AI15" s="51" t="n">
-        <v>528.1157031354352</v>
+        <v>604.6942885836913</v>
       </c>
       <c r="AJ15" s="51" t="n">
-        <v>301.3562294323492</v>
+        <v>382.2653703426579</v>
       </c>
       <c r="AK15" s="51" t="n">
-        <v>120.7498775002309</v>
+        <v>172.2246096071239</v>
       </c>
       <c r="AL15" s="51" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>38160.27336911231</v>
+        <v>38125.88082427603</v>
       </c>
       <c r="BM15" s="58" t="inlineStr">
         <is>
@@ -16661,13 +16661,13 @@
         <v>174.1412765880596</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>182.9973492167699</v>
+        <v>479.3382655600055</v>
       </c>
       <c r="Y19" s="51" t="n">
-        <v>163.1683814452249</v>
+        <v>174.8217241152231</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>172.3956310916597</v>
+        <v>566.0796357288673</v>
       </c>
       <c r="AA19" s="51" t="n">
         <v>0</v>
@@ -16781,7 +16781,7 @@
         <v>0</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>4622.641831005549</v>
+        <v>5324.32009465599</v>
       </c>
       <c r="BM19" s="58" t="inlineStr">
         <is>
@@ -17451,28 +17451,28 @@
         <v>0</v>
       </c>
       <c r="AD23" s="51" t="n">
-        <v>4724.664348946576</v>
+        <v>3808.617533493891</v>
       </c>
       <c r="AE23" s="51" t="n">
-        <v>4902.253120416409</v>
+        <v>4838.460828130443</v>
       </c>
       <c r="AF23" s="51" t="n">
-        <v>4867.309850921405</v>
+        <v>4171.705638120166</v>
       </c>
       <c r="AG23" s="51" t="n">
-        <v>5323.937291704803</v>
+        <v>5230.459102021628</v>
       </c>
       <c r="AH23" s="51" t="n">
-        <v>4078.347481086129</v>
+        <v>4601.577403523834</v>
       </c>
       <c r="AI23" s="51" t="n">
-        <v>5891.370279160043</v>
+        <v>5814.791693711786</v>
       </c>
       <c r="AJ23" s="51" t="n">
-        <v>4467.817249620765</v>
+        <v>5182.779096729934</v>
       </c>
       <c r="AK23" s="51" t="n">
-        <v>3070.632209149414</v>
+        <v>4379.618798924304</v>
       </c>
       <c r="AL23" s="51" t="n">
         <v>0</v>
@@ -17553,7 +17553,7 @@
         <v>0</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="BM23" s="67" t="inlineStr">
         <is>
@@ -17663,28 +17663,28 @@
         <v>-1465.03</v>
       </c>
       <c r="AD24" s="51" t="n">
-        <v>3081.374348946576</v>
+        <v>2165.327533493891</v>
       </c>
       <c r="AE24" s="51" t="n">
-        <v>4063.153120416409</v>
+        <v>3999.360828130443</v>
       </c>
       <c r="AF24" s="51" t="n">
-        <v>208.2298509214052</v>
+        <v>-487.3743618798344</v>
       </c>
       <c r="AG24" s="51" t="n">
-        <v>1498.157291704803</v>
+        <v>1404.679102021627</v>
       </c>
       <c r="AH24" s="51" t="n">
-        <v>-945.4225189138715</v>
+        <v>-422.1925964761667</v>
       </c>
       <c r="AI24" s="51" t="n">
-        <v>1791.660279160043</v>
+        <v>1715.081693711786</v>
       </c>
       <c r="AJ24" s="51" t="n">
-        <v>-1126.722750379235</v>
+        <v>-411.7609032700657</v>
       </c>
       <c r="AK24" s="51" t="n">
-        <v>-1422.697790850586</v>
+        <v>-113.7112010756964</v>
       </c>
       <c r="AL24" s="51" t="n">
         <v>-6154.98</v>
@@ -17765,7 +17765,7 @@
         <v>0</v>
       </c>
       <c r="BL24" s="68" t="n">
-        <v>22730.80183100554</v>
+        <v>23432.48009465598</v>
       </c>
       <c r="BM24" s="67" t="inlineStr">
         <is>
@@ -17957,43 +17957,43 @@
         <v>36807.77046925188</v>
       </c>
       <c r="X27" s="51" t="n">
-        <v>36990.76781846865</v>
+        <v>37287.10873481189</v>
       </c>
       <c r="Y27" s="51" t="n">
-        <v>37153.93619991388</v>
+        <v>37461.93045892711</v>
       </c>
       <c r="Z27" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AA27" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AB27" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AC27" s="51" t="n">
-        <v>37326.33183100554</v>
+        <v>38028.01009465598</v>
       </c>
       <c r="AD27" s="51" t="n">
-        <v>32601.66748205897</v>
+        <v>34219.39256116209</v>
       </c>
       <c r="AE27" s="51" t="n">
-        <v>27699.41436164256</v>
+        <v>29380.93173303165</v>
       </c>
       <c r="AF27" s="51" t="n">
-        <v>22832.10451072115</v>
+        <v>25209.22609491149</v>
       </c>
       <c r="AG27" s="51" t="n">
-        <v>17508.16721901635</v>
+        <v>19978.76699288986</v>
       </c>
       <c r="AH27" s="51" t="n">
-        <v>13429.81973793022</v>
+        <v>15377.18958936602</v>
       </c>
       <c r="AI27" s="51" t="n">
-        <v>7538.449458770179</v>
+        <v>9562.397895654238</v>
       </c>
       <c r="AJ27" s="51" t="n">
-        <v>3070.632209149414</v>
+        <v>4379.618798924304</v>
       </c>
       <c r="AK27" s="51" t="n">
         <v>0</v>
@@ -18077,7 +18077,7 @@
         <v>0</v>
       </c>
       <c r="BL27" s="52" t="n">
-        <v>1078873.617961689</v>
+        <v>1095711.934878298</v>
       </c>
       <c r="BM27" s="58" t="inlineStr">
         <is>
@@ -18849,46 +18849,46 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X31" s="51" t="n">
-        <v>1284.405766824072</v>
+        <v>988.064850480836</v>
       </c>
       <c r="Y31" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z31" s="51" t="n">
-        <v>1312.866050771856</v>
+        <v>931.4943908801665</v>
       </c>
       <c r="AA31" s="51" t="n">
-        <v>1467.824763479375</v>
+        <v>1495.417636415413</v>
       </c>
       <c r="AB31" s="51" t="n">
-        <v>1492.153350719365</v>
+        <v>1520.203564090807</v>
       </c>
       <c r="AC31" s="51" t="n">
-        <v>1467.824763479375</v>
+        <v>1495.417636415413</v>
       </c>
       <c r="AD31" s="51" t="n">
-        <v>6216.81769966594</v>
+        <v>5328.821097584698</v>
       </c>
       <c r="AE31" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF31" s="51" t="n">
-        <v>5971.593170138888</v>
+        <v>5343.025449877027</v>
       </c>
       <c r="AG31" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH31" s="51" t="n">
-        <v>4778.25205513027</v>
+        <v>5400.246403377681</v>
       </c>
       <c r="AI31" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ31" s="51" t="n">
-        <v>4769.173479053115</v>
+        <v>5565.044467072592</v>
       </c>
       <c r="AK31" s="51" t="n">
-        <v>3191.382086649645</v>
+        <v>4551.843408531427</v>
       </c>
       <c r="AL31" s="51" t="n">
         <v>0</v>
@@ -18969,7 +18969,7 @@
         <v>0</v>
       </c>
       <c r="BL31" s="52" t="n">
-        <v>75486.60520011785</v>
+        <v>76153.89091893201</v>
       </c>
       <c r="BM31" s="58" t="inlineStr">
         <is>
@@ -21951,190 +21951,190 @@
         </is>
       </c>
       <c r="C15" s="51" t="n">
-        <v>-651.9713368714761</v>
+        <v>655.1143745939253</v>
       </c>
       <c r="D15" s="51" t="n">
-        <v>-615.0966439918807</v>
+        <v>707.9819198386576</v>
       </c>
       <c r="E15" s="51" t="n">
-        <v>-600.5733396857972</v>
+        <v>734.549128681577</v>
       </c>
       <c r="F15" s="51" t="n">
-        <v>-562.2532857223232</v>
+        <v>789.9273535381026</v>
       </c>
       <c r="G15" s="51" t="n">
-        <v>-544.0686570007056</v>
+        <v>824.5447644261715</v>
       </c>
       <c r="H15" s="51" t="n">
-        <v>-514.4824772060829</v>
+        <v>871.7885150300467</v>
       </c>
       <c r="I15" s="51" t="n">
-        <v>-486.830642377583</v>
+        <v>908.9520914556761</v>
       </c>
       <c r="J15" s="51" t="n">
-        <v>-908.0437414302339</v>
+        <v>969.8207848092713</v>
       </c>
       <c r="K15" s="51" t="n">
-        <v>-891.8622833841346</v>
+        <v>996.6349527778393</v>
       </c>
       <c r="L15" s="51" t="n">
-        <v>-873.8283460277439</v>
+        <v>1060.223384607837</v>
       </c>
       <c r="M15" s="51" t="n">
-        <v>-835.12875894838</v>
+        <v>1120.146841475899</v>
       </c>
       <c r="N15" s="51" t="n">
-        <v>-816.174831372292</v>
+        <v>1187.687261244841</v>
       </c>
       <c r="O15" s="51" t="n">
-        <v>-764.5361370454169</v>
+        <v>1253.218645585758</v>
       </c>
       <c r="P15" s="51" t="n">
-        <v>-751.4286513165603</v>
+        <v>1312.951896619405</v>
       </c>
       <c r="Q15" s="51" t="n">
-        <v>-675.6073991875118</v>
+        <v>1385.324906394822</v>
       </c>
       <c r="R15" s="51" t="n">
-        <v>-652.5111827392628</v>
+        <v>1461.291588138776</v>
       </c>
       <c r="S15" s="51" t="n">
-        <v>-579.8910930473126</v>
+        <v>1535.04343874859</v>
       </c>
       <c r="T15" s="51" t="n">
-        <v>-554.1674325043709</v>
+        <v>1615.762702699066</v>
       </c>
       <c r="U15" s="51" t="n">
-        <v>-482.2856909486381</v>
+        <v>1689.734939543118</v>
       </c>
       <c r="V15" s="51" t="n">
-        <v>-453.9991848377199</v>
+        <v>1775.334571548982</v>
       </c>
       <c r="W15" s="51" t="n">
-        <v>-394.269672082849</v>
+        <v>1856.497995964273</v>
       </c>
       <c r="X15" s="51" t="n">
-        <v>-371.8780017926481</v>
+        <v>1933.806366406446</v>
       </c>
       <c r="Y15" s="51" t="n">
-        <v>-279.3307538511121</v>
+        <v>2022.69192865896</v>
       </c>
       <c r="Z15" s="51" t="n">
-        <v>-246.1443906004934</v>
+        <v>2118.731443842721</v>
       </c>
       <c r="AA15" s="51" t="n">
-        <v>2862.744612971182</v>
+        <v>4607.278452375285</v>
       </c>
       <c r="AB15" s="51" t="n">
-        <v>3082.892918434734</v>
+        <v>4776.369613776</v>
       </c>
       <c r="AC15" s="51" t="n">
-        <v>3132.923854640633</v>
+        <v>4759.925290806009</v>
       </c>
       <c r="AD15" s="51" t="n">
-        <v>3365.333811679907</v>
+        <v>4933.314456006903</v>
       </c>
       <c r="AE15" s="51" t="n">
-        <v>3481.764336407045</v>
+        <v>5016.091417597368</v>
       </c>
       <c r="AF15" s="51" t="n">
-        <v>3721.063927205155</v>
+        <v>5071.213301307228</v>
       </c>
       <c r="AG15" s="51" t="n">
-        <v>3860.622417300403</v>
+        <v>5053.280910902247</v>
       </c>
       <c r="AH15" s="51" t="n">
-        <v>4146.96485784826</v>
+        <v>5137.036948099522</v>
       </c>
       <c r="AI15" s="51" t="n">
-        <v>4420.133097826707</v>
+        <v>5250.977421564884</v>
       </c>
       <c r="AJ15" s="51" t="n">
-        <v>4738.809323908284</v>
+        <v>5338.01019650795</v>
       </c>
       <c r="AK15" s="51" t="n">
-        <v>4971.01061773881</v>
+        <v>5401.780310394376</v>
       </c>
       <c r="AL15" s="51" t="n">
-        <v>5321.552297014329</v>
+        <v>5491.312580732402</v>
       </c>
       <c r="AM15" s="51" t="n">
-        <v>5557.698223429625</v>
+        <v>5564.135766234725</v>
       </c>
       <c r="AN15" s="51" t="n">
-        <v>5631.718991452662</v>
+        <v>5625.280115314228</v>
       </c>
       <c r="AO15" s="51" t="n">
-        <v>5690.44622932455</v>
+        <v>5700.129335260623</v>
       </c>
       <c r="AP15" s="51" t="n">
-        <v>5804.291056329932</v>
+        <v>5794.606617060525</v>
       </c>
       <c r="AQ15" s="51" t="n">
-        <v>5840.408817857736</v>
+        <v>5850.091923793809</v>
       </c>
       <c r="AR15" s="51" t="n">
-        <v>5956.73921262886</v>
+        <v>5947.054773359453</v>
       </c>
       <c r="AS15" s="51" t="n">
-        <v>5989.996418436989</v>
+        <v>5999.679524373062</v>
       </c>
       <c r="AT15" s="51" t="n">
-        <v>6108.806165703902</v>
+        <v>6099.121726434495</v>
       </c>
       <c r="AU15" s="51" t="n">
-        <v>6197.395627679482</v>
+        <v>6203.833170484581</v>
       </c>
       <c r="AV15" s="51" t="n">
-        <v>6278.446037507464</v>
+        <v>6272.007161369031</v>
       </c>
       <c r="AW15" s="51" t="n">
-        <v>6307.013124286929</v>
+        <v>6316.696230223002</v>
       </c>
       <c r="AX15" s="51" t="n">
-        <v>6431.07729209279</v>
+        <v>6421.392852823384</v>
       </c>
       <c r="AY15" s="51" t="n">
-        <v>6438.247583607354</v>
+        <v>6447.930689543427</v>
       </c>
       <c r="AZ15" s="51" t="n">
-        <v>6564.486908197535</v>
+        <v>6554.802468928128</v>
       </c>
       <c r="BA15" s="51" t="n">
-        <v>6626.538002808436</v>
+        <v>6636.221108744508</v>
       </c>
       <c r="BB15" s="51" t="n">
-        <v>6755.89816307598</v>
+        <v>6746.213723806573</v>
       </c>
       <c r="BC15" s="51" t="n">
-        <v>6773.614117070485</v>
+        <v>6780.051659875585</v>
       </c>
       <c r="BD15" s="51" t="n">
-        <v>6860.996598210452</v>
+        <v>6854.557722072019</v>
       </c>
       <c r="BE15" s="51" t="n">
-        <v>6838.872701384834</v>
+        <v>6848.555807320907</v>
       </c>
       <c r="BF15" s="51" t="n">
-        <v>6971.752221297289</v>
+        <v>6962.067782027882</v>
       </c>
       <c r="BG15" s="51" t="n">
-        <v>6915.535076188208</v>
+        <v>6925.218182124281</v>
       </c>
       <c r="BH15" s="51" t="n">
-        <v>7049.685243196855</v>
+        <v>7040.000803927449</v>
       </c>
       <c r="BI15" s="51" t="n">
-        <v>6935.898175298783</v>
+        <v>6945.581281234856</v>
       </c>
       <c r="BJ15" s="51" t="n">
-        <v>7070.385852237438</v>
+        <v>7060.70141296803</v>
       </c>
       <c r="BK15" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>186251.5244043248</v>
+        <v>245276.4089620228</v>
       </c>
       <c r="BM15" s="67" t="inlineStr">
         <is>
@@ -22906,127 +22906,127 @@
         <v>0</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>0</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>0</v>
+        <v>381.3716598916898</v>
       </c>
       <c r="AA19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AB19" s="51" t="n">
-        <v>347.6088232202716</v>
+        <v>859.7465304796799</v>
       </c>
       <c r="AC19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AD19" s="51" t="n">
-        <v>1169.686379937697</v>
+        <v>887.9966020812425</v>
       </c>
       <c r="AE19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AF19" s="51" t="n">
-        <v>1296.509087450196</v>
+        <v>912.818394235301</v>
       </c>
       <c r="AG19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AH19" s="51" t="n">
-        <v>1441.365709526759</v>
+        <v>924.666650657914</v>
       </c>
       <c r="AI19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AJ19" s="51" t="n">
-        <v>1648.609635912298</v>
+        <v>960.841835371431</v>
       </c>
       <c r="AK19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AL19" s="51" t="n">
-        <v>1852.661324655565</v>
+        <v>988.4362645318324</v>
       </c>
       <c r="AM19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AN19" s="51" t="n">
-        <v>2014.095098678811</v>
+        <v>1012.550420756561</v>
       </c>
       <c r="AO19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AP19" s="51" t="n">
-        <v>2069.052711417807</v>
+        <v>1043.029191070895</v>
       </c>
       <c r="AQ19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AR19" s="51" t="n">
-        <v>2123.486645487587</v>
+        <v>1070.469859204702</v>
       </c>
       <c r="AS19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AT19" s="51" t="n">
-        <v>2177.78446514536</v>
+        <v>1097.841910758209</v>
       </c>
       <c r="AU19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AV19" s="51" t="n">
-        <v>2245.65149973365</v>
+        <v>1128.961289046425</v>
       </c>
       <c r="AW19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AX19" s="51" t="n">
-        <v>2292.856274948349</v>
+        <v>1155.850713508209</v>
       </c>
       <c r="AY19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AZ19" s="51" t="n">
-        <v>2340.49220852488</v>
+        <v>1179.864444407063</v>
       </c>
       <c r="BA19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BB19" s="51" t="n">
-        <v>2408.838509859194</v>
+        <v>1214.318470285183</v>
       </c>
       <c r="BC19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BD19" s="51" t="n">
-        <v>2454.229928750568</v>
+        <v>1233.820389972963</v>
       </c>
       <c r="BE19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BF19" s="51" t="n">
-        <v>2485.912486082782</v>
+        <v>1253.172200765019</v>
       </c>
       <c r="BG19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BH19" s="51" t="n">
-        <v>2513.739657489311</v>
+        <v>1267.200144706941</v>
       </c>
       <c r="BI19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BJ19" s="51" t="n">
-        <v>2521.13112495652</v>
+        <v>1270.926254334245</v>
       </c>
       <c r="BK19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>35403.7115717776</v>
+        <v>20140.22414240874</v>
       </c>
       <c r="BM19" s="58" t="inlineStr">
         <is>
@@ -23735,82 +23735,82 @@
         </is>
       </c>
       <c r="C23" s="51" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="D23" s="51" t="n">
-        <v>651.9713368714761</v>
+        <v>24344.88562540607</v>
       </c>
       <c r="E23" s="51" t="n">
-        <v>1267.067980863357</v>
+        <v>23636.90370556742</v>
       </c>
       <c r="F23" s="51" t="n">
-        <v>1867.641320549154</v>
+        <v>22902.35457688584</v>
       </c>
       <c r="G23" s="51" t="n">
-        <v>2429.894606271477</v>
+        <v>22112.42722334773</v>
       </c>
       <c r="H23" s="51" t="n">
-        <v>2973.963263272183</v>
+        <v>21287.88245892156</v>
       </c>
       <c r="I23" s="51" t="n">
-        <v>3488.445740478266</v>
+        <v>20416.09394389152</v>
       </c>
       <c r="J23" s="51" t="n">
-        <v>3975.276382855849</v>
+        <v>19507.14185243584</v>
       </c>
       <c r="K23" s="51" t="n">
-        <v>4883.320124286082</v>
+        <v>18537.32106762657</v>
       </c>
       <c r="L23" s="51" t="n">
-        <v>5775.182407670217</v>
+        <v>17540.68611484873</v>
       </c>
       <c r="M23" s="51" t="n">
-        <v>5997.039416826485</v>
+        <v>16480.46273024089</v>
       </c>
       <c r="N23" s="51" t="n">
-        <v>6217.071531782984</v>
+        <v>15360.31588876499</v>
       </c>
       <c r="O23" s="51" t="n">
-        <v>6432.67302346948</v>
+        <v>14172.62862752015</v>
       </c>
       <c r="P23" s="51" t="n">
-        <v>6634.955874792573</v>
+        <v>12919.40998193439</v>
       </c>
       <c r="Q23" s="51" t="n">
-        <v>6842.315869108428</v>
+        <v>11606.45808531499</v>
       </c>
       <c r="R23" s="51" t="n">
-        <v>7003.440791089856</v>
+        <v>10221.13317892016</v>
       </c>
       <c r="S23" s="51" t="n">
-        <v>7169.121331451536</v>
+        <v>8759.841590781387</v>
       </c>
       <c r="T23" s="51" t="n">
-        <v>6840.968683068615</v>
+        <v>7224.798152032797</v>
       </c>
       <c r="U23" s="51" t="n">
-        <v>6503.273832188852</v>
+        <v>5609.035449333731</v>
       </c>
       <c r="V23" s="51" t="n">
-        <v>6111.731177109747</v>
+        <v>3919.300509790613</v>
       </c>
       <c r="W23" s="51" t="n">
-        <v>5730.601602999086</v>
+        <v>2143.965938241631</v>
       </c>
       <c r="X23" s="51" t="n">
-        <v>5308.696443709642</v>
+        <v>287.4679422773584</v>
       </c>
       <c r="Y23" s="51" t="n">
-        <v>4916.038308456874</v>
+        <v>0</v>
       </c>
       <c r="Z23" s="51" t="n">
-        <v>4443.940410991425</v>
+        <v>0</v>
       </c>
       <c r="AA23" s="51" t="n">
-        <v>4014.477402404407</v>
+        <v>0</v>
       </c>
       <c r="AB23" s="51" t="n">
-        <v>1151.732789433225</v>
+        <v>0</v>
       </c>
       <c r="AC23" s="51" t="n">
         <v>0</v>
@@ -23918,7 +23918,7 @@
         <v>0</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>118630.8416520013</v>
+        <v>323990.5146440843</v>
       </c>
       <c r="BM23" s="58" t="inlineStr">
         <is>
@@ -24627,70 +24627,70 @@
         </is>
       </c>
       <c r="C27" s="51" t="n">
-        <v>0</v>
+        <v>655.1143745939253</v>
       </c>
       <c r="D27" s="51" t="n">
-        <v>0</v>
+        <v>707.9819198386576</v>
       </c>
       <c r="E27" s="51" t="n">
-        <v>0</v>
+        <v>734.549128681577</v>
       </c>
       <c r="F27" s="51" t="n">
-        <v>0</v>
+        <v>789.9273535381026</v>
       </c>
       <c r="G27" s="51" t="n">
-        <v>0</v>
+        <v>824.5447644261715</v>
       </c>
       <c r="H27" s="51" t="n">
-        <v>0</v>
+        <v>871.7885150300467</v>
       </c>
       <c r="I27" s="51" t="n">
-        <v>0</v>
+        <v>908.9520914556761</v>
       </c>
       <c r="J27" s="51" t="n">
-        <v>0</v>
+        <v>969.8207848092713</v>
       </c>
       <c r="K27" s="51" t="n">
-        <v>0</v>
+        <v>996.6349527778393</v>
       </c>
       <c r="L27" s="51" t="n">
-        <v>0</v>
+        <v>1060.223384607837</v>
       </c>
       <c r="M27" s="51" t="n">
-        <v>0</v>
+        <v>1120.146841475899</v>
       </c>
       <c r="N27" s="51" t="n">
-        <v>0</v>
+        <v>1187.687261244841</v>
       </c>
       <c r="O27" s="51" t="n">
-        <v>0</v>
+        <v>1253.218645585758</v>
       </c>
       <c r="P27" s="51" t="n">
-        <v>0</v>
+        <v>1312.951896619405</v>
       </c>
       <c r="Q27" s="51" t="n">
-        <v>0</v>
+        <v>1385.324906394822</v>
       </c>
       <c r="R27" s="51" t="n">
-        <v>0</v>
+        <v>1461.291588138776</v>
       </c>
       <c r="S27" s="51" t="n">
-        <v>0</v>
+        <v>1535.04343874859</v>
       </c>
       <c r="T27" s="51" t="n">
-        <v>0</v>
+        <v>1615.762702699066</v>
       </c>
       <c r="U27" s="51" t="n">
-        <v>0</v>
+        <v>1689.734939543118</v>
       </c>
       <c r="V27" s="51" t="n">
-        <v>0</v>
+        <v>1775.334571548982</v>
       </c>
       <c r="W27" s="51" t="n">
-        <v>0</v>
+        <v>1856.497995964273</v>
       </c>
       <c r="X27" s="51" t="n">
-        <v>0</v>
+        <v>287.4679422773584</v>
       </c>
       <c r="Y27" s="51" t="n">
         <v>0</v>
@@ -24699,10 +24699,10 @@
         <v>0</v>
       </c>
       <c r="AA27" s="51" t="n">
-        <v>2862.744612971182</v>
+        <v>0</v>
       </c>
       <c r="AB27" s="51" t="n">
-        <v>1151.732789433225</v>
+        <v>0</v>
       </c>
       <c r="AC27" s="51" t="n">
         <v>0</v>
@@ -24810,7 +24810,7 @@
         <v>0</v>
       </c>
       <c r="BL27" s="52" t="n">
-        <v>4014.477402404407</v>
+        <v>25000</v>
       </c>
       <c r="BM27" s="58" t="inlineStr">
         <is>
@@ -25519,79 +25519,79 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>651.9713368714761</v>
+        <v>24344.88562540607</v>
       </c>
       <c r="D31" s="51" t="n">
-        <v>1267.067980863357</v>
+        <v>23636.90370556742</v>
       </c>
       <c r="E31" s="51" t="n">
-        <v>1867.641320549154</v>
+        <v>22902.35457688584</v>
       </c>
       <c r="F31" s="51" t="n">
-        <v>2429.894606271477</v>
+        <v>22112.42722334773</v>
       </c>
       <c r="G31" s="51" t="n">
-        <v>2973.963263272183</v>
+        <v>21287.88245892156</v>
       </c>
       <c r="H31" s="51" t="n">
-        <v>3488.445740478266</v>
+        <v>20416.09394389152</v>
       </c>
       <c r="I31" s="51" t="n">
-        <v>3975.276382855849</v>
+        <v>19507.14185243584</v>
       </c>
       <c r="J31" s="51" t="n">
-        <v>4883.320124286082</v>
+        <v>18537.32106762657</v>
       </c>
       <c r="K31" s="51" t="n">
-        <v>5775.182407670217</v>
+        <v>17540.68611484873</v>
       </c>
       <c r="L31" s="51" t="n">
-        <v>6649.010753697961</v>
+        <v>16480.46273024089</v>
       </c>
       <c r="M31" s="51" t="n">
-        <v>6832.168175774865</v>
+        <v>15360.31588876499</v>
       </c>
       <c r="N31" s="51" t="n">
-        <v>7033.246363155276</v>
+        <v>14172.62862752015</v>
       </c>
       <c r="O31" s="51" t="n">
-        <v>7197.209160514896</v>
+        <v>12919.40998193439</v>
       </c>
       <c r="P31" s="51" t="n">
-        <v>7386.384526109134</v>
+        <v>11606.45808531499</v>
       </c>
       <c r="Q31" s="51" t="n">
-        <v>7517.92326829594</v>
+        <v>10221.13317892016</v>
       </c>
       <c r="R31" s="51" t="n">
-        <v>7655.951973829119</v>
+        <v>8759.841590781387</v>
       </c>
       <c r="S31" s="51" t="n">
-        <v>7749.012424498849</v>
+        <v>7224.798152032797</v>
       </c>
       <c r="T31" s="51" t="n">
-        <v>7395.136115572986</v>
+        <v>5609.035449333731</v>
       </c>
       <c r="U31" s="51" t="n">
-        <v>6985.55952313749</v>
+        <v>3919.300509790613</v>
       </c>
       <c r="V31" s="51" t="n">
-        <v>6565.730361947466</v>
+        <v>2143.965938241631</v>
       </c>
       <c r="W31" s="51" t="n">
-        <v>6124.871275081935</v>
+        <v>287.4679422773584</v>
       </c>
       <c r="X31" s="51" t="n">
-        <v>5680.57444550229</v>
+        <v>0</v>
       </c>
       <c r="Y31" s="51" t="n">
-        <v>5195.369062307986</v>
+        <v>0</v>
       </c>
       <c r="Z31" s="51" t="n">
-        <v>4690.084801591918</v>
+        <v>0</v>
       </c>
       <c r="AA31" s="51" t="n">
-        <v>1151.732789433225</v>
+        <v>0</v>
       </c>
       <c r="AB31" s="51" t="n">
         <v>0</v>
@@ -25702,7 +25702,7 @@
         <v>0</v>
       </c>
       <c r="BL31" s="52" t="n">
-        <v>129122.7281835694</v>
+        <v>298990.5146440843</v>
       </c>
       <c r="BM31" s="58" t="inlineStr">
         <is>
@@ -26474,127 +26474,127 @@
         <v>0</v>
       </c>
       <c r="X35" s="51" t="n">
-        <v>0</v>
+        <v>1646.338424129087</v>
       </c>
       <c r="Y35" s="51" t="n">
-        <v>0</v>
+        <v>2022.69192865896</v>
       </c>
       <c r="Z35" s="51" t="n">
-        <v>0</v>
+        <v>2118.731443842721</v>
       </c>
       <c r="AA35" s="51" t="n">
-        <v>0</v>
+        <v>4607.278452375285</v>
       </c>
       <c r="AB35" s="51" t="n">
-        <v>1931.160129001509</v>
+        <v>4776.369613776</v>
       </c>
       <c r="AC35" s="51" t="n">
-        <v>3132.923854640633</v>
+        <v>4759.925290806009</v>
       </c>
       <c r="AD35" s="51" t="n">
-        <v>3365.333811679907</v>
+        <v>4933.314456006903</v>
       </c>
       <c r="AE35" s="51" t="n">
-        <v>3481.764336407045</v>
+        <v>5016.091417597368</v>
       </c>
       <c r="AF35" s="51" t="n">
-        <v>3721.063927205155</v>
+        <v>5071.213301307228</v>
       </c>
       <c r="AG35" s="51" t="n">
-        <v>3860.622417300403</v>
+        <v>5053.280910902247</v>
       </c>
       <c r="AH35" s="51" t="n">
-        <v>4146.96485784826</v>
+        <v>5137.036948099522</v>
       </c>
       <c r="AI35" s="51" t="n">
-        <v>4420.133097826707</v>
+        <v>5250.977421564884</v>
       </c>
       <c r="AJ35" s="51" t="n">
-        <v>4738.809323908284</v>
+        <v>5338.01019650795</v>
       </c>
       <c r="AK35" s="51" t="n">
-        <v>4971.01061773881</v>
+        <v>5401.780310394376</v>
       </c>
       <c r="AL35" s="51" t="n">
-        <v>5321.552297014329</v>
+        <v>5491.312580732402</v>
       </c>
       <c r="AM35" s="51" t="n">
-        <v>5557.698223429625</v>
+        <v>5564.135766234725</v>
       </c>
       <c r="AN35" s="51" t="n">
-        <v>5631.718991452662</v>
+        <v>5625.280115314228</v>
       </c>
       <c r="AO35" s="51" t="n">
-        <v>5690.44622932455</v>
+        <v>5700.129335260623</v>
       </c>
       <c r="AP35" s="51" t="n">
-        <v>5804.291056329932</v>
+        <v>5794.606617060525</v>
       </c>
       <c r="AQ35" s="51" t="n">
-        <v>5840.408817857736</v>
+        <v>5850.091923793809</v>
       </c>
       <c r="AR35" s="51" t="n">
-        <v>5956.73921262886</v>
+        <v>5947.054773359453</v>
       </c>
       <c r="AS35" s="51" t="n">
-        <v>5989.996418436989</v>
+        <v>5999.679524373062</v>
       </c>
       <c r="AT35" s="51" t="n">
-        <v>6108.806165703902</v>
+        <v>6099.121726434495</v>
       </c>
       <c r="AU35" s="51" t="n">
-        <v>6197.395627679482</v>
+        <v>6203.833170484581</v>
       </c>
       <c r="AV35" s="51" t="n">
-        <v>6278.446037507464</v>
+        <v>6272.007161369031</v>
       </c>
       <c r="AW35" s="51" t="n">
-        <v>6307.013124286929</v>
+        <v>6316.696230223002</v>
       </c>
       <c r="AX35" s="51" t="n">
-        <v>6431.07729209279</v>
+        <v>6421.392852823384</v>
       </c>
       <c r="AY35" s="51" t="n">
-        <v>6438.247583607354</v>
+        <v>6447.930689543427</v>
       </c>
       <c r="AZ35" s="51" t="n">
-        <v>6564.486908197535</v>
+        <v>6554.802468928128</v>
       </c>
       <c r="BA35" s="51" t="n">
-        <v>6626.538002808436</v>
+        <v>6636.221108744508</v>
       </c>
       <c r="BB35" s="51" t="n">
-        <v>6755.89816307598</v>
+        <v>6746.213723806573</v>
       </c>
       <c r="BC35" s="51" t="n">
-        <v>6773.614117070485</v>
+        <v>6780.051659875585</v>
       </c>
       <c r="BD35" s="51" t="n">
-        <v>6860.996598210452</v>
+        <v>6854.557722072019</v>
       </c>
       <c r="BE35" s="51" t="n">
-        <v>6838.872701384834</v>
+        <v>6848.555807320907</v>
       </c>
       <c r="BF35" s="51" t="n">
-        <v>6971.752221297289</v>
+        <v>6962.067782027882</v>
       </c>
       <c r="BG35" s="51" t="n">
-        <v>6915.535076188208</v>
+        <v>6925.218182124281</v>
       </c>
       <c r="BH35" s="51" t="n">
-        <v>7049.685243196855</v>
+        <v>7040.000803927449</v>
       </c>
       <c r="BI35" s="51" t="n">
-        <v>6935.898175298783</v>
+        <v>6945.581281234856</v>
       </c>
       <c r="BJ35" s="51" t="n">
-        <v>7070.385852237438</v>
+        <v>7060.70141296803</v>
       </c>
       <c r="BK35" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL35" s="52" t="n">
-        <v>196743.4109358929</v>
+        <v>220276.4089620228</v>
       </c>
       <c r="BM35" s="58" t="inlineStr">
         <is>
@@ -27366,127 +27366,127 @@
         <v>0</v>
       </c>
       <c r="X39" s="51" t="n">
-        <v>0</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y39" s="51" t="n">
-        <v>0</v>
+        <v>364.0845471586127</v>
       </c>
       <c r="Z39" s="51" t="n">
-        <v>0</v>
+        <v>381.3716598916898</v>
       </c>
       <c r="AA39" s="51" t="n">
-        <v>0</v>
+        <v>829.3101214275513</v>
       </c>
       <c r="AB39" s="51" t="n">
-        <v>347.6088232202716</v>
+        <v>859.7465304796799</v>
       </c>
       <c r="AC39" s="51" t="n">
-        <v>563.9262938353139</v>
+        <v>856.7865523450815</v>
       </c>
       <c r="AD39" s="51" t="n">
-        <v>605.7600861023833</v>
+        <v>887.9966020812425</v>
       </c>
       <c r="AE39" s="51" t="n">
-        <v>626.717580553268</v>
+        <v>902.8964551675261</v>
       </c>
       <c r="AF39" s="51" t="n">
-        <v>669.7915068969279</v>
+        <v>912.818394235301</v>
       </c>
       <c r="AG39" s="51" t="n">
-        <v>694.9120351140726</v>
+        <v>909.5905639624045</v>
       </c>
       <c r="AH39" s="51" t="n">
-        <v>746.4536744126868</v>
+        <v>924.666650657914</v>
       </c>
       <c r="AI39" s="51" t="n">
-        <v>795.6239576088072</v>
+        <v>945.175935881679</v>
       </c>
       <c r="AJ39" s="51" t="n">
-        <v>852.985678303491</v>
+        <v>960.841835371431</v>
       </c>
       <c r="AK39" s="51" t="n">
-        <v>894.7819111929857</v>
+        <v>972.3204558709876</v>
       </c>
       <c r="AL39" s="51" t="n">
-        <v>957.8794134625792</v>
+        <v>988.4362645318324</v>
       </c>
       <c r="AM39" s="51" t="n">
-        <v>1000.385680217332</v>
+        <v>1001.54443792225</v>
       </c>
       <c r="AN39" s="51" t="n">
-        <v>1013.709418461479</v>
+        <v>1012.550420756561</v>
       </c>
       <c r="AO39" s="51" t="n">
-        <v>1024.280321278419</v>
+        <v>1026.023280346912</v>
       </c>
       <c r="AP39" s="51" t="n">
-        <v>1044.772390139388</v>
+        <v>1043.029191070895</v>
       </c>
       <c r="AQ39" s="51" t="n">
-        <v>1051.273587214392</v>
+        <v>1053.016546282885</v>
       </c>
       <c r="AR39" s="51" t="n">
-        <v>1072.213058273195</v>
+        <v>1070.469859204702</v>
       </c>
       <c r="AS39" s="51" t="n">
-        <v>1078.199355318658</v>
+        <v>1079.942314387151</v>
       </c>
       <c r="AT39" s="51" t="n">
-        <v>1099.585109826702</v>
+        <v>1097.841910758209</v>
       </c>
       <c r="AU39" s="51" t="n">
-        <v>1115.531212982307</v>
+        <v>1116.689970687225</v>
       </c>
       <c r="AV39" s="51" t="n">
-        <v>1130.120286751343</v>
+        <v>1128.961289046425</v>
       </c>
       <c r="AW39" s="51" t="n">
-        <v>1135.262362371647</v>
+        <v>1137.00532144014</v>
       </c>
       <c r="AX39" s="51" t="n">
-        <v>1157.593912576702</v>
+        <v>1155.850713508209</v>
       </c>
       <c r="AY39" s="51" t="n">
-        <v>1158.884565049324</v>
+        <v>1160.627524117817</v>
       </c>
       <c r="AZ39" s="51" t="n">
-        <v>1181.607643475556</v>
+        <v>1179.864444407063</v>
       </c>
       <c r="BA39" s="51" t="n">
-        <v>1192.776840505518</v>
+        <v>1194.519799574012</v>
       </c>
       <c r="BB39" s="51" t="n">
-        <v>1216.061669353676</v>
+        <v>1214.318470285183</v>
       </c>
       <c r="BC39" s="51" t="n">
-        <v>1219.250541072687</v>
+        <v>1220.409298777605</v>
       </c>
       <c r="BD39" s="51" t="n">
-        <v>1234.979387677881</v>
+        <v>1233.820389972963</v>
       </c>
       <c r="BE39" s="51" t="n">
-        <v>1230.99708624927</v>
+        <v>1232.740045317763</v>
       </c>
       <c r="BF39" s="51" t="n">
-        <v>1254.915399833512</v>
+        <v>1253.172200765019</v>
       </c>
       <c r="BG39" s="51" t="n">
-        <v>1244.796313713877</v>
+        <v>1246.539272782371</v>
       </c>
       <c r="BH39" s="51" t="n">
-        <v>1268.943343775434</v>
+        <v>1267.200144706941</v>
       </c>
       <c r="BI39" s="51" t="n">
-        <v>1248.461671553781</v>
+        <v>1250.204630622274</v>
       </c>
       <c r="BJ39" s="51" t="n">
-        <v>1272.669453402739</v>
+        <v>1270.926254334245</v>
       </c>
       <c r="BK39" s="51" t="n">
         <v>10.10239668311311</v>
       </c>
       <c r="BL39" s="52" t="n">
-        <v>35413.81396846072</v>
+        <v>39649.75361316411</v>
       </c>
       <c r="BM39" s="58" t="inlineStr">
         <is>
@@ -28258,127 +28258,127 @@
         <v>0</v>
       </c>
       <c r="X43" s="51" t="n">
-        <v>0</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="Z43" s="51" t="n">
-        <v>0</v>
+        <v>381.3716598916898</v>
       </c>
       <c r="AA43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AB43" s="51" t="n">
-        <v>347.6088232202716</v>
+        <v>859.7465304796799</v>
       </c>
       <c r="AC43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AD43" s="51" t="n">
-        <v>1169.686379937697</v>
+        <v>887.9966020812425</v>
       </c>
       <c r="AE43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AF43" s="51" t="n">
-        <v>1296.509087450196</v>
+        <v>912.818394235301</v>
       </c>
       <c r="AG43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AH43" s="51" t="n">
-        <v>1441.365709526759</v>
+        <v>924.666650657914</v>
       </c>
       <c r="AI43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AJ43" s="51" t="n">
-        <v>1648.609635912298</v>
+        <v>960.841835371431</v>
       </c>
       <c r="AK43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AL43" s="51" t="n">
-        <v>1852.661324655565</v>
+        <v>988.4362645318324</v>
       </c>
       <c r="AM43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AN43" s="51" t="n">
-        <v>2014.095098678811</v>
+        <v>1012.550420756561</v>
       </c>
       <c r="AO43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AP43" s="51" t="n">
-        <v>2069.052711417807</v>
+        <v>1043.029191070895</v>
       </c>
       <c r="AQ43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AR43" s="51" t="n">
-        <v>2123.486645487587</v>
+        <v>1070.469859204702</v>
       </c>
       <c r="AS43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AT43" s="51" t="n">
-        <v>2177.78446514536</v>
+        <v>1097.841910758209</v>
       </c>
       <c r="AU43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AV43" s="51" t="n">
-        <v>2245.65149973365</v>
+        <v>1128.961289046425</v>
       </c>
       <c r="AW43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AX43" s="51" t="n">
-        <v>2292.856274948349</v>
+        <v>1155.850713508209</v>
       </c>
       <c r="AY43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AZ43" s="51" t="n">
-        <v>2340.49220852488</v>
+        <v>1179.864444407063</v>
       </c>
       <c r="BA43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BB43" s="51" t="n">
-        <v>2408.838509859194</v>
+        <v>1214.318470285183</v>
       </c>
       <c r="BC43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BD43" s="51" t="n">
-        <v>2454.229928750568</v>
+        <v>1233.820389972963</v>
       </c>
       <c r="BE43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BF43" s="51" t="n">
-        <v>2485.912486082782</v>
+        <v>1253.172200765019</v>
       </c>
       <c r="BG43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BH43" s="51" t="n">
-        <v>2513.739657489311</v>
+        <v>1267.200144706941</v>
       </c>
       <c r="BI43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BJ43" s="51" t="n">
-        <v>2521.13112495652</v>
+        <v>1270.926254334245</v>
       </c>
       <c r="BK43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BL43" s="52" t="n">
-        <v>35403.7115717776</v>
+        <v>20140.22414240874</v>
       </c>
       <c r="BM43" s="58" t="inlineStr">
         <is>
@@ -30267,127 +30267,127 @@
         <v>0</v>
       </c>
       <c r="X11" s="51" t="n">
-        <v>0</v>
+        <v>296.3409163432357</v>
       </c>
       <c r="Y11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="Z11" s="51" t="n">
-        <v>0</v>
+        <v>381.3716598916898</v>
       </c>
       <c r="AA11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AB11" s="51" t="n">
-        <v>347.6088232202716</v>
+        <v>859.7465304796799</v>
       </c>
       <c r="AC11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AD11" s="51" t="n">
-        <v>1169.686379937697</v>
+        <v>887.9966020812425</v>
       </c>
       <c r="AE11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AF11" s="51" t="n">
-        <v>1296.509087450196</v>
+        <v>912.818394235301</v>
       </c>
       <c r="AG11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AH11" s="51" t="n">
-        <v>1441.365709526759</v>
+        <v>924.666650657914</v>
       </c>
       <c r="AI11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AJ11" s="51" t="n">
-        <v>1648.609635912298</v>
+        <v>960.841835371431</v>
       </c>
       <c r="AK11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AL11" s="51" t="n">
-        <v>1852.661324655565</v>
+        <v>988.4362645318324</v>
       </c>
       <c r="AM11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AN11" s="51" t="n">
-        <v>2014.095098678811</v>
+        <v>1012.550420756561</v>
       </c>
       <c r="AO11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AP11" s="51" t="n">
-        <v>2069.052711417807</v>
+        <v>1043.029191070895</v>
       </c>
       <c r="AQ11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AR11" s="51" t="n">
-        <v>2123.486645487587</v>
+        <v>1070.469859204702</v>
       </c>
       <c r="AS11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AT11" s="51" t="n">
-        <v>2177.78446514536</v>
+        <v>1097.841910758209</v>
       </c>
       <c r="AU11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AV11" s="51" t="n">
-        <v>2245.65149973365</v>
+        <v>1128.961289046425</v>
       </c>
       <c r="AW11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AX11" s="51" t="n">
-        <v>2292.856274948349</v>
+        <v>1155.850713508209</v>
       </c>
       <c r="AY11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AZ11" s="51" t="n">
-        <v>2340.49220852488</v>
+        <v>1179.864444407063</v>
       </c>
       <c r="BA11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BB11" s="51" t="n">
-        <v>2408.838509859194</v>
+        <v>1214.318470285183</v>
       </c>
       <c r="BC11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BD11" s="51" t="n">
-        <v>2454.229928750568</v>
+        <v>1233.820389972963</v>
       </c>
       <c r="BE11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BF11" s="51" t="n">
-        <v>2485.912486082782</v>
+        <v>1253.172200765019</v>
       </c>
       <c r="BG11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BH11" s="51" t="n">
-        <v>2513.739657489311</v>
+        <v>1267.200144706941</v>
       </c>
       <c r="BI11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BJ11" s="51" t="n">
-        <v>2521.13112495652</v>
+        <v>1270.926254334245</v>
       </c>
       <c r="BK11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>35403.7115717776</v>
+        <v>20140.22414240874</v>
       </c>
       <c r="BM11" s="58" t="inlineStr">
         <is>
@@ -31159,127 +31159,127 @@
         <v>3607.952524064416</v>
       </c>
       <c r="X15" s="51" t="n">
-        <v>3647.600353999189</v>
+        <v>3351.259437655953</v>
       </c>
       <c r="Y15" s="51" t="n">
         <v>3667.635538833556</v>
       </c>
       <c r="Z15" s="51" t="n">
-        <v>3728.425078151239</v>
+        <v>3347.053418259549</v>
       </c>
       <c r="AA15" s="51" t="n">
         <v>6140.284473381875</v>
       </c>
       <c r="AB15" s="51" t="n">
-        <v>5894.448320991136</v>
+        <v>5382.310613731728</v>
       </c>
       <c r="AC15" s="51" t="n">
         <v>6115.456541519213</v>
       </c>
       <c r="AD15" s="51" t="n">
-        <v>5047.131319728243</v>
+        <v>5328.821097584698</v>
       </c>
       <c r="AE15" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF15" s="51" t="n">
-        <v>4959.334756662132</v>
+        <v>5343.025449877027</v>
       </c>
       <c r="AG15" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH15" s="51" t="n">
-        <v>4883.547344508836</v>
+        <v>5400.246403377681</v>
       </c>
       <c r="AI15" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ15" s="51" t="n">
-        <v>4877.276666531725</v>
+        <v>5565.044467072592</v>
       </c>
       <c r="AK15" s="51" t="n">
         <v>6570.28887112497</v>
       </c>
       <c r="AL15" s="51" t="n">
-        <v>4826.52736201291</v>
+        <v>5690.752422136643</v>
       </c>
       <c r="AM15" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN15" s="51" t="n">
-        <v>4795.815559440517</v>
+        <v>5797.360237362767</v>
       </c>
       <c r="AO15" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP15" s="51" t="n">
-        <v>4913.430011578792</v>
+        <v>5939.453531925704</v>
       </c>
       <c r="AQ15" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR15" s="51" t="n">
-        <v>5011.444233807939</v>
+        <v>6064.461020090825</v>
       </c>
       <c r="AS15" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT15" s="51" t="n">
-        <v>5109.213367225208</v>
+        <v>6189.155921612359</v>
       </c>
       <c r="AU15" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV15" s="51" t="n">
-        <v>5210.986204440481</v>
+        <v>6327.676415127706</v>
       </c>
       <c r="AW15" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX15" s="51" t="n">
-        <v>5316.412683811108</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY15" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ15" s="51" t="n">
-        <v>5402.186366339321</v>
+        <v>6562.814130457138</v>
       </c>
       <c r="BA15" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB15" s="51" t="n">
-        <v>5525.251319883452</v>
+        <v>6719.771359457463</v>
       </c>
       <c r="BC15" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD15" s="51" t="n">
-        <v>5584.95833612655</v>
+        <v>6805.367874904156</v>
       </c>
       <c r="BE15" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF15" s="51" t="n">
-        <v>5664.031401881173</v>
+        <v>6896.771687198937</v>
       </c>
       <c r="BG15" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH15" s="51" t="n">
-        <v>5714.13725237421</v>
+        <v>6960.676765156581</v>
       </c>
       <c r="BI15" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ15" s="51" t="n">
-        <v>5727.446393947584</v>
+        <v>6977.651264569858</v>
       </c>
       <c r="BK15" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>303031.6256704517</v>
+        <v>318295.1130998204</v>
       </c>
       <c r="BM15" s="58" t="inlineStr">
         <is>
@@ -31807,127 +31807,127 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>1284.405766824072</v>
+        <v>988.064850480836</v>
       </c>
       <c r="Y19" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>1312.866050771856</v>
+        <v>931.4943908801665</v>
       </c>
       <c r="AA19" s="51" t="n">
         <v>2760.620551308993</v>
       </c>
       <c r="AB19" s="51" t="n">
-        <v>2458.767869823124</v>
+        <v>1946.630162563717</v>
       </c>
       <c r="AC19" s="51" t="n">
         <v>2749.45812076629</v>
       </c>
       <c r="AD19" s="51" t="n">
-        <v>1625.342869902177</v>
+        <v>1907.032647758631</v>
       </c>
       <c r="AE19" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF19" s="51" t="n">
-        <v>4959.334756662132</v>
+        <v>5343.025449877027</v>
       </c>
       <c r="AG19" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH19" s="51" t="n">
-        <v>4883.547344508836</v>
+        <v>5400.246403377681</v>
       </c>
       <c r="AI19" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ19" s="51" t="n">
-        <v>4877.276666531725</v>
+        <v>5565.044467072592</v>
       </c>
       <c r="AK19" s="51" t="n">
         <v>6570.28887112497</v>
       </c>
       <c r="AL19" s="51" t="n">
-        <v>4826.52736201291</v>
+        <v>5690.752422136643</v>
       </c>
       <c r="AM19" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN19" s="51" t="n">
-        <v>4795.815559440517</v>
+        <v>5797.360237362767</v>
       </c>
       <c r="AO19" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP19" s="51" t="n">
-        <v>4913.430011578792</v>
+        <v>5939.453531925704</v>
       </c>
       <c r="AQ19" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR19" s="51" t="n">
-        <v>5011.444233807939</v>
+        <v>6064.461020090825</v>
       </c>
       <c r="AS19" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT19" s="51" t="n">
-        <v>5109.213367225208</v>
+        <v>6189.155921612359</v>
       </c>
       <c r="AU19" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV19" s="51" t="n">
-        <v>5210.986204440481</v>
+        <v>6327.676415127706</v>
       </c>
       <c r="AW19" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX19" s="51" t="n">
-        <v>5316.412683811108</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY19" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ19" s="51" t="n">
-        <v>5402.186366339321</v>
+        <v>6562.814130457138</v>
       </c>
       <c r="BA19" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB19" s="51" t="n">
-        <v>5525.251319883452</v>
+        <v>6719.771359457463</v>
       </c>
       <c r="BC19" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD19" s="51" t="n">
-        <v>5584.95833612655</v>
+        <v>6805.367874904156</v>
       </c>
       <c r="BE19" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF19" s="51" t="n">
-        <v>5664.031401881173</v>
+        <v>6896.771687198937</v>
       </c>
       <c r="BG19" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH19" s="51" t="n">
-        <v>5714.13725237421</v>
+        <v>6960.676765156581</v>
       </c>
       <c r="BI19" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ19" s="51" t="n">
-        <v>5727.446393947584</v>
+        <v>6977.651264569858</v>
       </c>
       <c r="BK19" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>237205.2373902452</v>
+        <v>252468.7248196141</v>
       </c>
       <c r="BM19" s="77" t="inlineStr">
         <is>
@@ -32455,127 +32455,127 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X23" s="51" t="n">
-        <v>1284.405766824072</v>
+        <v>988.064850480836</v>
       </c>
       <c r="Y23" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z23" s="51" t="n">
-        <v>1312.866050771856</v>
+        <v>931.4943908801665</v>
       </c>
       <c r="AA23" s="51" t="n">
         <v>2760.620551308993</v>
       </c>
       <c r="AB23" s="51" t="n">
-        <v>2458.767869823124</v>
+        <v>1946.630162563717</v>
       </c>
       <c r="AC23" s="51" t="n">
         <v>2749.45812076629</v>
       </c>
       <c r="AD23" s="51" t="n">
-        <v>1625.342869902177</v>
+        <v>1907.032647758631</v>
       </c>
       <c r="AE23" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF23" s="51" t="n">
-        <v>4959.334756662132</v>
+        <v>5343.025449877027</v>
       </c>
       <c r="AG23" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH23" s="51" t="n">
-        <v>4883.547344508836</v>
+        <v>5400.246403377681</v>
       </c>
       <c r="AI23" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ23" s="51" t="n">
-        <v>4877.276666531725</v>
+        <v>5565.044467072592</v>
       </c>
       <c r="AK23" s="51" t="n">
         <v>6570.28887112497</v>
       </c>
       <c r="AL23" s="51" t="n">
-        <v>4826.52736201291</v>
+        <v>5690.752422136643</v>
       </c>
       <c r="AM23" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN23" s="51" t="n">
-        <v>4795.815559440517</v>
+        <v>5797.360237362767</v>
       </c>
       <c r="AO23" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP23" s="51" t="n">
-        <v>4913.430011578792</v>
+        <v>5939.453531925704</v>
       </c>
       <c r="AQ23" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR23" s="51" t="n">
-        <v>5011.444233807939</v>
+        <v>6064.461020090825</v>
       </c>
       <c r="AS23" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT23" s="51" t="n">
-        <v>5109.213367225208</v>
+        <v>6189.155921612359</v>
       </c>
       <c r="AU23" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV23" s="51" t="n">
-        <v>5210.986204440481</v>
+        <v>6327.676415127706</v>
       </c>
       <c r="AW23" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX23" s="51" t="n">
-        <v>5316.412683811108</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY23" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ23" s="51" t="n">
-        <v>5402.186366339321</v>
+        <v>6562.814130457138</v>
       </c>
       <c r="BA23" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB23" s="51" t="n">
-        <v>5525.251319883452</v>
+        <v>6719.771359457463</v>
       </c>
       <c r="BC23" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD23" s="51" t="n">
-        <v>5584.95833612655</v>
+        <v>6805.367874904156</v>
       </c>
       <c r="BE23" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF23" s="51" t="n">
-        <v>5664.031401881173</v>
+        <v>6896.771687198937</v>
       </c>
       <c r="BG23" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH23" s="51" t="n">
-        <v>5714.13725237421</v>
+        <v>6960.676765156581</v>
       </c>
       <c r="BI23" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ23" s="51" t="n">
-        <v>5727.446393947584</v>
+        <v>6977.651264569858</v>
       </c>
       <c r="BK23" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>237205.2373902452</v>
+        <v>252468.7248196141</v>
       </c>
       <c r="BM23" s="77" t="inlineStr">
         <is>
@@ -33755,88 +33755,88 @@
         <v>0</v>
       </c>
       <c r="AK7" s="51" t="n">
-        <v>6449.538993624739</v>
+        <v>6398.064261517846</v>
       </c>
       <c r="AL7" s="51" t="n">
-        <v>4740.166944215696</v>
+        <v>5690.752422136643</v>
       </c>
       <c r="AM7" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN7" s="51" t="n">
-        <v>4795.815799440517</v>
+        <v>5797.360237362767</v>
       </c>
       <c r="AO7" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP7" s="51" t="n">
-        <v>4913.430251578792</v>
+        <v>5939.453531925704</v>
       </c>
       <c r="AQ7" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR7" s="51" t="n">
-        <v>5011.444473807939</v>
+        <v>6064.461020090825</v>
       </c>
       <c r="AS7" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT7" s="51" t="n">
-        <v>5109.213607225208</v>
+        <v>6189.155921612359</v>
       </c>
       <c r="AU7" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV7" s="51" t="n">
-        <v>5210.986444440481</v>
+        <v>6327.676415127706</v>
       </c>
       <c r="AW7" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX7" s="51" t="n">
-        <v>5316.412923811107</v>
+        <v>6453.418245251248</v>
       </c>
       <c r="AY7" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ7" s="51" t="n">
-        <v>5402.186606339322</v>
+        <v>6562.814130457138</v>
       </c>
       <c r="BA7" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB7" s="51" t="n">
-        <v>5525.251559883452</v>
+        <v>6719.771359457463</v>
       </c>
       <c r="BC7" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD7" s="51" t="n">
-        <v>5584.95857612655</v>
+        <v>6805.367874904156</v>
       </c>
       <c r="BE7" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF7" s="51" t="n">
-        <v>5664.031641881174</v>
+        <v>6896.771687198937</v>
       </c>
       <c r="BG7" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH7" s="51" t="n">
-        <v>5714.137492374211</v>
+        <v>6960.676765156581</v>
       </c>
       <c r="BI7" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ7" s="51" t="n">
-        <v>5727.446633947584</v>
+        <v>6977.651264569858</v>
       </c>
       <c r="BK7" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>165471.1104720874</v>
+        <v>180089.4836601599</v>
       </c>
       <c r="BM7" s="79" t="inlineStr">
         <is>
@@ -33967,88 +33967,88 @@
         <v>0</v>
       </c>
       <c r="AK8" s="51" t="n">
-        <v>6449.538993624739</v>
+        <v>6398.064261517846</v>
       </c>
       <c r="AL8" s="51" t="n">
-        <v>4737.8779021845</v>
+        <v>5688.463380105447</v>
       </c>
       <c r="AM8" s="51" t="n">
         <v>6279.82438136977</v>
       </c>
       <c r="AN8" s="51" t="n">
-        <v>-1959.429144773435</v>
+        <v>-957.884706851185</v>
       </c>
       <c r="AO8" s="51" t="n">
         <v>1829.598176827532</v>
       </c>
       <c r="AP8" s="51" t="n">
-        <v>-1985.258154936995</v>
+        <v>-959.2348745900836</v>
       </c>
       <c r="AQ8" s="51" t="n">
         <v>2399.662843169288</v>
       </c>
       <c r="AR8" s="51" t="n">
-        <v>-2011.917109238403</v>
+        <v>-958.9005629555177</v>
       </c>
       <c r="AS8" s="51" t="n">
         <v>2553.912986264261</v>
       </c>
       <c r="AT8" s="51" t="n">
-        <v>-2078.87031963043</v>
+        <v>-998.9280052432796</v>
       </c>
       <c r="AU8" s="51" t="n">
         <v>2653.013886220987</v>
       </c>
       <c r="AV8" s="51" t="n">
-        <v>-2200.436815279101</v>
+        <v>-1083.746844591877</v>
       </c>
       <c r="AW8" s="51" t="n">
         <v>2650.095104931563</v>
       </c>
       <c r="AX8" s="51" t="n">
-        <v>-2221.180840919063</v>
+        <v>-1084.175519478922</v>
       </c>
       <c r="AY8" s="51" t="n">
         <v>2664.474182350282</v>
       </c>
       <c r="AZ8" s="51" t="n">
-        <v>-2284.155045305553</v>
+        <v>-1123.527521187737</v>
       </c>
       <c r="BA8" s="51" t="n">
         <v>2754.947169664165</v>
       </c>
       <c r="BB8" s="51" t="n">
-        <v>-2329.878229089789</v>
+        <v>-1135.358429515777</v>
       </c>
       <c r="BC8" s="51" t="n">
         <v>2791.409369359826</v>
       </c>
       <c r="BD8" s="51" t="n">
-        <v>-2436.795736644717</v>
+        <v>-1216.386437867111</v>
       </c>
       <c r="BE8" s="51" t="n">
         <v>2784.06653034275</v>
       </c>
       <c r="BF8" s="51" t="n">
-        <v>-2443.096749953369</v>
+        <v>-1210.356704635606</v>
       </c>
       <c r="BG8" s="51" t="n">
         <v>2767.937934958465</v>
       </c>
       <c r="BH8" s="51" t="n">
-        <v>-2491.048874562813</v>
+        <v>-1244.509601780442</v>
       </c>
       <c r="BI8" s="51" t="n">
         <v>2724.195775499138</v>
       </c>
       <c r="BJ8" s="51" t="n">
-        <v>-2520.688204336309</v>
+        <v>-1270.483573714036</v>
       </c>
       <c r="BK8" s="51" t="n">
         <v>-5316.083126731314</v>
       </c>
       <c r="BL8" s="80" t="n">
-        <v>13761.71688536589</v>
+        <v>28380.09007343833</v>
       </c>
       <c r="BM8" s="79" t="inlineStr">
         <is>
@@ -37638,7 +37638,7 @@
       <c r="BJ11" s="70" t="inlineStr"/>
       <c r="BK11" s="70" t="inlineStr"/>
       <c r="BL11" s="83" t="n">
-        <v>0.1132136369574784</v>
+        <v>0.1158773428956301</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -37972,7 +37972,7 @@
         </is>
       </c>
       <c r="BL12" s="85" t="n">
-        <v>-0.002886363042521586</v>
+        <v>-0.0002226571043698472</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -40917,7 +40917,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03T20:06:50+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -41035,7 +41035,7 @@
       </c>
       <c r="B9" s="89" t="inlineStr">
         <is>
-          <t>0.113214</t>
+          <t>0.115877</t>
         </is>
       </c>
       <c r="C9" s="89" t="inlineStr">
@@ -41045,7 +41045,7 @@
       </c>
       <c r="D9" s="89" t="inlineStr">
         <is>
-          <t>-0.002886</t>
+          <t>-0.000223</t>
         </is>
       </c>
       <c r="E9" s="90" t="inlineStr">
@@ -41360,7 +41360,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CIRR Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-03T20:06:50+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -41412,7 +41412,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03T20:06:50+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -42376,7 +42376,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCalibration Residual Closeout&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-03T20:06:50+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -42532,7 +42532,7 @@
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>237205.23739024517</t>
+          <t>252468.7248196141</t>
         </is>
       </c>
       <c r="E6" s="21" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>237205.23739024517</t>
+          <t>252468.7248196141</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
@@ -42753,22 +42753,22 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Opening Balance</t>
+          <t>Debt Service</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>756328.0823817672</t>
+          <t>66181.34723683617</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>781474.3749637025</t>
+          <t>32853.2998091612</t>
         </is>
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>25146.292581935297</t>
+          <t>-33328.04742767497</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
@@ -42783,12 +42783,12 @@
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
+          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
         </is>
       </c>
       <c r="I9" s="21" t="inlineStr">
         <is>
-          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
+          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
         </is>
       </c>
       <c r="J9" s="21" t="inlineStr">
@@ -42818,7 +42818,7 @@
       </c>
       <c r="O9" s="21" t="inlineStr">
         <is>
-          <t>No debt sizing rewrite is implied.</t>
+          <t>Derived from existing interest and principal rows.</t>
         </is>
       </c>
     </row>
@@ -42830,22 +42830,22 @@
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>Closing Balance</t>
+          <t>Opening Balance</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>712969.5518136513</t>
+          <t>756328.0823817672</t>
         </is>
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>738115.3749637026</t>
+          <t>781474.3749637025</t>
         </is>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>25145.823150051292</t>
+          <t>25146.292581935297</t>
         </is>
       </c>
       <c r="F10" s="21" t="inlineStr">
@@ -42860,12 +42860,12 @@
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
+          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
         </is>
       </c>
       <c r="I10" s="21" t="inlineStr">
         <is>
-          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
+          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
         </is>
       </c>
       <c r="J10" s="21" t="inlineStr">
@@ -42895,34 +42895,34 @@
       </c>
       <c r="O10" s="21" t="inlineStr">
         <is>
-          <t>No runtime change implied.</t>
+          <t>No debt sizing rewrite is implied.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>SHL</t>
+          <t>Senior Debt</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Principal Repaid</t>
+          <t>Closing Balance</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>14595.529999999999</t>
+          <t>712969.5518136513</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>37326.33183100554</t>
+          <t>738115.3749637026</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>22730.80183100554</t>
+          <t>25145.823150051292</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
@@ -42937,22 +42937,22 @@
       </c>
       <c r="H11" s="21" t="inlineStr">
         <is>
-          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
+          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
         </is>
       </c>
       <c r="I11" s="21" t="inlineStr">
         <is>
-          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
+          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
         </is>
       </c>
       <c r="J11" s="21" t="inlineStr">
         <is>
-          <t>Stakeholder review only</t>
+          <t>Review only</t>
         </is>
       </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>Sponsor / SHL</t>
+          <t>Debt</t>
         </is>
       </c>
       <c r="L11" s="21" t="inlineStr">
@@ -42972,7 +42972,7 @@
       </c>
       <c r="O11" s="21" t="inlineStr">
         <is>
-          <t>No new SHL timing change is made here.</t>
+          <t>No runtime change implied.</t>
         </is>
       </c>
     </row>
@@ -42984,22 +42984,22 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Gross Accrued Interest</t>
+          <t>Principal Repaid</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>38755.380000000005</t>
+          <t>14595.529999999999</t>
         </is>
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>44068.95868964389</t>
+          <t>38028.01009465598</t>
         </is>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>5313.578689643888</t>
+          <t>23432.480094655984</t>
         </is>
       </c>
       <c r="F12" s="21" t="inlineStr">
@@ -43014,17 +43014,17 @@
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
+          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
         </is>
       </c>
       <c r="I12" s="21" t="inlineStr">
         <is>
-          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
+          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
         </is>
       </c>
       <c r="J12" s="21" t="inlineStr">
         <is>
-          <t>Review only</t>
+          <t>Stakeholder review only</t>
         </is>
       </c>
       <c r="K12" s="21" t="inlineStr">
@@ -43049,34 +43049,34 @@
       </c>
       <c r="O12" s="21" t="inlineStr">
         <is>
-          <t>Gross accrued interest is the authoritative model-side SHL P&amp;L bridge.</t>
+          <t>No new SHL timing change is made here.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>SHL</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>Total OPEX</t>
+          <t>Gross Accrued Interest</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>84674.77873934136</t>
+          <t>38755.380000000005</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>85408.27413448405</t>
+          <t>44736.24440845805</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>733.4953951426869</t>
+          <t>5980.864408458045</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -43091,22 +43091,22 @@
       </c>
       <c r="H13" s="21" t="inlineStr">
         <is>
-          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
+          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
         </is>
       </c>
       <c r="I13" s="21" t="inlineStr">
         <is>
-          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
+          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
         </is>
       </c>
       <c r="J13" s="21" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Review only</t>
         </is>
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Sponsor / SHL</t>
         </is>
       </c>
       <c r="L13" s="21" t="inlineStr">
@@ -43126,34 +43126,34 @@
       </c>
       <c r="O13" s="21" t="inlineStr">
         <is>
-          <t>Residual is documented rather than runtime-fixed here.</t>
+          <t>Gross accrued interest is the authoritative model-side SHL P&amp;L bridge.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Interest</t>
+          <t>Total OPEX</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>22822.816668720287</t>
+          <t>84674.77873934136</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>22467.388280206447</t>
+          <t>85408.27413448405</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>-355.4283885138393</t>
+          <t>733.4953951426869</t>
         </is>
       </c>
       <c r="F14" s="21" t="inlineStr">
@@ -43168,22 +43168,22 @@
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
-          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
+          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
         </is>
       </c>
       <c r="I14" s="21" t="inlineStr">
         <is>
-          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
+          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
         </is>
       </c>
       <c r="J14" s="21" t="inlineStr">
         <is>
-          <t>Review only</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
-          <t>Debt</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="L14" s="21" t="inlineStr">
@@ -43203,7 +43203,7 @@
       </c>
       <c r="O14" s="21" t="inlineStr">
         <is>
-          <t>The residual is small relative to total debt service.</t>
+          <t>Residual is documented rather than runtime-fixed here.</t>
         </is>
       </c>
     </row>
@@ -43215,22 +43215,22 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>Debt Service</t>
+          <t>Interest</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
         <is>
-          <t>66181.34723683617</t>
+          <t>22822.816668720287</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>65826.38828020645</t>
+          <t>22467.388280206447</t>
         </is>
       </c>
       <c r="E15" s="21" t="inlineStr">
         <is>
-          <t>-354.9589566297218</t>
+          <t>-355.4283885138393</t>
         </is>
       </c>
       <c r="F15" s="21" t="inlineStr">
@@ -43245,12 +43245,12 @@
       </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
+          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
         </is>
       </c>
       <c r="I15" s="21" t="inlineStr">
         <is>
-          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
+          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
         </is>
       </c>
       <c r="J15" s="21" t="inlineStr">
@@ -43280,7 +43280,7 @@
       </c>
       <c r="O15" s="21" t="inlineStr">
         <is>
-          <t>Derived from existing interest and principal rows.</t>
+          <t>The residual is small relative to total debt service.</t>
         </is>
       </c>
     </row>
@@ -43456,12 +43456,12 @@
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>0.11321363695747841</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>-0.0028863630425215864</t>
+          <t>-0.0002226571043698472</t>
         </is>
       </c>
       <c r="F18" s="21" t="inlineStr">
@@ -43610,7 +43610,7 @@
       </c>
       <c r="D20" s="21" t="inlineStr">
         <is>
-          <t>186251.52440432477</t>
+          <t>245276.4089620228</t>
         </is>
       </c>
       <c r="E20" s="21" t="inlineStr">
@@ -43687,12 +43687,12 @@
       </c>
       <c r="D21" s="21" t="inlineStr">
         <is>
-          <t>0.113214</t>
+          <t>0.115877</t>
         </is>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
-          <t>-0.002886</t>
+          <t>-0.000223</t>
         </is>
       </c>
       <c r="F21" s="21" t="inlineStr">
@@ -44303,7 +44303,7 @@
       </c>
       <c r="D29" s="21" t="inlineStr">
         <is>
-          <t>303031.62567045167</t>
+          <t>318295.11309982045</t>
         </is>
       </c>
       <c r="E29" s="21" t="inlineStr">
@@ -44380,7 +44380,7 @@
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
-          <t>35403.7115717776</t>
+          <t>20140.224142408744</t>
         </is>
       </c>
       <c r="E30" s="21" t="inlineStr">
@@ -44996,7 +44996,7 @@
       </c>
       <c r="D38" s="21" t="inlineStr">
         <is>
-          <t>38160.27336911231</t>
+          <t>38125.88082427603</t>
         </is>
       </c>
       <c r="E38" s="21" t="inlineStr">
@@ -45073,7 +45073,7 @@
       </c>
       <c r="D39" s="21" t="inlineStr">
         <is>
-          <t>1078873.6179616887</t>
+          <t>1095711.9348782978</t>
         </is>
       </c>
       <c r="E39" s="21" t="inlineStr">
@@ -45150,7 +45150,7 @@
       </c>
       <c r="D40" s="21" t="inlineStr">
         <is>
-          <t>1111577.3079616884</t>
+          <t>1128415.624878298</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
@@ -45227,7 +45227,7 @@
       </c>
       <c r="D41" s="21" t="inlineStr">
         <is>
-          <t>4622.641831005549</t>
+          <t>5324.32009465599</t>
         </is>
       </c>
       <c r="E41" s="21" t="inlineStr">
@@ -45304,7 +45304,7 @@
       </c>
       <c r="D42" s="21" t="inlineStr">
         <is>
-          <t>75486.60520011785</t>
+          <t>76153.89091893201</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr">
@@ -45458,7 +45458,7 @@
       </c>
       <c r="D44" s="21" t="inlineStr">
         <is>
-          <t>35413.81396846072</t>
+          <t>39649.75361316411</t>
         </is>
       </c>
       <c r="E44" s="21" t="inlineStr">
@@ -45535,7 +45535,7 @@
       </c>
       <c r="D45" s="21" t="inlineStr">
         <is>
-          <t>35403.7115717776</t>
+          <t>20140.224142408744</t>
         </is>
       </c>
       <c r="E45" s="21" t="inlineStr">
@@ -45612,7 +45612,7 @@
       </c>
       <c r="D46" s="21" t="inlineStr">
         <is>
-          <t>129122.7281835694</t>
+          <t>298990.5146440843</t>
         </is>
       </c>
       <c r="E46" s="21" t="inlineStr">
@@ -45689,7 +45689,7 @@
       </c>
       <c r="D47" s="21" t="inlineStr">
         <is>
-          <t>118630.84165200125</t>
+          <t>323990.5146440843</t>
         </is>
       </c>
       <c r="E47" s="21" t="inlineStr">
@@ -45766,7 +45766,7 @@
       </c>
       <c r="D48" s="21" t="inlineStr">
         <is>
-          <t>4014.4774024044073</t>
+          <t>24999.999999999996</t>
         </is>
       </c>
       <c r="E48" s="21" t="inlineStr">
@@ -45843,7 +45843,7 @@
       </c>
       <c r="D49" s="21" t="inlineStr">
         <is>
-          <t>35403.7115717776</t>
+          <t>20140.224142408744</t>
         </is>
       </c>
       <c r="E49" s="21" t="inlineStr">
@@ -45997,7 +45997,7 @@
       </c>
       <c r="D51" s="21" t="inlineStr">
         <is>
-          <t>196743.41093589287</t>
+          <t>220276.40896202278</t>
         </is>
       </c>
       <c r="E51" s="21" t="inlineStr">
@@ -46074,12 +46074,12 @@
       </c>
       <c r="D52" s="21" t="inlineStr">
         <is>
-          <t>165471.11047208743</t>
+          <t>180089.48366015987</t>
         </is>
       </c>
       <c r="E52" s="21" t="inlineStr">
         <is>
-          <t>13761.716885365895</t>
+          <t>28380.090073438332</t>
         </is>
       </c>
       <c r="F52" s="21" t="inlineStr">
@@ -48100,7 +48100,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>2026-07-03T20:06:50+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -48134,7 +48134,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>27324f9094fb4ed78ad275fbe664d0ffce4c2df5</t>
+          <t>dd4f044670c5062e420f95ef114df3f9b594e621</t>
         </is>
       </c>
     </row>
@@ -48146,7 +48146,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-07-03T20:06:50+00:00</t>
+          <t>2026-07-02T08:48:06+00:00</t>
         </is>
       </c>
     </row>
@@ -48214,7 +48214,7 @@
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>0.11321363695747841</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -48294,7 +48294,7 @@
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>165471.11047208743</t>
+          <t>180089.48366015987</t>
         </is>
       </c>
     </row>
@@ -48386,7 +48386,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03T20:06:50+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49382,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CNavigation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-03T20:06:50+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -49432,7 +49432,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03T20:06:50+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49905,7 +49905,7 @@
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Opening Balance</t>
+          <t>Senior Debt / Debt Service</t>
         </is>
       </c>
       <c r="B31" s="41" t="inlineStr">
@@ -49915,19 +49915,19 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
+          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
-          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
+          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Closing Balance</t>
+          <t>Senior Debt / Opening Balance</t>
         </is>
       </c>
       <c r="B32" s="41" t="inlineStr">
@@ -49937,12 +49937,12 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
+          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
-          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
+          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
         </is>
       </c>
     </row>
@@ -49990,7 +49990,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Dashboard&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-03T20:06:50+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -50039,7 +50039,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-03T20:06:50+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -50129,7 +50129,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.11321363695747841</t>
+          <t>0.11587734289563015</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -50399,7 +50399,7 @@
     <row r="22">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Opening Balance</t>
+          <t>Senior Debt / Debt Service</t>
         </is>
       </c>
       <c r="B22" s="41" t="inlineStr">
@@ -50409,12 +50409,12 @@
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
+          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
         <is>
-          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
+          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -50426,7 +50426,7 @@
     <row r="23">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Closing Balance</t>
+          <t>Senior Debt / Opening Balance</t>
         </is>
       </c>
       <c r="B23" s="41" t="inlineStr">
@@ -50436,12 +50436,12 @@
       </c>
       <c r="C23" s="21" t="inlineStr">
         <is>
-          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
+          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
         </is>
       </c>
       <c r="D23" s="21" t="inlineStr">
         <is>
-          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
+          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -50453,7 +50453,7 @@
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>SHL / Principal Repaid</t>
+          <t>Senior Debt / Closing Balance</t>
         </is>
       </c>
       <c r="B24" s="41" t="inlineStr">
@@ -50463,12 +50463,12 @@
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
+          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
+          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -50485,7 +50485,7 @@
     <row r="25">
       <c r="A25" s="21" t="inlineStr">
         <is>
-          <t>SHL / Gross Accrued Interest</t>
+          <t>SHL / Principal Repaid</t>
         </is>
       </c>
       <c r="B25" s="41" t="inlineStr">
@@ -50495,12 +50495,12 @@
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
+          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
         <is>
-          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
+          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
         </is>
       </c>
       <c r="F25" s="22" t="inlineStr">
@@ -50512,7 +50512,7 @@
     <row r="26">
       <c r="A26" s="21" t="inlineStr">
         <is>
-          <t>OPEX / Total OPEX</t>
+          <t>SHL / Gross Accrued Interest</t>
         </is>
       </c>
       <c r="B26" s="41" t="inlineStr">
@@ -50522,12 +50522,12 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
+          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
         <is>
-          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
+          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -50544,7 +50544,7 @@
     <row r="27">
       <c r="A27" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Interest</t>
+          <t>OPEX / Total OPEX</t>
         </is>
       </c>
       <c r="B27" s="41" t="inlineStr">
@@ -50554,12 +50554,12 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
+          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
         <is>
-          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
+          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -50576,7 +50576,7 @@
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Debt Service</t>
+          <t>Senior Debt / Interest</t>
         </is>
       </c>
       <c r="B28" s="41" t="inlineStr">
@@ -50586,12 +50586,12 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
+          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
         </is>
       </c>
       <c r="D28" s="21" t="inlineStr">
         <is>
-          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
+          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -50638,7 +50638,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-03T20:06:50+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
chore: update governance report artifacts from main merge
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8W8EHSADMzvD3ufdXTkMr
</commit_message>
<xml_diff>
--- a/reports/phase10_calibration_reconciliation_pack.xlsx
+++ b/reports/phase10_calibration_reconciliation_pack.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-05T16:17:08+00:00</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-05T16:17:08+00:00</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-05T16:17:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t>0.11587734289563015</t>
+          <t>0.11321363695747841</t>
         </is>
       </c>
       <c r="C8" s="21" t="inlineStr">
@@ -1966,7 +1966,7 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>180089.48366015987</t>
+          <t>165471.11047208743</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>76153.89091893201</t>
+          <t>75486.60520011785</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
@@ -2087,7 +2087,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CRuntime Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Cruntime-derived values inside a review pack&amp;R2026-07-05T16:17:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5911,7 +5911,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-05T16:17:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6436,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCO2 &amp; Balancing Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-05T16:17:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -11857,88 +11857,88 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>2116.361416666667</v>
+        <v>1989.106693769401</v>
       </c>
       <c r="D19" s="51" t="n">
-        <v>2144.69175</v>
+        <v>2022.075313003147</v>
       </c>
       <c r="E19" s="51" t="n">
-        <v>2144.914083333334</v>
+        <v>2011.897283088215</v>
       </c>
       <c r="F19" s="51" t="n">
-        <v>2169.311</v>
+        <v>2045.243646896307</v>
       </c>
       <c r="G19" s="51" t="n">
-        <v>2194.979083333334</v>
+        <v>2041.09207119988</v>
       </c>
       <c r="H19" s="51" t="n">
-        <v>2189.918</v>
+        <v>2063.521654399878</v>
       </c>
       <c r="I19" s="51" t="n">
-        <v>2243.1435</v>
+        <v>2059.740388389284</v>
       </c>
       <c r="J19" s="51" t="n">
-        <v>2287.658</v>
+        <v>2093.87973184325</v>
       </c>
       <c r="K19" s="51" t="n">
-        <v>2342.122833333333</v>
+        <v>2079.711488155402</v>
       </c>
       <c r="L19" s="51" t="n">
-        <v>2395.111416666667</v>
+        <v>2114.181844312673</v>
       </c>
       <c r="M19" s="51" t="n">
-        <v>2435.872083333333</v>
+        <v>2119.985981148247</v>
       </c>
       <c r="N19" s="51" t="n">
-        <v>2484.465916666667</v>
+        <v>2155.123870338549</v>
       </c>
       <c r="O19" s="51" t="n">
-        <v>2875.376522231662</v>
+        <v>2164.704254947222</v>
       </c>
       <c r="P19" s="51" t="n">
-        <v>2829.374203596205</v>
+        <v>2188.492213792796</v>
       </c>
       <c r="Q19" s="51" t="n">
-        <v>0</v>
+        <v>2200.570150808295</v>
       </c>
       <c r="R19" s="51" t="n">
-        <v>0</v>
+        <v>2237.043689219482</v>
       </c>
       <c r="S19" s="51" t="n">
-        <v>0</v>
+        <v>2245.580238898558</v>
       </c>
       <c r="T19" s="51" t="n">
-        <v>0</v>
+        <v>2282.799800869252</v>
       </c>
       <c r="U19" s="51" t="n">
-        <v>0</v>
+        <v>2289.065099472558</v>
       </c>
       <c r="V19" s="51" t="n">
-        <v>0</v>
+        <v>2327.005404988678</v>
       </c>
       <c r="W19" s="51" t="n">
-        <v>0</v>
+        <v>2337.507689488432</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>0</v>
+        <v>2363.194587175117</v>
       </c>
       <c r="Y19" s="51" t="n">
-        <v>0</v>
+        <v>2376.174912802545</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>0</v>
+        <v>2415.559027379383</v>
       </c>
       <c r="AA19" s="51" t="n">
-        <v>0</v>
+        <v>3379.663922072882</v>
       </c>
       <c r="AB19" s="51" t="n">
-        <v>0</v>
+        <v>3435.680451168012</v>
       </c>
       <c r="AC19" s="51" t="n">
-        <v>0</v>
+        <v>3365.998420752923</v>
       </c>
       <c r="AD19" s="51" t="n">
-        <v>0</v>
+        <v>3421.788449826067</v>
       </c>
       <c r="AE19" s="51" t="n">
         <v>0</v>
@@ -12040,7 +12040,7 @@
         <v>0</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>32853.2998091612</v>
+        <v>65826.38828020645</v>
       </c>
       <c r="BM19" s="67" t="inlineStr">
         <is>
@@ -12069,88 +12069,88 @@
       </c>
       <c r="B20" s="50" t="inlineStr"/>
       <c r="C20" s="51" t="n">
-        <v>2.257460346299922e-05</v>
+        <v>-127.2547003226625</v>
       </c>
       <c r="D20" s="51" t="n">
-        <v>-6.747457253809444</v>
+        <v>-129.3638942506627</v>
       </c>
       <c r="E20" s="51" t="n">
-        <v>0.2223582974293095</v>
+        <v>-132.7944419476889</v>
       </c>
       <c r="F20" s="51" t="n">
-        <v>-10.92810169395852</v>
+        <v>-134.9954547976515</v>
       </c>
       <c r="G20" s="51" t="n">
-        <v>50.06501789420463</v>
+        <v>-103.8219942392489</v>
       </c>
       <c r="H20" s="51" t="n">
-        <v>21.43345032527623</v>
+        <v>-104.9628952748462</v>
       </c>
       <c r="I20" s="51" t="n">
-        <v>73.83252306620261</v>
+        <v>-109.5705885445132</v>
       </c>
       <c r="J20" s="51" t="n">
-        <v>82.39159250928833</v>
+        <v>-111.3866756474617</v>
       </c>
       <c r="K20" s="51" t="n">
-        <v>147.1437090325076</v>
+        <v>-115.2676361454241</v>
       </c>
       <c r="L20" s="51" t="n">
-        <v>163.7514229022922</v>
+        <v>-117.1781494517013</v>
       </c>
       <c r="M20" s="51" t="n">
-        <v>245.9541162268556</v>
+        <v>-69.9319859582306</v>
       </c>
       <c r="N20" s="51" t="n">
-        <v>258.2509666799729</v>
+        <v>-71.09107964814484</v>
       </c>
       <c r="O20" s="51" t="n">
-        <v>632.2329906401042</v>
+        <v>-78.43927664433613</v>
       </c>
       <c r="P20" s="51" t="n">
-        <v>561.5807430860605</v>
+        <v>-79.30124671734939</v>
       </c>
       <c r="Q20" s="51" t="n">
-        <v>-2287.658040589451</v>
+        <v>-87.08788978115626</v>
       </c>
       <c r="R20" s="51" t="n">
-        <v>-2325.575024687618</v>
+        <v>-88.53133546813615</v>
       </c>
       <c r="S20" s="51" t="n">
-        <v>-2342.122838844162</v>
+        <v>-96.54259994560471</v>
       </c>
       <c r="T20" s="51" t="n">
-        <v>-2380.942554405116</v>
+        <v>-98.1427535358639</v>
       </c>
       <c r="U20" s="51" t="n">
-        <v>-2395.111402698671</v>
+        <v>-106.0463032261123</v>
       </c>
       <c r="V20" s="51" t="n">
-        <v>-2434.809381748925</v>
+        <v>-107.8039767602477</v>
       </c>
       <c r="W20" s="51" t="n">
-        <v>-2435.872062636206</v>
+        <v>-98.36437314777368</v>
       </c>
       <c r="X20" s="51" t="n">
-        <v>-2462.63988750034</v>
+        <v>-99.44530032522243</v>
       </c>
       <c r="Y20" s="51" t="n">
-        <v>-2484.465931235276</v>
+        <v>-108.2910184327302</v>
       </c>
       <c r="Z20" s="51" t="n">
-        <v>-2525.644924570668</v>
+        <v>-110.0858971912849</v>
       </c>
       <c r="AA20" s="51" t="n">
-        <v>-2875.303013382943</v>
+        <v>504.3609086899392</v>
       </c>
       <c r="AB20" s="51" t="n">
-        <v>-2922.959969405866</v>
+        <v>512.7204817621459</v>
       </c>
       <c r="AC20" s="51" t="n">
-        <v>-2829.332458574896</v>
+        <v>536.6659621780268</v>
       </c>
       <c r="AD20" s="51" t="n">
-        <v>-2844.793291681864</v>
+        <v>576.9951581442028</v>
       </c>
       <c r="AE20" s="51" t="n">
         <v>0</v>
@@ -12252,7 +12252,7 @@
         <v>0</v>
       </c>
       <c r="BL20" s="68" t="n">
-        <v>-33328.04742767497</v>
+        <v>-354.9589566297218</v>
       </c>
       <c r="BM20" s="67" t="inlineStr">
         <is>
@@ -13194,20 +13194,48 @@
       <c r="P27" s="75" t="n">
         <v>1.19388468780374</v>
       </c>
-      <c r="Q27" s="70" t="n"/>
-      <c r="R27" s="70" t="n"/>
-      <c r="S27" s="70" t="n"/>
-      <c r="T27" s="70" t="n"/>
-      <c r="U27" s="70" t="n"/>
-      <c r="V27" s="70" t="n"/>
-      <c r="W27" s="70" t="n"/>
-      <c r="X27" s="70" t="n"/>
-      <c r="Y27" s="70" t="n"/>
-      <c r="Z27" s="70" t="n"/>
-      <c r="AA27" s="70" t="n"/>
-      <c r="AB27" s="70" t="n"/>
-      <c r="AC27" s="70" t="n"/>
-      <c r="AD27" s="70" t="n"/>
+      <c r="Q27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="R27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="S27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="T27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="U27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="V27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="W27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="X27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="Y27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="Z27" s="75" t="n">
+        <v>1.543504023661211</v>
+      </c>
+      <c r="AA27" s="75" t="n">
+        <v>1.816832861184551</v>
+      </c>
+      <c r="AB27" s="75" t="n">
+        <v>1.816832861184551</v>
+      </c>
+      <c r="AC27" s="75" t="n">
+        <v>1.816832861184551</v>
+      </c>
+      <c r="AD27" s="75" t="n">
+        <v>1.816832861184609</v>
+      </c>
       <c r="AE27" s="70" t="n"/>
       <c r="AF27" s="70" t="n"/>
       <c r="AG27" s="70" t="n"/>
@@ -13310,75 +13338,47 @@
       <c r="P28" s="75" t="n">
         <v>-0.006115312196260048</v>
       </c>
-      <c r="Q28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="R28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="T28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="U28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="V28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="W28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="X28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Y28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="Z28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AA28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AB28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AC28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="AD28" s="59" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="Q28" s="75" t="n">
+        <v>0.3435040236612112</v>
+      </c>
+      <c r="R28" s="75" t="n">
+        <v>0.343504023661211</v>
+      </c>
+      <c r="S28" s="75" t="n">
+        <v>0.3435040236612112</v>
+      </c>
+      <c r="T28" s="75" t="n">
+        <v>0.3435040236612112</v>
+      </c>
+      <c r="U28" s="75" t="n">
+        <v>0.3435040236612115</v>
+      </c>
+      <c r="V28" s="75" t="n">
+        <v>0.3435040236612115</v>
+      </c>
+      <c r="W28" s="75" t="n">
+        <v>0.3435040236612112</v>
+      </c>
+      <c r="X28" s="75" t="n">
+        <v>0.3435040236612115</v>
+      </c>
+      <c r="Y28" s="75" t="n">
+        <v>0.3435040236612112</v>
+      </c>
+      <c r="Z28" s="75" t="n">
+        <v>0.3435040236612112</v>
+      </c>
+      <c r="AA28" s="75" t="n">
+        <v>0.4043967420309842</v>
+      </c>
+      <c r="AB28" s="75" t="n">
+        <v>0.4043967420309844</v>
+      </c>
+      <c r="AC28" s="75" t="n">
+        <v>0.4042120165976311</v>
+      </c>
+      <c r="AD28" s="75" t="n">
+        <v>0.404212016597689</v>
       </c>
       <c r="AE28" s="59" t="inlineStr">
         <is>
@@ -14232,43 +14232,43 @@
         <v>36807.77046925188</v>
       </c>
       <c r="Y7" s="51" t="n">
-        <v>37287.10873481189</v>
+        <v>36990.76781846865</v>
       </c>
       <c r="Z7" s="51" t="n">
-        <v>37461.93045892712</v>
+        <v>37153.93619991388</v>
       </c>
       <c r="AA7" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AB7" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AC7" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AD7" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AE7" s="51" t="n">
-        <v>34219.39256116209</v>
+        <v>32601.66748205897</v>
       </c>
       <c r="AF7" s="51" t="n">
-        <v>29380.93173303165</v>
+        <v>27699.41436164256</v>
       </c>
       <c r="AG7" s="51" t="n">
-        <v>25209.22609491149</v>
+        <v>22832.10451072115</v>
       </c>
       <c r="AH7" s="51" t="n">
-        <v>19978.76699288986</v>
+        <v>17508.16721901635</v>
       </c>
       <c r="AI7" s="51" t="n">
-        <v>15377.18958936602</v>
+        <v>13429.81973793022</v>
       </c>
       <c r="AJ7" s="51" t="n">
-        <v>9562.397895654238</v>
+        <v>7538.449458770179</v>
       </c>
       <c r="AK7" s="51" t="n">
-        <v>4379.618798924304</v>
+        <v>3070.632209149414</v>
       </c>
       <c r="AL7" s="51" t="n">
         <v>0</v>
@@ -14349,7 +14349,7 @@
         <v>0</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>1128415.624878298</v>
+        <v>1111577.307961688</v>
       </c>
       <c r="BM7" s="58" t="inlineStr">
         <is>
@@ -15004,43 +15004,43 @@
         <v>1467.403116040841</v>
       </c>
       <c r="Y11" s="51" t="n">
-        <v>1466.282350146234</v>
+        <v>1454.629007476236</v>
       </c>
       <c r="Z11" s="51" t="n">
-        <v>1497.574026609034</v>
+        <v>1485.261681863516</v>
       </c>
       <c r="AA11" s="51" t="n">
-        <v>1495.417636415413</v>
+        <v>1467.824763479375</v>
       </c>
       <c r="AB11" s="51" t="n">
-        <v>1520.203564090807</v>
+        <v>1492.153350719365</v>
       </c>
       <c r="AC11" s="51" t="n">
-        <v>1495.417636415413</v>
+        <v>1467.824763479375</v>
       </c>
       <c r="AD11" s="51" t="n">
-        <v>1520.203564090807</v>
+        <v>1492.153350719365</v>
       </c>
       <c r="AE11" s="51" t="n">
-        <v>1349.384713328492</v>
+        <v>1285.592421042525</v>
       </c>
       <c r="AF11" s="51" t="n">
-        <v>1171.319811756862</v>
+        <v>1104.283319217483</v>
       </c>
       <c r="AG11" s="51" t="n">
-        <v>991.3303696112138</v>
+        <v>897.8521799280383</v>
       </c>
       <c r="AH11" s="51" t="n">
-        <v>798.6689998538479</v>
+        <v>699.9045740441409</v>
       </c>
       <c r="AI11" s="51" t="n">
-        <v>604.6942885836913</v>
+        <v>528.1157031354352</v>
       </c>
       <c r="AJ11" s="51" t="n">
-        <v>382.2653703426579</v>
+        <v>301.3562294323492</v>
       </c>
       <c r="AK11" s="51" t="n">
-        <v>172.2246096071239</v>
+        <v>120.7498775002309</v>
       </c>
       <c r="AL11" s="51" t="n">
         <v>0</v>
@@ -15121,7 +15121,7 @@
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>44736.24440845805</v>
+        <v>44068.95868964389</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -15216,43 +15216,43 @@
         <v>346.4431160408415</v>
       </c>
       <c r="Y12" s="51" t="n">
-        <v>332.8523501462341</v>
+        <v>321.1990074762359</v>
       </c>
       <c r="Z12" s="51" t="n">
-        <v>355.7840266090338</v>
+        <v>343.4716818635161</v>
       </c>
       <c r="AA12" s="51" t="n">
-        <v>331.427636415413</v>
+        <v>303.8347634793749</v>
       </c>
       <c r="AB12" s="51" t="n">
-        <v>-214.3164359091934</v>
+        <v>-242.3666492806353</v>
       </c>
       <c r="AC12" s="51" t="n">
-        <v>-207.4223635845869</v>
+        <v>-235.015236520625</v>
       </c>
       <c r="AD12" s="51" t="n">
-        <v>-96.75643590919344</v>
+        <v>-124.8066492806354</v>
       </c>
       <c r="AE12" s="51" t="n">
-        <v>-228.1052866715081</v>
+        <v>-291.8975789574747</v>
       </c>
       <c r="AF12" s="51" t="n">
-        <v>-355.5501882431381</v>
+        <v>-422.5866807825169</v>
       </c>
       <c r="AG12" s="51" t="n">
-        <v>-364.4196303887862</v>
+        <v>-457.8978200719617</v>
       </c>
       <c r="AH12" s="51" t="n">
-        <v>-383.201000146152</v>
+        <v>-481.965425955859</v>
       </c>
       <c r="AI12" s="51" t="n">
-        <v>-394.1657114163087</v>
+        <v>-470.7442968645648</v>
       </c>
       <c r="AJ12" s="51" t="n">
-        <v>-437.6646296573421</v>
+        <v>-518.5737705676509</v>
       </c>
       <c r="AK12" s="51" t="n">
-        <v>-435.6753903928761</v>
+        <v>-487.1501224997691</v>
       </c>
       <c r="AL12" s="51" t="n">
         <v>-419.74</v>
@@ -15333,7 +15333,7 @@
         <v>0</v>
       </c>
       <c r="BL12" s="68" t="n">
-        <v>5980.864408458045</v>
+        <v>5313.578689643888</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -15769,46 +15769,46 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X15" s="51" t="n">
-        <v>988.064850480836</v>
+        <v>1284.405766824072</v>
       </c>
       <c r="Y15" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z15" s="51" t="n">
-        <v>931.4943908801665</v>
+        <v>1312.866050771856</v>
       </c>
       <c r="AA15" s="51" t="n">
-        <v>1495.417636415413</v>
+        <v>1467.824763479375</v>
       </c>
       <c r="AB15" s="51" t="n">
-        <v>1520.203564090807</v>
+        <v>1492.153350719365</v>
       </c>
       <c r="AC15" s="51" t="n">
-        <v>1495.417636415413</v>
+        <v>1467.824763479375</v>
       </c>
       <c r="AD15" s="51" t="n">
-        <v>1520.203564090807</v>
+        <v>1492.153350719365</v>
       </c>
       <c r="AE15" s="51" t="n">
-        <v>1349.384713328492</v>
+        <v>1285.592421042525</v>
       </c>
       <c r="AF15" s="51" t="n">
-        <v>1171.319811756862</v>
+        <v>1104.283319217483</v>
       </c>
       <c r="AG15" s="51" t="n">
-        <v>991.3303696112138</v>
+        <v>897.8521799280383</v>
       </c>
       <c r="AH15" s="51" t="n">
-        <v>798.6689998538479</v>
+        <v>699.9045740441409</v>
       </c>
       <c r="AI15" s="51" t="n">
-        <v>604.6942885836913</v>
+        <v>528.1157031354352</v>
       </c>
       <c r="AJ15" s="51" t="n">
-        <v>382.2653703426579</v>
+        <v>301.3562294323492</v>
       </c>
       <c r="AK15" s="51" t="n">
-        <v>172.2246096071239</v>
+        <v>120.7498775002309</v>
       </c>
       <c r="AL15" s="51" t="n">
         <v>0</v>
@@ -15889,7 +15889,7 @@
         <v>0</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>38125.88082427603</v>
+        <v>38160.27336911231</v>
       </c>
       <c r="BM15" s="58" t="inlineStr">
         <is>
@@ -16661,13 +16661,13 @@
         <v>174.1412765880596</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>479.3382655600055</v>
+        <v>182.9973492167699</v>
       </c>
       <c r="Y19" s="51" t="n">
-        <v>174.8217241152231</v>
+        <v>163.1683814452249</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>566.0796357288673</v>
+        <v>172.3956310916597</v>
       </c>
       <c r="AA19" s="51" t="n">
         <v>0</v>
@@ -16781,7 +16781,7 @@
         <v>0</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>5324.32009465599</v>
+        <v>4622.641831005549</v>
       </c>
       <c r="BM19" s="58" t="inlineStr">
         <is>
@@ -17451,28 +17451,28 @@
         <v>0</v>
       </c>
       <c r="AD23" s="51" t="n">
-        <v>3808.617533493891</v>
+        <v>4724.664348946576</v>
       </c>
       <c r="AE23" s="51" t="n">
-        <v>4838.460828130443</v>
+        <v>4902.253120416409</v>
       </c>
       <c r="AF23" s="51" t="n">
-        <v>4171.705638120166</v>
+        <v>4867.309850921405</v>
       </c>
       <c r="AG23" s="51" t="n">
-        <v>5230.459102021628</v>
+        <v>5323.937291704803</v>
       </c>
       <c r="AH23" s="51" t="n">
-        <v>4601.577403523834</v>
+        <v>4078.347481086129</v>
       </c>
       <c r="AI23" s="51" t="n">
-        <v>5814.791693711786</v>
+        <v>5891.370279160043</v>
       </c>
       <c r="AJ23" s="51" t="n">
-        <v>5182.779096729934</v>
+        <v>4467.817249620765</v>
       </c>
       <c r="AK23" s="51" t="n">
-        <v>4379.618798924304</v>
+        <v>3070.632209149414</v>
       </c>
       <c r="AL23" s="51" t="n">
         <v>0</v>
@@ -17553,7 +17553,7 @@
         <v>0</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="BM23" s="67" t="inlineStr">
         <is>
@@ -17663,28 +17663,28 @@
         <v>-1465.03</v>
       </c>
       <c r="AD24" s="51" t="n">
-        <v>2165.327533493891</v>
+        <v>3081.374348946576</v>
       </c>
       <c r="AE24" s="51" t="n">
-        <v>3999.360828130443</v>
+        <v>4063.153120416409</v>
       </c>
       <c r="AF24" s="51" t="n">
-        <v>-487.3743618798344</v>
+        <v>208.2298509214052</v>
       </c>
       <c r="AG24" s="51" t="n">
-        <v>1404.679102021627</v>
+        <v>1498.157291704803</v>
       </c>
       <c r="AH24" s="51" t="n">
-        <v>-422.1925964761667</v>
+        <v>-945.4225189138715</v>
       </c>
       <c r="AI24" s="51" t="n">
-        <v>1715.081693711786</v>
+        <v>1791.660279160043</v>
       </c>
       <c r="AJ24" s="51" t="n">
-        <v>-411.7609032700657</v>
+        <v>-1126.722750379235</v>
       </c>
       <c r="AK24" s="51" t="n">
-        <v>-113.7112010756964</v>
+        <v>-1422.697790850586</v>
       </c>
       <c r="AL24" s="51" t="n">
         <v>-6154.98</v>
@@ -17765,7 +17765,7 @@
         <v>0</v>
       </c>
       <c r="BL24" s="68" t="n">
-        <v>23432.48009465598</v>
+        <v>22730.80183100554</v>
       </c>
       <c r="BM24" s="67" t="inlineStr">
         <is>
@@ -17957,43 +17957,43 @@
         <v>36807.77046925188</v>
       </c>
       <c r="X27" s="51" t="n">
-        <v>37287.10873481189</v>
+        <v>36990.76781846865</v>
       </c>
       <c r="Y27" s="51" t="n">
-        <v>37461.93045892711</v>
+        <v>37153.93619991388</v>
       </c>
       <c r="Z27" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AA27" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AB27" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AC27" s="51" t="n">
-        <v>38028.01009465598</v>
+        <v>37326.33183100554</v>
       </c>
       <c r="AD27" s="51" t="n">
-        <v>34219.39256116209</v>
+        <v>32601.66748205897</v>
       </c>
       <c r="AE27" s="51" t="n">
-        <v>29380.93173303165</v>
+        <v>27699.41436164256</v>
       </c>
       <c r="AF27" s="51" t="n">
-        <v>25209.22609491149</v>
+        <v>22832.10451072115</v>
       </c>
       <c r="AG27" s="51" t="n">
-        <v>19978.76699288986</v>
+        <v>17508.16721901635</v>
       </c>
       <c r="AH27" s="51" t="n">
-        <v>15377.18958936602</v>
+        <v>13429.81973793022</v>
       </c>
       <c r="AI27" s="51" t="n">
-        <v>9562.397895654238</v>
+        <v>7538.449458770179</v>
       </c>
       <c r="AJ27" s="51" t="n">
-        <v>4379.618798924304</v>
+        <v>3070.632209149414</v>
       </c>
       <c r="AK27" s="51" t="n">
         <v>0</v>
@@ -18077,7 +18077,7 @@
         <v>0</v>
       </c>
       <c r="BL27" s="52" t="n">
-        <v>1095711.934878298</v>
+        <v>1078873.617961689</v>
       </c>
       <c r="BM27" s="58" t="inlineStr">
         <is>
@@ -18849,46 +18849,46 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X31" s="51" t="n">
-        <v>988.064850480836</v>
+        <v>1284.405766824072</v>
       </c>
       <c r="Y31" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z31" s="51" t="n">
-        <v>931.4943908801665</v>
+        <v>1312.866050771856</v>
       </c>
       <c r="AA31" s="51" t="n">
-        <v>1495.417636415413</v>
+        <v>1467.824763479375</v>
       </c>
       <c r="AB31" s="51" t="n">
-        <v>1520.203564090807</v>
+        <v>1492.153350719365</v>
       </c>
       <c r="AC31" s="51" t="n">
-        <v>1495.417636415413</v>
+        <v>1467.824763479375</v>
       </c>
       <c r="AD31" s="51" t="n">
-        <v>5328.821097584698</v>
+        <v>6216.81769966594</v>
       </c>
       <c r="AE31" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF31" s="51" t="n">
-        <v>5343.025449877027</v>
+        <v>5971.593170138888</v>
       </c>
       <c r="AG31" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH31" s="51" t="n">
-        <v>5400.246403377681</v>
+        <v>4778.25205513027</v>
       </c>
       <c r="AI31" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ31" s="51" t="n">
-        <v>5565.044467072592</v>
+        <v>4769.173479053115</v>
       </c>
       <c r="AK31" s="51" t="n">
-        <v>4551.843408531427</v>
+        <v>3191.382086649645</v>
       </c>
       <c r="AL31" s="51" t="n">
         <v>0</v>
@@ -18969,7 +18969,7 @@
         <v>0</v>
       </c>
       <c r="BL31" s="52" t="n">
-        <v>76153.89091893201</v>
+        <v>75486.60520011785</v>
       </c>
       <c r="BM31" s="58" t="inlineStr">
         <is>
@@ -21951,190 +21951,190 @@
         </is>
       </c>
       <c r="C15" s="51" t="n">
-        <v>655.1143745939253</v>
+        <v>-1241.067170204809</v>
       </c>
       <c r="D15" s="51" t="n">
-        <v>707.9819198386576</v>
+        <v>-1204.192477325214</v>
       </c>
       <c r="E15" s="51" t="n">
-        <v>734.549128681577</v>
+        <v>-1189.669173019131</v>
       </c>
       <c r="F15" s="51" t="n">
-        <v>789.9273535381026</v>
+        <v>-1151.349119055657</v>
       </c>
       <c r="G15" s="51" t="n">
-        <v>824.5447644261715</v>
+        <v>-1133.164490334039</v>
       </c>
       <c r="H15" s="51" t="n">
-        <v>871.7885150300467</v>
+        <v>-1103.578310539416</v>
       </c>
       <c r="I15" s="51" t="n">
-        <v>908.9520914556761</v>
+        <v>-1075.926475710916</v>
       </c>
       <c r="J15" s="51" t="n">
-        <v>969.8207848092713</v>
+        <v>-1497.139574763567</v>
       </c>
       <c r="K15" s="51" t="n">
-        <v>996.6349527778393</v>
+        <v>-1480.958116717468</v>
       </c>
       <c r="L15" s="51" t="n">
-        <v>1060.223384607837</v>
+        <v>-1462.924179361077</v>
       </c>
       <c r="M15" s="51" t="n">
-        <v>1120.146841475899</v>
+        <v>-1424.224592281713</v>
       </c>
       <c r="N15" s="51" t="n">
-        <v>1187.687261244841</v>
+        <v>-1405.270664705625</v>
       </c>
       <c r="O15" s="51" t="n">
-        <v>1253.218645585758</v>
+        <v>-1353.63197037875</v>
       </c>
       <c r="P15" s="51" t="n">
-        <v>1312.951896619405</v>
+        <v>-1340.524484649894</v>
       </c>
       <c r="Q15" s="51" t="n">
-        <v>1385.324906394822</v>
+        <v>-1264.703232520845</v>
       </c>
       <c r="R15" s="51" t="n">
-        <v>1461.291588138776</v>
+        <v>-1241.607016072596</v>
       </c>
       <c r="S15" s="51" t="n">
-        <v>1535.04343874859</v>
+        <v>-1168.986926380646</v>
       </c>
       <c r="T15" s="51" t="n">
-        <v>1615.762702699066</v>
+        <v>-1143.263265837704</v>
       </c>
       <c r="U15" s="51" t="n">
-        <v>1689.734939543118</v>
+        <v>-1071.381524281971</v>
       </c>
       <c r="V15" s="51" t="n">
-        <v>1775.334571548982</v>
+        <v>-1043.095018171053</v>
       </c>
       <c r="W15" s="51" t="n">
-        <v>1856.497995964273</v>
+        <v>-983.3655054161823</v>
       </c>
       <c r="X15" s="51" t="n">
-        <v>1933.806366406446</v>
+        <v>-960.9738351259814</v>
       </c>
       <c r="Y15" s="51" t="n">
-        <v>2022.69192865896</v>
+        <v>-868.4265871844455</v>
       </c>
       <c r="Z15" s="51" t="n">
-        <v>2118.731443842721</v>
+        <v>-835.2402239338267</v>
       </c>
       <c r="AA15" s="51" t="n">
-        <v>4607.278452375285</v>
+        <v>2273.648779637848</v>
       </c>
       <c r="AB15" s="51" t="n">
-        <v>4776.369613776</v>
+        <v>2493.797085101402</v>
       </c>
       <c r="AC15" s="51" t="n">
-        <v>4759.925290806009</v>
+        <v>2543.8280213073</v>
       </c>
       <c r="AD15" s="51" t="n">
-        <v>4933.314456006903</v>
+        <v>2776.237978346574</v>
       </c>
       <c r="AE15" s="51" t="n">
-        <v>5016.091417597368</v>
+        <v>2892.668503073712</v>
       </c>
       <c r="AF15" s="51" t="n">
-        <v>5071.213301307228</v>
+        <v>3131.968093871822</v>
       </c>
       <c r="AG15" s="51" t="n">
-        <v>5053.280910902247</v>
+        <v>3271.52658396707</v>
       </c>
       <c r="AH15" s="51" t="n">
-        <v>5137.036948099522</v>
+        <v>3557.869024514927</v>
       </c>
       <c r="AI15" s="51" t="n">
-        <v>5250.977421564884</v>
+        <v>3831.037264493374</v>
       </c>
       <c r="AJ15" s="51" t="n">
-        <v>5338.01019650795</v>
+        <v>4149.71349057495</v>
       </c>
       <c r="AK15" s="51" t="n">
-        <v>5401.780310394376</v>
+        <v>4381.914784405477</v>
       </c>
       <c r="AL15" s="51" t="n">
-        <v>5491.312580732402</v>
+        <v>4732.456463680996</v>
       </c>
       <c r="AM15" s="51" t="n">
-        <v>5564.135766234725</v>
+        <v>4968.602390096292</v>
       </c>
       <c r="AN15" s="51" t="n">
-        <v>5625.280115314228</v>
+        <v>5042.623158119328</v>
       </c>
       <c r="AO15" s="51" t="n">
-        <v>5700.129335260623</v>
+        <v>5101.350395991216</v>
       </c>
       <c r="AP15" s="51" t="n">
-        <v>5794.606617060525</v>
+        <v>5215.195222996599</v>
       </c>
       <c r="AQ15" s="51" t="n">
-        <v>5850.091923793809</v>
+        <v>7018.600484524402</v>
       </c>
       <c r="AR15" s="51" t="n">
-        <v>5947.054773359453</v>
+        <v>7134.930879295526</v>
       </c>
       <c r="AS15" s="51" t="n">
-        <v>5999.679524373062</v>
+        <v>7168.188085103656</v>
       </c>
       <c r="AT15" s="51" t="n">
-        <v>6099.121726434495</v>
+        <v>7286.997832370568</v>
       </c>
       <c r="AU15" s="51" t="n">
-        <v>6203.833170484581</v>
+        <v>7375.587294346148</v>
       </c>
       <c r="AV15" s="51" t="n">
-        <v>6272.007161369031</v>
+        <v>7456.637704174131</v>
       </c>
       <c r="AW15" s="51" t="n">
-        <v>6316.696230223002</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX15" s="51" t="n">
-        <v>6421.392852823384</v>
+        <v>7609.268958759457</v>
       </c>
       <c r="AY15" s="51" t="n">
-        <v>6447.930689543427</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ15" s="51" t="n">
-        <v>6554.802468928128</v>
+        <v>7742.678574864201</v>
       </c>
       <c r="BA15" s="51" t="n">
-        <v>6636.221108744508</v>
+        <v>7804.729669475102</v>
       </c>
       <c r="BB15" s="51" t="n">
-        <v>6746.213723806573</v>
+        <v>7934.089829742647</v>
       </c>
       <c r="BC15" s="51" t="n">
-        <v>6780.051659875585</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD15" s="51" t="n">
-        <v>6854.557722072019</v>
+        <v>8039.188264877119</v>
       </c>
       <c r="BE15" s="51" t="n">
-        <v>6848.555807320907</v>
+        <v>8017.0643680515</v>
       </c>
       <c r="BF15" s="51" t="n">
-        <v>6962.067782027882</v>
+        <v>8149.943887963956</v>
       </c>
       <c r="BG15" s="51" t="n">
-        <v>6925.218182124281</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH15" s="51" t="n">
-        <v>7040.000803927449</v>
+        <v>8227.876909863522</v>
       </c>
       <c r="BI15" s="51" t="n">
-        <v>6945.581281234856</v>
+        <v>8114.08984196545</v>
       </c>
       <c r="BJ15" s="51" t="n">
-        <v>7060.70141296803</v>
+        <v>8248.577518904103</v>
       </c>
       <c r="BK15" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>245276.4089620228</v>
+        <v>186251.5244043248</v>
       </c>
       <c r="BM15" s="67" t="inlineStr">
         <is>
@@ -22906,127 +22906,127 @@
         <v>0</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>296.3409163432357</v>
+        <v>0</v>
       </c>
       <c r="Y19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>381.3716598916898</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AB19" s="51" t="n">
-        <v>859.7465304796799</v>
+        <v>0</v>
       </c>
       <c r="AC19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AD19" s="51" t="n">
-        <v>887.9966020812425</v>
+        <v>138.810953157969</v>
       </c>
       <c r="AE19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AF19" s="51" t="n">
-        <v>912.818394235301</v>
+        <v>1084.434587450196</v>
       </c>
       <c r="AG19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AH19" s="51" t="n">
-        <v>924.666650657914</v>
+        <v>1229.291209526759</v>
       </c>
       <c r="AI19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AJ19" s="51" t="n">
-        <v>960.841835371431</v>
+        <v>1436.535135912298</v>
       </c>
       <c r="AK19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AL19" s="51" t="n">
-        <v>988.4362645318324</v>
+        <v>1640.586824655565</v>
       </c>
       <c r="AM19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AN19" s="51" t="n">
-        <v>1012.550420756561</v>
+        <v>1802.020598678811</v>
       </c>
       <c r="AO19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AP19" s="51" t="n">
-        <v>1043.029191070895</v>
+        <v>1856.978211417807</v>
       </c>
       <c r="AQ19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AR19" s="51" t="n">
-        <v>1070.469859204702</v>
+        <v>2547.635645487587</v>
       </c>
       <c r="AS19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AT19" s="51" t="n">
-        <v>1097.841910758209</v>
+        <v>2601.93346514536</v>
       </c>
       <c r="AU19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AV19" s="51" t="n">
-        <v>1128.961289046425</v>
+        <v>2669.80049973365</v>
       </c>
       <c r="AW19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AX19" s="51" t="n">
-        <v>1155.850713508209</v>
+        <v>2717.005274948349</v>
       </c>
       <c r="AY19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AZ19" s="51" t="n">
-        <v>1179.864444407063</v>
+        <v>2764.64120852488</v>
       </c>
       <c r="BA19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BB19" s="51" t="n">
-        <v>1214.318470285183</v>
+        <v>2832.987509859195</v>
       </c>
       <c r="BC19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BD19" s="51" t="n">
-        <v>1233.820389972963</v>
+        <v>2878.378928750569</v>
       </c>
       <c r="BE19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BF19" s="51" t="n">
-        <v>1253.172200765019</v>
+        <v>2910.061486082782</v>
       </c>
       <c r="BG19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BH19" s="51" t="n">
-        <v>1267.200144706941</v>
+        <v>2937.888657489311</v>
       </c>
       <c r="BI19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BJ19" s="51" t="n">
-        <v>1270.926254334245</v>
+        <v>2945.280124956519</v>
       </c>
       <c r="BK19" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>20140.22414240874</v>
+        <v>36994.27032177761</v>
       </c>
       <c r="BM19" s="58" t="inlineStr">
         <is>
@@ -23735,88 +23735,88 @@
         </is>
       </c>
       <c r="C23" s="51" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="D23" s="51" t="n">
-        <v>24344.88562540607</v>
+        <v>1241.067170204809</v>
       </c>
       <c r="E23" s="51" t="n">
-        <v>23636.90370556742</v>
+        <v>2445.259647530023</v>
       </c>
       <c r="F23" s="51" t="n">
-        <v>22902.35457688584</v>
+        <v>3634.928820549154</v>
       </c>
       <c r="G23" s="51" t="n">
-        <v>22112.42722334773</v>
+        <v>4786.27793960481</v>
       </c>
       <c r="H23" s="51" t="n">
-        <v>21287.88245892156</v>
+        <v>5919.442429938848</v>
       </c>
       <c r="I23" s="51" t="n">
-        <v>20416.09394389152</v>
+        <v>7023.020740478265</v>
       </c>
       <c r="J23" s="51" t="n">
-        <v>19507.14185243584</v>
+        <v>8098.947216189181</v>
       </c>
       <c r="K23" s="51" t="n">
-        <v>18537.32106762657</v>
+        <v>9596.086790952748</v>
       </c>
       <c r="L23" s="51" t="n">
-        <v>17540.68611484873</v>
+        <v>11077.04490767022</v>
       </c>
       <c r="M23" s="51" t="n">
-        <v>16480.46273024089</v>
+        <v>11298.90191682648</v>
       </c>
       <c r="N23" s="51" t="n">
-        <v>15360.31588876499</v>
+        <v>11518.93403178298</v>
       </c>
       <c r="O23" s="51" t="n">
-        <v>14172.62862752015</v>
+        <v>11734.53552346948</v>
       </c>
       <c r="P23" s="51" t="n">
-        <v>12919.40998193439</v>
+        <v>11936.81837479257</v>
       </c>
       <c r="Q23" s="51" t="n">
-        <v>11606.45808531499</v>
+        <v>12144.17836910843</v>
       </c>
       <c r="R23" s="51" t="n">
-        <v>10221.13317892016</v>
+        <v>12305.30329108986</v>
       </c>
       <c r="S23" s="51" t="n">
-        <v>8759.841590781387</v>
+        <v>12470.98383145154</v>
       </c>
       <c r="T23" s="51" t="n">
-        <v>7224.798152032797</v>
+        <v>12142.83118306861</v>
       </c>
       <c r="U23" s="51" t="n">
-        <v>5609.035449333731</v>
+        <v>11805.13633218885</v>
       </c>
       <c r="V23" s="51" t="n">
-        <v>3919.300509790613</v>
+        <v>11413.59367710975</v>
       </c>
       <c r="W23" s="51" t="n">
-        <v>2143.965938241631</v>
+        <v>11032.46410299909</v>
       </c>
       <c r="X23" s="51" t="n">
-        <v>287.4679422773584</v>
+        <v>10610.55894370964</v>
       </c>
       <c r="Y23" s="51" t="n">
-        <v>0</v>
+        <v>10217.90080845688</v>
       </c>
       <c r="Z23" s="51" t="n">
-        <v>0</v>
+        <v>9745.802910991426</v>
       </c>
       <c r="AA23" s="51" t="n">
-        <v>0</v>
+        <v>9316.339902404405</v>
       </c>
       <c r="AB23" s="51" t="n">
-        <v>0</v>
+        <v>7042.691122766559</v>
       </c>
       <c r="AC23" s="51" t="n">
-        <v>0</v>
+        <v>4548.894037665157</v>
       </c>
       <c r="AD23" s="51" t="n">
-        <v>0</v>
+        <v>2005.066016357857</v>
       </c>
       <c r="AE23" s="51" t="n">
         <v>0</v>
@@ -23918,7 +23918,7 @@
         <v>0</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>323990.5146440843</v>
+        <v>237113.0100393576</v>
       </c>
       <c r="BM23" s="58" t="inlineStr">
         <is>
@@ -24627,70 +24627,70 @@
         </is>
       </c>
       <c r="C27" s="51" t="n">
-        <v>655.1143745939253</v>
+        <v>0</v>
       </c>
       <c r="D27" s="51" t="n">
-        <v>707.9819198386576</v>
+        <v>0</v>
       </c>
       <c r="E27" s="51" t="n">
-        <v>734.549128681577</v>
+        <v>0</v>
       </c>
       <c r="F27" s="51" t="n">
-        <v>789.9273535381026</v>
+        <v>0</v>
       </c>
       <c r="G27" s="51" t="n">
-        <v>824.5447644261715</v>
+        <v>0</v>
       </c>
       <c r="H27" s="51" t="n">
-        <v>871.7885150300467</v>
+        <v>0</v>
       </c>
       <c r="I27" s="51" t="n">
-        <v>908.9520914556761</v>
+        <v>0</v>
       </c>
       <c r="J27" s="51" t="n">
-        <v>969.8207848092713</v>
+        <v>0</v>
       </c>
       <c r="K27" s="51" t="n">
-        <v>996.6349527778393</v>
+        <v>0</v>
       </c>
       <c r="L27" s="51" t="n">
-        <v>1060.223384607837</v>
+        <v>0</v>
       </c>
       <c r="M27" s="51" t="n">
-        <v>1120.146841475899</v>
+        <v>0</v>
       </c>
       <c r="N27" s="51" t="n">
-        <v>1187.687261244841</v>
+        <v>0</v>
       </c>
       <c r="O27" s="51" t="n">
-        <v>1253.218645585758</v>
+        <v>0</v>
       </c>
       <c r="P27" s="51" t="n">
-        <v>1312.951896619405</v>
+        <v>0</v>
       </c>
       <c r="Q27" s="51" t="n">
-        <v>1385.324906394822</v>
+        <v>0</v>
       </c>
       <c r="R27" s="51" t="n">
-        <v>1461.291588138776</v>
+        <v>0</v>
       </c>
       <c r="S27" s="51" t="n">
-        <v>1535.04343874859</v>
+        <v>0</v>
       </c>
       <c r="T27" s="51" t="n">
-        <v>1615.762702699066</v>
+        <v>0</v>
       </c>
       <c r="U27" s="51" t="n">
-        <v>1689.734939543118</v>
+        <v>0</v>
       </c>
       <c r="V27" s="51" t="n">
-        <v>1775.334571548982</v>
+        <v>0</v>
       </c>
       <c r="W27" s="51" t="n">
-        <v>1856.497995964273</v>
+        <v>0</v>
       </c>
       <c r="X27" s="51" t="n">
-        <v>287.4679422773584</v>
+        <v>0</v>
       </c>
       <c r="Y27" s="51" t="n">
         <v>0</v>
@@ -24699,16 +24699,16 @@
         <v>0</v>
       </c>
       <c r="AA27" s="51" t="n">
-        <v>0</v>
+        <v>2273.648779637848</v>
       </c>
       <c r="AB27" s="51" t="n">
-        <v>0</v>
+        <v>2493.797085101402</v>
       </c>
       <c r="AC27" s="51" t="n">
-        <v>0</v>
+        <v>2543.8280213073</v>
       </c>
       <c r="AD27" s="51" t="n">
-        <v>0</v>
+        <v>2005.066016357857</v>
       </c>
       <c r="AE27" s="51" t="n">
         <v>0</v>
@@ -24810,7 +24810,7 @@
         <v>0</v>
       </c>
       <c r="BL27" s="52" t="n">
-        <v>25000</v>
+        <v>9316.339902404407</v>
       </c>
       <c r="BM27" s="58" t="inlineStr">
         <is>
@@ -25519,85 +25519,85 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>24344.88562540607</v>
+        <v>1241.067170204809</v>
       </c>
       <c r="D31" s="51" t="n">
-        <v>23636.90370556742</v>
+        <v>2445.259647530023</v>
       </c>
       <c r="E31" s="51" t="n">
-        <v>22902.35457688584</v>
+        <v>3634.928820549154</v>
       </c>
       <c r="F31" s="51" t="n">
-        <v>22112.42722334773</v>
+        <v>4786.27793960481</v>
       </c>
       <c r="G31" s="51" t="n">
-        <v>21287.88245892156</v>
+        <v>5919.442429938848</v>
       </c>
       <c r="H31" s="51" t="n">
-        <v>20416.09394389152</v>
+        <v>7023.020740478265</v>
       </c>
       <c r="I31" s="51" t="n">
-        <v>19507.14185243584</v>
+        <v>8098.947216189181</v>
       </c>
       <c r="J31" s="51" t="n">
-        <v>18537.32106762657</v>
+        <v>9596.086790952748</v>
       </c>
       <c r="K31" s="51" t="n">
-        <v>17540.68611484873</v>
+        <v>11077.04490767022</v>
       </c>
       <c r="L31" s="51" t="n">
-        <v>16480.46273024089</v>
+        <v>12539.96908703129</v>
       </c>
       <c r="M31" s="51" t="n">
-        <v>15360.31588876499</v>
+        <v>12723.1265091082</v>
       </c>
       <c r="N31" s="51" t="n">
-        <v>14172.62862752015</v>
+        <v>12924.20469648861</v>
       </c>
       <c r="O31" s="51" t="n">
-        <v>12919.40998193439</v>
+        <v>13088.16749384823</v>
       </c>
       <c r="P31" s="51" t="n">
-        <v>11606.45808531499</v>
+        <v>13277.34285944247</v>
       </c>
       <c r="Q31" s="51" t="n">
-        <v>10221.13317892016</v>
+        <v>13408.88160162927</v>
       </c>
       <c r="R31" s="51" t="n">
-        <v>8759.841590781387</v>
+        <v>13546.91030716245</v>
       </c>
       <c r="S31" s="51" t="n">
-        <v>7224.798152032797</v>
+        <v>13639.97075783218</v>
       </c>
       <c r="T31" s="51" t="n">
-        <v>5609.035449333731</v>
+        <v>13286.09444890632</v>
       </c>
       <c r="U31" s="51" t="n">
-        <v>3919.300509790613</v>
+        <v>12876.51785647082</v>
       </c>
       <c r="V31" s="51" t="n">
-        <v>2143.965938241631</v>
+        <v>12456.6886952808</v>
       </c>
       <c r="W31" s="51" t="n">
-        <v>287.4679422773584</v>
+        <v>12015.82960841527</v>
       </c>
       <c r="X31" s="51" t="n">
-        <v>0</v>
+        <v>11571.53277883562</v>
       </c>
       <c r="Y31" s="51" t="n">
-        <v>0</v>
+        <v>11086.32739564132</v>
       </c>
       <c r="Z31" s="51" t="n">
-        <v>0</v>
+        <v>10581.04313492525</v>
       </c>
       <c r="AA31" s="51" t="n">
-        <v>0</v>
+        <v>7042.691122766559</v>
       </c>
       <c r="AB31" s="51" t="n">
-        <v>0</v>
+        <v>4548.894037665157</v>
       </c>
       <c r="AC31" s="51" t="n">
-        <v>0</v>
+        <v>2005.066016357857</v>
       </c>
       <c r="AD31" s="51" t="n">
         <v>0</v>
@@ -25702,7 +25702,7 @@
         <v>0</v>
       </c>
       <c r="BL31" s="52" t="n">
-        <v>298990.5146440843</v>
+        <v>256441.3340709257</v>
       </c>
       <c r="BM31" s="58" t="inlineStr">
         <is>
@@ -26474,127 +26474,127 @@
         <v>0</v>
       </c>
       <c r="X35" s="51" t="n">
-        <v>1646.338424129087</v>
+        <v>0</v>
       </c>
       <c r="Y35" s="51" t="n">
-        <v>2022.69192865896</v>
+        <v>0</v>
       </c>
       <c r="Z35" s="51" t="n">
-        <v>2118.731443842721</v>
+        <v>0</v>
       </c>
       <c r="AA35" s="51" t="n">
-        <v>4607.278452375285</v>
+        <v>0</v>
       </c>
       <c r="AB35" s="51" t="n">
-        <v>4776.369613776</v>
+        <v>0</v>
       </c>
       <c r="AC35" s="51" t="n">
-        <v>4759.925290806009</v>
+        <v>0</v>
       </c>
       <c r="AD35" s="51" t="n">
-        <v>4933.314456006903</v>
+        <v>771.1719619887167</v>
       </c>
       <c r="AE35" s="51" t="n">
-        <v>5016.091417597368</v>
+        <v>2892.668503073712</v>
       </c>
       <c r="AF35" s="51" t="n">
-        <v>5071.213301307228</v>
+        <v>3131.968093871822</v>
       </c>
       <c r="AG35" s="51" t="n">
-        <v>5053.280910902247</v>
+        <v>3271.52658396707</v>
       </c>
       <c r="AH35" s="51" t="n">
-        <v>5137.036948099522</v>
+        <v>3557.869024514927</v>
       </c>
       <c r="AI35" s="51" t="n">
-        <v>5250.977421564884</v>
+        <v>3831.037264493374</v>
       </c>
       <c r="AJ35" s="51" t="n">
-        <v>5338.01019650795</v>
+        <v>4149.71349057495</v>
       </c>
       <c r="AK35" s="51" t="n">
-        <v>5401.780310394376</v>
+        <v>4381.914784405477</v>
       </c>
       <c r="AL35" s="51" t="n">
-        <v>5491.312580732402</v>
+        <v>4732.456463680996</v>
       </c>
       <c r="AM35" s="51" t="n">
-        <v>5564.135766234725</v>
+        <v>4968.602390096292</v>
       </c>
       <c r="AN35" s="51" t="n">
-        <v>5625.280115314228</v>
+        <v>5042.623158119328</v>
       </c>
       <c r="AO35" s="51" t="n">
-        <v>5700.129335260623</v>
+        <v>5101.350395991216</v>
       </c>
       <c r="AP35" s="51" t="n">
-        <v>5794.606617060525</v>
+        <v>5215.195222996599</v>
       </c>
       <c r="AQ35" s="51" t="n">
-        <v>5850.091923793809</v>
+        <v>7018.600484524402</v>
       </c>
       <c r="AR35" s="51" t="n">
-        <v>5947.054773359453</v>
+        <v>7134.930879295526</v>
       </c>
       <c r="AS35" s="51" t="n">
-        <v>5999.679524373062</v>
+        <v>7168.188085103656</v>
       </c>
       <c r="AT35" s="51" t="n">
-        <v>6099.121726434495</v>
+        <v>7286.997832370568</v>
       </c>
       <c r="AU35" s="51" t="n">
-        <v>6203.833170484581</v>
+        <v>7375.587294346148</v>
       </c>
       <c r="AV35" s="51" t="n">
-        <v>6272.007161369031</v>
+        <v>7456.637704174131</v>
       </c>
       <c r="AW35" s="51" t="n">
-        <v>6316.696230223002</v>
+        <v>7485.204790953596</v>
       </c>
       <c r="AX35" s="51" t="n">
-        <v>6421.392852823384</v>
+        <v>7609.268958759457</v>
       </c>
       <c r="AY35" s="51" t="n">
-        <v>6447.930689543427</v>
+        <v>7616.439250274021</v>
       </c>
       <c r="AZ35" s="51" t="n">
-        <v>6554.802468928128</v>
+        <v>7742.678574864201</v>
       </c>
       <c r="BA35" s="51" t="n">
-        <v>6636.221108744508</v>
+        <v>7804.729669475102</v>
       </c>
       <c r="BB35" s="51" t="n">
-        <v>6746.213723806573</v>
+        <v>7934.089829742647</v>
       </c>
       <c r="BC35" s="51" t="n">
-        <v>6780.051659875585</v>
+        <v>7951.805783737152</v>
       </c>
       <c r="BD35" s="51" t="n">
-        <v>6854.557722072019</v>
+        <v>8039.188264877119</v>
       </c>
       <c r="BE35" s="51" t="n">
-        <v>6848.555807320907</v>
+        <v>8017.0643680515</v>
       </c>
       <c r="BF35" s="51" t="n">
-        <v>6962.067782027882</v>
+        <v>8149.943887963956</v>
       </c>
       <c r="BG35" s="51" t="n">
-        <v>6925.218182124281</v>
+        <v>8093.726742854875</v>
       </c>
       <c r="BH35" s="51" t="n">
-        <v>7040.000803927449</v>
+        <v>8227.876909863522</v>
       </c>
       <c r="BI35" s="51" t="n">
-        <v>6945.581281234856</v>
+        <v>8114.08984196545</v>
       </c>
       <c r="BJ35" s="51" t="n">
-        <v>7060.70141296803</v>
+        <v>8248.577518904103</v>
       </c>
       <c r="BK35" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL35" s="52" t="n">
-        <v>220276.4089620228</v>
+        <v>205579.8484358929</v>
       </c>
       <c r="BM35" s="58" t="inlineStr">
         <is>
@@ -27299,7 +27299,7 @@
       </c>
       <c r="B39" s="50" t="inlineStr">
         <is>
-          <t>runtime.cit_accrual_audit_keur</t>
+          <t>runtime.tax_keur</t>
         </is>
       </c>
       <c r="C39" s="51" t="n">
@@ -27366,127 +27366,127 @@
         <v>0</v>
       </c>
       <c r="X39" s="51" t="n">
-        <v>296.3409163432357</v>
+        <v>0</v>
       </c>
       <c r="Y39" s="51" t="n">
-        <v>364.0845471586127</v>
+        <v>0</v>
       </c>
       <c r="Z39" s="51" t="n">
-        <v>381.3716598916898</v>
+        <v>0</v>
       </c>
       <c r="AA39" s="51" t="n">
-        <v>829.3101214275513</v>
+        <v>0</v>
       </c>
       <c r="AB39" s="51" t="n">
-        <v>859.7465304796799</v>
+        <v>0</v>
       </c>
       <c r="AC39" s="51" t="n">
-        <v>856.7865523450815</v>
+        <v>0</v>
       </c>
       <c r="AD39" s="51" t="n">
-        <v>887.9966020812425</v>
+        <v>138.810953157969</v>
       </c>
       <c r="AE39" s="51" t="n">
-        <v>902.8964551675261</v>
+        <v>520.680330553268</v>
       </c>
       <c r="AF39" s="51" t="n">
-        <v>912.818394235301</v>
+        <v>563.7542568969279</v>
       </c>
       <c r="AG39" s="51" t="n">
-        <v>909.5905639624045</v>
+        <v>588.8747851140726</v>
       </c>
       <c r="AH39" s="51" t="n">
-        <v>924.666650657914</v>
+        <v>640.4164244126869</v>
       </c>
       <c r="AI39" s="51" t="n">
-        <v>945.175935881679</v>
+        <v>689.5867076088073</v>
       </c>
       <c r="AJ39" s="51" t="n">
-        <v>960.841835371431</v>
+        <v>746.9484283034909</v>
       </c>
       <c r="AK39" s="51" t="n">
-        <v>972.3204558709876</v>
+        <v>788.7446611929859</v>
       </c>
       <c r="AL39" s="51" t="n">
-        <v>988.4362645318324</v>
+        <v>851.8421634625794</v>
       </c>
       <c r="AM39" s="51" t="n">
-        <v>1001.54443792225</v>
+        <v>894.3484302173325</v>
       </c>
       <c r="AN39" s="51" t="n">
-        <v>1012.550420756561</v>
+        <v>907.672168461479</v>
       </c>
       <c r="AO39" s="51" t="n">
-        <v>1026.023280346912</v>
+        <v>918.2430712784188</v>
       </c>
       <c r="AP39" s="51" t="n">
-        <v>1043.029191070895</v>
+        <v>938.7351401393878</v>
       </c>
       <c r="AQ39" s="51" t="n">
-        <v>1053.016546282885</v>
+        <v>1263.348087214392</v>
       </c>
       <c r="AR39" s="51" t="n">
-        <v>1070.469859204702</v>
+        <v>1284.287558273195</v>
       </c>
       <c r="AS39" s="51" t="n">
-        <v>1079.942314387151</v>
+        <v>1290.273855318658</v>
       </c>
       <c r="AT39" s="51" t="n">
-        <v>1097.841910758209</v>
+        <v>1311.659609826702</v>
       </c>
       <c r="AU39" s="51" t="n">
-        <v>1116.689970687225</v>
+        <v>1327.605712982307</v>
       </c>
       <c r="AV39" s="51" t="n">
-        <v>1128.961289046425</v>
+        <v>1342.194786751343</v>
       </c>
       <c r="AW39" s="51" t="n">
-        <v>1137.00532144014</v>
+        <v>1347.336862371647</v>
       </c>
       <c r="AX39" s="51" t="n">
-        <v>1155.850713508209</v>
+        <v>1369.668412576702</v>
       </c>
       <c r="AY39" s="51" t="n">
-        <v>1160.627524117817</v>
+        <v>1370.959065049324</v>
       </c>
       <c r="AZ39" s="51" t="n">
-        <v>1179.864444407063</v>
+        <v>1393.682143475556</v>
       </c>
       <c r="BA39" s="51" t="n">
-        <v>1194.519799574012</v>
+        <v>1404.851340505518</v>
       </c>
       <c r="BB39" s="51" t="n">
-        <v>1214.318470285183</v>
+        <v>1428.136169353676</v>
       </c>
       <c r="BC39" s="51" t="n">
-        <v>1220.409298777605</v>
+        <v>1431.325041072687</v>
       </c>
       <c r="BD39" s="51" t="n">
-        <v>1233.820389972963</v>
+        <v>1447.053887677881</v>
       </c>
       <c r="BE39" s="51" t="n">
-        <v>1232.740045317763</v>
+        <v>1443.07158624927</v>
       </c>
       <c r="BF39" s="51" t="n">
-        <v>1253.172200765019</v>
+        <v>1466.989899833512</v>
       </c>
       <c r="BG39" s="51" t="n">
-        <v>1246.539272782371</v>
+        <v>1456.870813713877</v>
       </c>
       <c r="BH39" s="51" t="n">
-        <v>1267.200144706941</v>
+        <v>1481.017843775434</v>
       </c>
       <c r="BI39" s="51" t="n">
-        <v>1250.204630622274</v>
+        <v>1460.536171553781</v>
       </c>
       <c r="BJ39" s="51" t="n">
-        <v>1270.926254334245</v>
+        <v>1484.743953402738</v>
       </c>
       <c r="BK39" s="51" t="n">
         <v>10.10239668311311</v>
       </c>
       <c r="BL39" s="52" t="n">
-        <v>39649.75361316411</v>
+        <v>37004.37271846071</v>
       </c>
       <c r="BM39" s="58" t="inlineStr">
         <is>
@@ -27836,7 +27836,7 @@
       </c>
       <c r="BO40" s="58" t="inlineStr">
         <is>
-          <t>The runtime audit field exists for CIT accrual, but the committed Excel evidence pack does not include a matching row.</t>
+          <t>The runtime CIT accrual is in tax_keur, but the committed Excel evidence pack does not include a matching row.</t>
         </is>
       </c>
       <c r="BP40" s="58" t="inlineStr">
@@ -28191,7 +28191,7 @@
       </c>
       <c r="B43" s="50" t="inlineStr">
         <is>
-          <t>runtime.cash_tax_current_period_audit_keur</t>
+          <t>runtime.corporate_tax_cash_keur</t>
         </is>
       </c>
       <c r="C43" s="51" t="n">
@@ -28258,127 +28258,127 @@
         <v>0</v>
       </c>
       <c r="X43" s="51" t="n">
-        <v>296.3409163432357</v>
+        <v>0</v>
       </c>
       <c r="Y43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="Z43" s="51" t="n">
-        <v>381.3716598916898</v>
+        <v>0</v>
       </c>
       <c r="AA43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AB43" s="51" t="n">
-        <v>859.7465304796799</v>
+        <v>0</v>
       </c>
       <c r="AC43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AD43" s="51" t="n">
-        <v>887.9966020812425</v>
+        <v>138.810953157969</v>
       </c>
       <c r="AE43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AF43" s="51" t="n">
-        <v>912.818394235301</v>
+        <v>1084.434587450196</v>
       </c>
       <c r="AG43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AH43" s="51" t="n">
-        <v>924.666650657914</v>
+        <v>1229.291209526759</v>
       </c>
       <c r="AI43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AJ43" s="51" t="n">
-        <v>960.841835371431</v>
+        <v>1436.535135912298</v>
       </c>
       <c r="AK43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AL43" s="51" t="n">
-        <v>988.4362645318324</v>
+        <v>1640.586824655565</v>
       </c>
       <c r="AM43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AN43" s="51" t="n">
-        <v>1012.550420756561</v>
+        <v>1802.020598678811</v>
       </c>
       <c r="AO43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AP43" s="51" t="n">
-        <v>1043.029191070895</v>
+        <v>1856.978211417807</v>
       </c>
       <c r="AQ43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AR43" s="51" t="n">
-        <v>1070.469859204702</v>
+        <v>2547.635645487587</v>
       </c>
       <c r="AS43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AT43" s="51" t="n">
-        <v>1097.841910758209</v>
+        <v>2601.93346514536</v>
       </c>
       <c r="AU43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AV43" s="51" t="n">
-        <v>1128.961289046425</v>
+        <v>2669.80049973365</v>
       </c>
       <c r="AW43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AX43" s="51" t="n">
-        <v>1155.850713508209</v>
+        <v>2717.005274948349</v>
       </c>
       <c r="AY43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AZ43" s="51" t="n">
-        <v>1179.864444407063</v>
+        <v>2764.64120852488</v>
       </c>
       <c r="BA43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BB43" s="51" t="n">
-        <v>1214.318470285183</v>
+        <v>2832.987509859195</v>
       </c>
       <c r="BC43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BD43" s="51" t="n">
-        <v>1233.820389972963</v>
+        <v>2878.378928750569</v>
       </c>
       <c r="BE43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BF43" s="51" t="n">
-        <v>1253.172200765019</v>
+        <v>2910.061486082782</v>
       </c>
       <c r="BG43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BH43" s="51" t="n">
-        <v>1267.200144706941</v>
+        <v>2937.888657489311</v>
       </c>
       <c r="BI43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BJ43" s="51" t="n">
-        <v>1270.926254334245</v>
+        <v>2945.280124956519</v>
       </c>
       <c r="BK43" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BL43" s="52" t="n">
-        <v>20140.22414240874</v>
+        <v>36994.27032177761</v>
       </c>
       <c r="BM43" s="58" t="inlineStr">
         <is>
@@ -28728,7 +28728,7 @@
       </c>
       <c r="BO44" s="58" t="inlineStr">
         <is>
-          <t>Current-period cash tax is already exposed through runtime audit fields, but the committed Excel evidence pack has no matching line.</t>
+          <t>Current-period cash tax is in corporate_tax_cash_keur, but the committed Excel evidence pack has no matching line.</t>
         </is>
       </c>
       <c r="BP44" s="58" t="inlineStr">
@@ -30267,127 +30267,127 @@
         <v>0</v>
       </c>
       <c r="X11" s="51" t="n">
-        <v>296.3409163432357</v>
+        <v>0</v>
       </c>
       <c r="Y11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="Z11" s="51" t="n">
-        <v>381.3716598916898</v>
+        <v>0</v>
       </c>
       <c r="AA11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AB11" s="51" t="n">
-        <v>859.7465304796799</v>
+        <v>0</v>
       </c>
       <c r="AC11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AD11" s="51" t="n">
-        <v>887.9966020812425</v>
+        <v>138.810953157969</v>
       </c>
       <c r="AE11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AF11" s="51" t="n">
-        <v>912.818394235301</v>
+        <v>1084.434587450196</v>
       </c>
       <c r="AG11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AH11" s="51" t="n">
-        <v>924.666650657914</v>
+        <v>1229.291209526759</v>
       </c>
       <c r="AI11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AJ11" s="51" t="n">
-        <v>960.841835371431</v>
+        <v>1436.535135912298</v>
       </c>
       <c r="AK11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AL11" s="51" t="n">
-        <v>988.4362645318324</v>
+        <v>1640.586824655565</v>
       </c>
       <c r="AM11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AN11" s="51" t="n">
-        <v>1012.550420756561</v>
+        <v>1802.020598678811</v>
       </c>
       <c r="AO11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AP11" s="51" t="n">
-        <v>1043.029191070895</v>
+        <v>1856.978211417807</v>
       </c>
       <c r="AQ11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AR11" s="51" t="n">
-        <v>1070.469859204702</v>
+        <v>2547.635645487587</v>
       </c>
       <c r="AS11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AT11" s="51" t="n">
-        <v>1097.841910758209</v>
+        <v>2601.93346514536</v>
       </c>
       <c r="AU11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AV11" s="51" t="n">
-        <v>1128.961289046425</v>
+        <v>2669.80049973365</v>
       </c>
       <c r="AW11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AX11" s="51" t="n">
-        <v>1155.850713508209</v>
+        <v>2717.005274948349</v>
       </c>
       <c r="AY11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="AZ11" s="51" t="n">
-        <v>1179.864444407063</v>
+        <v>2764.64120852488</v>
       </c>
       <c r="BA11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BB11" s="51" t="n">
-        <v>1214.318470285183</v>
+        <v>2832.987509859195</v>
       </c>
       <c r="BC11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BD11" s="51" t="n">
-        <v>1233.820389972963</v>
+        <v>2878.378928750569</v>
       </c>
       <c r="BE11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BF11" s="51" t="n">
-        <v>1253.172200765019</v>
+        <v>2910.061486082782</v>
       </c>
       <c r="BG11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BH11" s="51" t="n">
-        <v>1267.200144706941</v>
+        <v>2937.888657489311</v>
       </c>
       <c r="BI11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BJ11" s="51" t="n">
-        <v>1270.926254334245</v>
+        <v>2945.280124956519</v>
       </c>
       <c r="BK11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="BL11" s="52" t="n">
-        <v>20140.22414240874</v>
+        <v>36994.27032177761</v>
       </c>
       <c r="BM11" s="58" t="inlineStr">
         <is>
@@ -31159,127 +31159,127 @@
         <v>3607.952524064416</v>
       </c>
       <c r="X15" s="51" t="n">
-        <v>3351.259437655953</v>
+        <v>3647.600353999189</v>
       </c>
       <c r="Y15" s="51" t="n">
         <v>3667.635538833556</v>
       </c>
       <c r="Z15" s="51" t="n">
-        <v>3347.053418259549</v>
+        <v>3728.425078151239</v>
       </c>
       <c r="AA15" s="51" t="n">
         <v>6140.284473381875</v>
       </c>
       <c r="AB15" s="51" t="n">
-        <v>5382.310613731728</v>
+        <v>6242.057144211408</v>
       </c>
       <c r="AC15" s="51" t="n">
         <v>6115.456541519213</v>
       </c>
       <c r="AD15" s="51" t="n">
-        <v>5328.821097584698</v>
+        <v>6078.006746507971</v>
       </c>
       <c r="AE15" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF15" s="51" t="n">
-        <v>5343.025449877027</v>
+        <v>5171.409256662132</v>
       </c>
       <c r="AG15" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH15" s="51" t="n">
-        <v>5400.246403377681</v>
+        <v>5095.621844508836</v>
       </c>
       <c r="AI15" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ15" s="51" t="n">
-        <v>5565.044467072592</v>
+        <v>5089.351166531726</v>
       </c>
       <c r="AK15" s="51" t="n">
         <v>6570.28887112497</v>
       </c>
       <c r="AL15" s="51" t="n">
-        <v>5690.752422136643</v>
+        <v>5038.601862012911</v>
       </c>
       <c r="AM15" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN15" s="51" t="n">
-        <v>5797.360237362767</v>
+        <v>5007.890059440517</v>
       </c>
       <c r="AO15" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP15" s="51" t="n">
-        <v>5939.453531925704</v>
+        <v>5125.504511578793</v>
       </c>
       <c r="AQ15" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR15" s="51" t="n">
-        <v>6064.461020090825</v>
+        <v>4587.295233807939</v>
       </c>
       <c r="AS15" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT15" s="51" t="n">
-        <v>6189.155921612359</v>
+        <v>4685.064367225208</v>
       </c>
       <c r="AU15" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV15" s="51" t="n">
-        <v>6327.676415127706</v>
+        <v>4786.83720444048</v>
       </c>
       <c r="AW15" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX15" s="51" t="n">
-        <v>6453.418245251248</v>
+        <v>4892.263683811108</v>
       </c>
       <c r="AY15" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ15" s="51" t="n">
-        <v>6562.814130457138</v>
+        <v>4978.037366339322</v>
       </c>
       <c r="BA15" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB15" s="51" t="n">
-        <v>6719.771359457463</v>
+        <v>5101.102319883452</v>
       </c>
       <c r="BC15" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD15" s="51" t="n">
-        <v>6805.367874904156</v>
+        <v>5160.80933612655</v>
       </c>
       <c r="BE15" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF15" s="51" t="n">
-        <v>6896.771687198937</v>
+        <v>5239.882401881174</v>
       </c>
       <c r="BG15" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH15" s="51" t="n">
-        <v>6960.676765156581</v>
+        <v>5289.988252374211</v>
       </c>
       <c r="BI15" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ15" s="51" t="n">
-        <v>6977.651264569858</v>
+        <v>5303.297393947584</v>
       </c>
       <c r="BK15" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL15" s="52" t="n">
-        <v>318295.1130998204</v>
+        <v>301441.0669204517</v>
       </c>
       <c r="BM15" s="58" t="inlineStr">
         <is>
@@ -31807,127 +31807,127 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X19" s="51" t="n">
-        <v>988.064850480836</v>
+        <v>1284.405766824072</v>
       </c>
       <c r="Y19" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z19" s="51" t="n">
-        <v>931.4943908801665</v>
+        <v>1312.866050771856</v>
       </c>
       <c r="AA19" s="51" t="n">
         <v>2760.620551308993</v>
       </c>
       <c r="AB19" s="51" t="n">
-        <v>1946.630162563717</v>
+        <v>2806.376693043396</v>
       </c>
       <c r="AC19" s="51" t="n">
         <v>2749.45812076629</v>
       </c>
       <c r="AD19" s="51" t="n">
-        <v>1907.032647758631</v>
+        <v>2656.218296681904</v>
       </c>
       <c r="AE19" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF19" s="51" t="n">
-        <v>5343.025449877027</v>
+        <v>5171.409256662132</v>
       </c>
       <c r="AG19" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH19" s="51" t="n">
-        <v>5400.246403377681</v>
+        <v>5095.621844508836</v>
       </c>
       <c r="AI19" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ19" s="51" t="n">
-        <v>5565.044467072592</v>
+        <v>5089.351166531726</v>
       </c>
       <c r="AK19" s="51" t="n">
         <v>6570.28887112497</v>
       </c>
       <c r="AL19" s="51" t="n">
-        <v>5690.752422136643</v>
+        <v>5038.601862012911</v>
       </c>
       <c r="AM19" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN19" s="51" t="n">
-        <v>5797.360237362767</v>
+        <v>5007.890059440517</v>
       </c>
       <c r="AO19" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP19" s="51" t="n">
-        <v>5939.453531925704</v>
+        <v>5125.504511578793</v>
       </c>
       <c r="AQ19" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR19" s="51" t="n">
-        <v>6064.461020090825</v>
+        <v>4587.295233807939</v>
       </c>
       <c r="AS19" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT19" s="51" t="n">
-        <v>6189.155921612359</v>
+        <v>4685.064367225208</v>
       </c>
       <c r="AU19" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV19" s="51" t="n">
-        <v>6327.676415127706</v>
+        <v>4786.83720444048</v>
       </c>
       <c r="AW19" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX19" s="51" t="n">
-        <v>6453.418245251248</v>
+        <v>4892.263683811108</v>
       </c>
       <c r="AY19" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ19" s="51" t="n">
-        <v>6562.814130457138</v>
+        <v>4978.037366339322</v>
       </c>
       <c r="BA19" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB19" s="51" t="n">
-        <v>6719.771359457463</v>
+        <v>5101.102319883452</v>
       </c>
       <c r="BC19" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD19" s="51" t="n">
-        <v>6805.367874904156</v>
+        <v>5160.80933612655</v>
       </c>
       <c r="BE19" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF19" s="51" t="n">
-        <v>6896.771687198937</v>
+        <v>5239.882401881174</v>
       </c>
       <c r="BG19" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH19" s="51" t="n">
-        <v>6960.676765156581</v>
+        <v>5289.988252374211</v>
       </c>
       <c r="BI19" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ19" s="51" t="n">
-        <v>6977.651264569858</v>
+        <v>5303.297393947584</v>
       </c>
       <c r="BK19" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL19" s="52" t="n">
-        <v>252468.7248196141</v>
+        <v>235614.6786402452</v>
       </c>
       <c r="BM19" s="77" t="inlineStr">
         <is>
@@ -32455,127 +32455,127 @@
         <v>1270.444834575984</v>
       </c>
       <c r="X23" s="51" t="n">
-        <v>988.064850480836</v>
+        <v>1284.405766824072</v>
       </c>
       <c r="Y23" s="51" t="n">
         <v>1291.460626031011</v>
       </c>
       <c r="Z23" s="51" t="n">
-        <v>931.4943908801665</v>
+        <v>1312.866050771856</v>
       </c>
       <c r="AA23" s="51" t="n">
         <v>2760.620551308993</v>
       </c>
       <c r="AB23" s="51" t="n">
-        <v>1946.630162563717</v>
+        <v>2806.376693043396</v>
       </c>
       <c r="AC23" s="51" t="n">
         <v>2749.45812076629</v>
       </c>
       <c r="AD23" s="51" t="n">
-        <v>1907.032647758631</v>
+        <v>2656.218296681904</v>
       </c>
       <c r="AE23" s="51" t="n">
         <v>6187.845541458934</v>
       </c>
       <c r="AF23" s="51" t="n">
-        <v>5343.025449877027</v>
+        <v>5171.409256662132</v>
       </c>
       <c r="AG23" s="51" t="n">
         <v>6221.789471632841</v>
       </c>
       <c r="AH23" s="51" t="n">
-        <v>5400.246403377681</v>
+        <v>5095.621844508836</v>
       </c>
       <c r="AI23" s="51" t="n">
         <v>6419.485982295478</v>
       </c>
       <c r="AJ23" s="51" t="n">
-        <v>5565.044467072592</v>
+        <v>5089.351166531726</v>
       </c>
       <c r="AK23" s="51" t="n">
         <v>6570.28887112497</v>
       </c>
       <c r="AL23" s="51" t="n">
-        <v>5690.752422136643</v>
+        <v>5038.601862012911</v>
       </c>
       <c r="AM23" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN23" s="51" t="n">
-        <v>5797.360237362767</v>
+        <v>5007.890059440517</v>
       </c>
       <c r="AO23" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP23" s="51" t="n">
-        <v>5939.453531925704</v>
+        <v>5125.504511578793</v>
       </c>
       <c r="AQ23" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR23" s="51" t="n">
-        <v>6064.461020090825</v>
+        <v>4587.295233807939</v>
       </c>
       <c r="AS23" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT23" s="51" t="n">
-        <v>6189.155921612359</v>
+        <v>4685.064367225208</v>
       </c>
       <c r="AU23" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV23" s="51" t="n">
-        <v>6327.676415127706</v>
+        <v>4786.83720444048</v>
       </c>
       <c r="AW23" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX23" s="51" t="n">
-        <v>6453.418245251248</v>
+        <v>4892.263683811108</v>
       </c>
       <c r="AY23" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ23" s="51" t="n">
-        <v>6562.814130457138</v>
+        <v>4978.037366339322</v>
       </c>
       <c r="BA23" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB23" s="51" t="n">
-        <v>6719.771359457463</v>
+        <v>5101.102319883452</v>
       </c>
       <c r="BC23" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD23" s="51" t="n">
-        <v>6805.367874904156</v>
+        <v>5160.80933612655</v>
       </c>
       <c r="BE23" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF23" s="51" t="n">
-        <v>6896.771687198937</v>
+        <v>5239.882401881174</v>
       </c>
       <c r="BG23" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH23" s="51" t="n">
-        <v>6960.676765156581</v>
+        <v>5289.988252374211</v>
       </c>
       <c r="BI23" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ23" s="51" t="n">
-        <v>6977.651264569858</v>
+        <v>5303.297393947584</v>
       </c>
       <c r="BK23" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL23" s="52" t="n">
-        <v>252468.7248196141</v>
+        <v>235614.6786402452</v>
       </c>
       <c r="BM23" s="77" t="inlineStr">
         <is>
@@ -33755,88 +33755,88 @@
         <v>0</v>
       </c>
       <c r="AK7" s="51" t="n">
-        <v>6398.064261517846</v>
+        <v>6449.538993624739</v>
       </c>
       <c r="AL7" s="51" t="n">
-        <v>5690.752422136643</v>
+        <v>4740.166944215696</v>
       </c>
       <c r="AM7" s="51" t="n">
         <v>6735.889890096291</v>
       </c>
       <c r="AN7" s="51" t="n">
-        <v>5797.360237362767</v>
+        <v>4795.815799440517</v>
       </c>
       <c r="AO7" s="51" t="n">
         <v>6868.637895991216</v>
       </c>
       <c r="AP7" s="51" t="n">
-        <v>5939.453531925704</v>
+        <v>4913.430251578792</v>
       </c>
       <c r="AQ7" s="51" t="n">
         <v>7018.600484524402</v>
       </c>
       <c r="AR7" s="51" t="n">
-        <v>6064.461020090825</v>
+        <v>5011.444473807939</v>
       </c>
       <c r="AS7" s="51" t="n">
         <v>7168.188085103656</v>
       </c>
       <c r="AT7" s="51" t="n">
-        <v>6189.155921612359</v>
+        <v>5109.213607225208</v>
       </c>
       <c r="AU7" s="51" t="n">
         <v>7375.587294346148</v>
       </c>
       <c r="AV7" s="51" t="n">
-        <v>6327.676415127706</v>
+        <v>5210.986444440481</v>
       </c>
       <c r="AW7" s="51" t="n">
         <v>7485.204790953596</v>
       </c>
       <c r="AX7" s="51" t="n">
-        <v>6453.418245251248</v>
+        <v>5316.412923811107</v>
       </c>
       <c r="AY7" s="51" t="n">
         <v>7616.439250274021</v>
       </c>
       <c r="AZ7" s="51" t="n">
-        <v>6562.814130457138</v>
+        <v>5402.186606339322</v>
       </c>
       <c r="BA7" s="51" t="n">
         <v>7804.729669475102</v>
       </c>
       <c r="BB7" s="51" t="n">
-        <v>6719.771359457463</v>
+        <v>5525.251559883452</v>
       </c>
       <c r="BC7" s="51" t="n">
         <v>7951.805783737152</v>
       </c>
       <c r="BD7" s="51" t="n">
-        <v>6805.367874904156</v>
+        <v>5584.95857612655</v>
       </c>
       <c r="BE7" s="51" t="n">
         <v>8017.0643680515</v>
       </c>
       <c r="BF7" s="51" t="n">
-        <v>6896.771687198937</v>
+        <v>5664.031641881174</v>
       </c>
       <c r="BG7" s="51" t="n">
         <v>8093.726742854875</v>
       </c>
       <c r="BH7" s="51" t="n">
-        <v>6960.676765156581</v>
+        <v>5714.137492374211</v>
       </c>
       <c r="BI7" s="51" t="n">
         <v>8114.08984196545</v>
       </c>
       <c r="BJ7" s="51" t="n">
-        <v>6977.651264569858</v>
+        <v>5727.446633947584</v>
       </c>
       <c r="BK7" s="51" t="n">
         <v>56.12442601729508</v>
       </c>
       <c r="BL7" s="52" t="n">
-        <v>180089.4836601599</v>
+        <v>165471.1104720874</v>
       </c>
       <c r="BM7" s="79" t="inlineStr">
         <is>
@@ -33967,88 +33967,88 @@
         <v>0</v>
       </c>
       <c r="AK8" s="51" t="n">
-        <v>6398.064261517846</v>
+        <v>6449.538993624739</v>
       </c>
       <c r="AL8" s="51" t="n">
-        <v>5688.463380105447</v>
+        <v>4737.8779021845</v>
       </c>
       <c r="AM8" s="51" t="n">
         <v>6279.82438136977</v>
       </c>
       <c r="AN8" s="51" t="n">
-        <v>-957.884706851185</v>
+        <v>-1959.429144773435</v>
       </c>
       <c r="AO8" s="51" t="n">
         <v>1829.598176827532</v>
       </c>
       <c r="AP8" s="51" t="n">
-        <v>-959.2348745900836</v>
+        <v>-1985.258154936995</v>
       </c>
       <c r="AQ8" s="51" t="n">
         <v>2399.662843169288</v>
       </c>
       <c r="AR8" s="51" t="n">
-        <v>-958.9005629555177</v>
+        <v>-2011.917109238403</v>
       </c>
       <c r="AS8" s="51" t="n">
         <v>2553.912986264261</v>
       </c>
       <c r="AT8" s="51" t="n">
-        <v>-998.9280052432796</v>
+        <v>-2078.87031963043</v>
       </c>
       <c r="AU8" s="51" t="n">
         <v>2653.013886220987</v>
       </c>
       <c r="AV8" s="51" t="n">
-        <v>-1083.746844591877</v>
+        <v>-2200.436815279101</v>
       </c>
       <c r="AW8" s="51" t="n">
         <v>2650.095104931563</v>
       </c>
       <c r="AX8" s="51" t="n">
-        <v>-1084.175519478922</v>
+        <v>-2221.180840919063</v>
       </c>
       <c r="AY8" s="51" t="n">
         <v>2664.474182350282</v>
       </c>
       <c r="AZ8" s="51" t="n">
-        <v>-1123.527521187737</v>
+        <v>-2284.155045305553</v>
       </c>
       <c r="BA8" s="51" t="n">
         <v>2754.947169664165</v>
       </c>
       <c r="BB8" s="51" t="n">
-        <v>-1135.358429515777</v>
+        <v>-2329.878229089789</v>
       </c>
       <c r="BC8" s="51" t="n">
         <v>2791.409369359826</v>
       </c>
       <c r="BD8" s="51" t="n">
-        <v>-1216.386437867111</v>
+        <v>-2436.795736644717</v>
       </c>
       <c r="BE8" s="51" t="n">
         <v>2784.06653034275</v>
       </c>
       <c r="BF8" s="51" t="n">
-        <v>-1210.356704635606</v>
+        <v>-2443.096749953369</v>
       </c>
       <c r="BG8" s="51" t="n">
         <v>2767.937934958465</v>
       </c>
       <c r="BH8" s="51" t="n">
-        <v>-1244.509601780442</v>
+        <v>-2491.048874562813</v>
       </c>
       <c r="BI8" s="51" t="n">
         <v>2724.195775499138</v>
       </c>
       <c r="BJ8" s="51" t="n">
-        <v>-1270.483573714036</v>
+        <v>-2520.688204336309</v>
       </c>
       <c r="BK8" s="51" t="n">
         <v>-5316.083126731314</v>
       </c>
       <c r="BL8" s="80" t="n">
-        <v>28380.09007343833</v>
+        <v>13761.71688536589</v>
       </c>
       <c r="BM8" s="79" t="inlineStr">
         <is>
@@ -37638,7 +37638,7 @@
       <c r="BJ11" s="70" t="inlineStr"/>
       <c r="BK11" s="70" t="inlineStr"/>
       <c r="BL11" s="83" t="n">
-        <v>0.1158773428956301</v>
+        <v>0.1132136369574784</v>
       </c>
       <c r="BM11" s="67" t="inlineStr">
         <is>
@@ -37972,7 +37972,7 @@
         </is>
       </c>
       <c r="BL12" s="85" t="n">
-        <v>-0.0002226571043698472</v>
+        <v>-0.002886363042521586</v>
       </c>
       <c r="BM12" s="67" t="inlineStr">
         <is>
@@ -40917,7 +40917,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-05T16:17:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -41035,7 +41035,7 @@
       </c>
       <c r="B9" s="89" t="inlineStr">
         <is>
-          <t>0.115877</t>
+          <t>0.113214</t>
         </is>
       </c>
       <c r="C9" s="89" t="inlineStr">
@@ -41045,7 +41045,7 @@
       </c>
       <c r="D9" s="89" t="inlineStr">
         <is>
-          <t>-0.000223</t>
+          <t>-0.002886</t>
         </is>
       </c>
       <c r="E9" s="90" t="inlineStr">
@@ -41360,7 +41360,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CIRR Reconciliation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-05T16:17:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -41412,7 +41412,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-05T16:17:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -42376,7 +42376,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CCalibration Residual Closeout&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-05T16:17:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -42532,7 +42532,7 @@
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>252468.7248196141</t>
+          <t>235614.6786402452</t>
         </is>
       </c>
       <c r="E6" s="21" t="inlineStr">
@@ -42609,7 +42609,7 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>252468.7248196141</t>
+          <t>235614.6786402452</t>
         </is>
       </c>
       <c r="E7" s="21" t="inlineStr">
@@ -42753,22 +42753,22 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>Debt Service</t>
+          <t>Opening Balance</t>
         </is>
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>66181.34723683617</t>
+          <t>756328.0823817672</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>32853.2998091612</t>
+          <t>781474.3749637025</t>
         </is>
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>-33328.04742767497</t>
+          <t>25146.292581935297</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
@@ -42783,12 +42783,12 @@
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
-          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
+          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
         </is>
       </c>
       <c r="I9" s="21" t="inlineStr">
         <is>
-          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
+          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
         </is>
       </c>
       <c r="J9" s="21" t="inlineStr">
@@ -42818,7 +42818,7 @@
       </c>
       <c r="O9" s="21" t="inlineStr">
         <is>
-          <t>Derived from existing interest and principal rows.</t>
+          <t>No debt sizing rewrite is implied.</t>
         </is>
       </c>
     </row>
@@ -42830,22 +42830,22 @@
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>Opening Balance</t>
+          <t>Closing Balance</t>
         </is>
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>756328.0823817672</t>
+          <t>712969.5518136513</t>
         </is>
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>781474.3749637025</t>
+          <t>738115.3749637026</t>
         </is>
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>25146.292581935297</t>
+          <t>25145.823150051292</t>
         </is>
       </c>
       <c r="F10" s="21" t="inlineStr">
@@ -42860,12 +42860,12 @@
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
-          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
+          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
         </is>
       </c>
       <c r="I10" s="21" t="inlineStr">
         <is>
-          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
+          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
         </is>
       </c>
       <c r="J10" s="21" t="inlineStr">
@@ -42895,34 +42895,34 @@
       </c>
       <c r="O10" s="21" t="inlineStr">
         <is>
-          <t>No debt sizing rewrite is implied.</t>
+          <t>No runtime change implied.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt</t>
+          <t>SHL</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Closing Balance</t>
+          <t>Principal Repaid</t>
         </is>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>712969.5518136513</t>
+          <t>14595.529999999999</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>738115.3749637026</t>
+          <t>37326.33183100554</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>25145.823150051292</t>
+          <t>22730.80183100554</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
@@ -42937,22 +42937,22 @@
       </c>
       <c r="H11" s="21" t="inlineStr">
         <is>
-          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
+          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
         </is>
       </c>
       <c r="I11" s="21" t="inlineStr">
         <is>
-          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
+          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
         </is>
       </c>
       <c r="J11" s="21" t="inlineStr">
         <is>
-          <t>Review only</t>
+          <t>Stakeholder review only</t>
         </is>
       </c>
       <c r="K11" s="21" t="inlineStr">
         <is>
-          <t>Debt</t>
+          <t>Sponsor / SHL</t>
         </is>
       </c>
       <c r="L11" s="21" t="inlineStr">
@@ -42972,7 +42972,7 @@
       </c>
       <c r="O11" s="21" t="inlineStr">
         <is>
-          <t>No runtime change implied.</t>
+          <t>No new SHL timing change is made here.</t>
         </is>
       </c>
     </row>
@@ -42984,22 +42984,22 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Principal Repaid</t>
+          <t>Gross Accrued Interest</t>
         </is>
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>14595.529999999999</t>
+          <t>38755.380000000005</t>
         </is>
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>38028.01009465598</t>
+          <t>44068.95868964389</t>
         </is>
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>23432.480094655984</t>
+          <t>5313.578689643888</t>
         </is>
       </c>
       <c r="F12" s="21" t="inlineStr">
@@ -43014,17 +43014,17 @@
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
+          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
         </is>
       </c>
       <c r="I12" s="21" t="inlineStr">
         <is>
-          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
+          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
         </is>
       </c>
       <c r="J12" s="21" t="inlineStr">
         <is>
-          <t>Stakeholder review only</t>
+          <t>Review only</t>
         </is>
       </c>
       <c r="K12" s="21" t="inlineStr">
@@ -43049,34 +43049,34 @@
       </c>
       <c r="O12" s="21" t="inlineStr">
         <is>
-          <t>No new SHL timing change is made here.</t>
+          <t>Gross accrued interest is the authoritative model-side SHL P&amp;L bridge.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>SHL</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>Gross Accrued Interest</t>
+          <t>Total OPEX</t>
         </is>
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>38755.380000000005</t>
+          <t>84674.77873934136</t>
         </is>
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>44736.24440845805</t>
+          <t>85408.27413448405</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
         <is>
-          <t>5980.864408458045</t>
+          <t>733.4953951426869</t>
         </is>
       </c>
       <c r="F13" s="21" t="inlineStr">
@@ -43091,22 +43091,22 @@
       </c>
       <c r="H13" s="21" t="inlineStr">
         <is>
-          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
+          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
         </is>
       </c>
       <c r="I13" s="21" t="inlineStr">
         <is>
-          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
+          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
         </is>
       </c>
       <c r="J13" s="21" t="inlineStr">
         <is>
-          <t>Review only</t>
+          <t>None</t>
         </is>
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
-          <t>Sponsor / SHL</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="L13" s="21" t="inlineStr">
@@ -43126,34 +43126,34 @@
       </c>
       <c r="O13" s="21" t="inlineStr">
         <is>
-          <t>Gross accrued interest is the authoritative model-side SHL P&amp;L bridge.</t>
+          <t>Residual is documented rather than runtime-fixed here.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>Senior Debt</t>
         </is>
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Total OPEX</t>
+          <t>Interest</t>
         </is>
       </c>
       <c r="C14" s="21" t="inlineStr">
         <is>
-          <t>84674.77873934136</t>
+          <t>22822.816668720287</t>
         </is>
       </c>
       <c r="D14" s="21" t="inlineStr">
         <is>
-          <t>85408.27413448405</t>
+          <t>22467.388280206447</t>
         </is>
       </c>
       <c r="E14" s="21" t="inlineStr">
         <is>
-          <t>733.4953951426869</t>
+          <t>-355.4283885138393</t>
         </is>
       </c>
       <c r="F14" s="21" t="inlineStr">
@@ -43168,22 +43168,22 @@
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
-          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
+          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
         </is>
       </c>
       <c r="I14" s="21" t="inlineStr">
         <is>
-          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
+          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
         </is>
       </c>
       <c r="J14" s="21" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Review only</t>
         </is>
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Debt</t>
         </is>
       </c>
       <c r="L14" s="21" t="inlineStr">
@@ -43203,7 +43203,7 @@
       </c>
       <c r="O14" s="21" t="inlineStr">
         <is>
-          <t>Residual is documented rather than runtime-fixed here.</t>
+          <t>The residual is small relative to total debt service.</t>
         </is>
       </c>
     </row>
@@ -43215,22 +43215,22 @@
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>Interest</t>
+          <t>Debt Service</t>
         </is>
       </c>
       <c r="C15" s="21" t="inlineStr">
         <is>
-          <t>22822.816668720287</t>
+          <t>66181.34723683617</t>
         </is>
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>22467.388280206447</t>
+          <t>65826.38828020645</t>
         </is>
       </c>
       <c r="E15" s="21" t="inlineStr">
         <is>
-          <t>-355.4283885138393</t>
+          <t>-354.9589566297218</t>
         </is>
       </c>
       <c r="F15" s="21" t="inlineStr">
@@ -43245,12 +43245,12 @@
       </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
+          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
         </is>
       </c>
       <c r="I15" s="21" t="inlineStr">
         <is>
-          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
+          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
         </is>
       </c>
       <c r="J15" s="21" t="inlineStr">
@@ -43280,7 +43280,7 @@
       </c>
       <c r="O15" s="21" t="inlineStr">
         <is>
-          <t>The residual is small relative to total debt service.</t>
+          <t>Derived from existing interest and principal rows.</t>
         </is>
       </c>
     </row>
@@ -43456,12 +43456,12 @@
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>0.11587734289563015</t>
+          <t>0.11321363695747841</t>
         </is>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>-0.0002226571043698472</t>
+          <t>-0.0028863630425215864</t>
         </is>
       </c>
       <c r="F18" s="21" t="inlineStr">
@@ -43610,7 +43610,7 @@
       </c>
       <c r="D20" s="21" t="inlineStr">
         <is>
-          <t>245276.4089620228</t>
+          <t>186251.52440432477</t>
         </is>
       </c>
       <c r="E20" s="21" t="inlineStr">
@@ -43687,12 +43687,12 @@
       </c>
       <c r="D21" s="21" t="inlineStr">
         <is>
-          <t>0.115877</t>
+          <t>0.113214</t>
         </is>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
-          <t>-0.000223</t>
+          <t>-0.002886</t>
         </is>
       </c>
       <c r="F21" s="21" t="inlineStr">
@@ -44303,7 +44303,7 @@
       </c>
       <c r="D29" s="21" t="inlineStr">
         <is>
-          <t>318295.11309982045</t>
+          <t>301441.0669204517</t>
         </is>
       </c>
       <c r="E29" s="21" t="inlineStr">
@@ -44380,7 +44380,7 @@
       </c>
       <c r="D30" s="21" t="inlineStr">
         <is>
-          <t>20140.224142408744</t>
+          <t>36994.27032177761</t>
         </is>
       </c>
       <c r="E30" s="21" t="inlineStr">
@@ -44996,7 +44996,7 @@
       </c>
       <c r="D38" s="21" t="inlineStr">
         <is>
-          <t>38125.88082427603</t>
+          <t>38160.27336911231</t>
         </is>
       </c>
       <c r="E38" s="21" t="inlineStr">
@@ -45073,7 +45073,7 @@
       </c>
       <c r="D39" s="21" t="inlineStr">
         <is>
-          <t>1095711.9348782978</t>
+          <t>1078873.6179616887</t>
         </is>
       </c>
       <c r="E39" s="21" t="inlineStr">
@@ -45150,7 +45150,7 @@
       </c>
       <c r="D40" s="21" t="inlineStr">
         <is>
-          <t>1128415.624878298</t>
+          <t>1111577.3079616884</t>
         </is>
       </c>
       <c r="E40" s="21" t="inlineStr">
@@ -45227,7 +45227,7 @@
       </c>
       <c r="D41" s="21" t="inlineStr">
         <is>
-          <t>5324.32009465599</t>
+          <t>4622.641831005549</t>
         </is>
       </c>
       <c r="E41" s="21" t="inlineStr">
@@ -45304,7 +45304,7 @@
       </c>
       <c r="D42" s="21" t="inlineStr">
         <is>
-          <t>76153.89091893201</t>
+          <t>75486.60520011785</t>
         </is>
       </c>
       <c r="E42" s="21" t="inlineStr">
@@ -45458,7 +45458,7 @@
       </c>
       <c r="D44" s="21" t="inlineStr">
         <is>
-          <t>39649.75361316411</t>
+          <t>37004.37271846071</t>
         </is>
       </c>
       <c r="E44" s="21" t="inlineStr">
@@ -45478,7 +45478,7 @@
       </c>
       <c r="H44" s="21" t="inlineStr">
         <is>
-          <t>The runtime audit field exists for CIT accrual, but the committed Excel evidence pack does not include a matching row.</t>
+          <t>The runtime CIT accrual is in tax_keur, but the committed Excel evidence pack does not include a matching row.</t>
         </is>
       </c>
       <c r="I44" s="21" t="inlineStr">
@@ -45535,7 +45535,7 @@
       </c>
       <c r="D45" s="21" t="inlineStr">
         <is>
-          <t>20140.224142408744</t>
+          <t>36994.27032177761</t>
         </is>
       </c>
       <c r="E45" s="21" t="inlineStr">
@@ -45555,7 +45555,7 @@
       </c>
       <c r="H45" s="21" t="inlineStr">
         <is>
-          <t>Current-period cash tax is already exposed through runtime audit fields, but the committed Excel evidence pack has no matching line.</t>
+          <t>Current-period cash tax is in corporate_tax_cash_keur, but the committed Excel evidence pack has no matching line.</t>
         </is>
       </c>
       <c r="I45" s="21" t="inlineStr">
@@ -45612,7 +45612,7 @@
       </c>
       <c r="D46" s="21" t="inlineStr">
         <is>
-          <t>298990.5146440843</t>
+          <t>256441.33407092572</t>
         </is>
       </c>
       <c r="E46" s="21" t="inlineStr">
@@ -45689,7 +45689,7 @@
       </c>
       <c r="D47" s="21" t="inlineStr">
         <is>
-          <t>323990.5146440843</t>
+          <t>237113.0100393576</t>
         </is>
       </c>
       <c r="E47" s="21" t="inlineStr">
@@ -45766,7 +45766,7 @@
       </c>
       <c r="D48" s="21" t="inlineStr">
         <is>
-          <t>24999.999999999996</t>
+          <t>9316.339902404407</t>
         </is>
       </c>
       <c r="E48" s="21" t="inlineStr">
@@ -45843,7 +45843,7 @@
       </c>
       <c r="D49" s="21" t="inlineStr">
         <is>
-          <t>20140.224142408744</t>
+          <t>36994.27032177761</t>
         </is>
       </c>
       <c r="E49" s="21" t="inlineStr">
@@ -45997,7 +45997,7 @@
       </c>
       <c r="D51" s="21" t="inlineStr">
         <is>
-          <t>220276.40896202278</t>
+          <t>205579.8484358929</t>
         </is>
       </c>
       <c r="E51" s="21" t="inlineStr">
@@ -46074,12 +46074,12 @@
       </c>
       <c r="D52" s="21" t="inlineStr">
         <is>
-          <t>180089.48366015987</t>
+          <t>165471.11047208743</t>
         </is>
       </c>
       <c r="E52" s="21" t="inlineStr">
         <is>
-          <t>28380.090073438332</t>
+          <t>13761.716885365895</t>
         </is>
       </c>
       <c r="F52" s="21" t="inlineStr">
@@ -48100,7 +48100,7 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-05T16:17:08+00:00</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -48134,7 +48134,7 @@
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>dd4f044670c5062e420f95ef114df3f9b594e621</t>
+          <t>bad8f0b75a91ec90293d7dbc06fffe555159fe1c</t>
         </is>
       </c>
     </row>
@@ -48146,7 +48146,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>2026-07-02T08:48:06+00:00</t>
+          <t>2026-07-05T16:17:08+00:00</t>
         </is>
       </c>
     </row>
@@ -48214,7 +48214,7 @@
       </c>
       <c r="B18" s="24" t="inlineStr">
         <is>
-          <t>0.11587734289563015</t>
+          <t>0.11321363695747841</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -48294,7 +48294,7 @@
       </c>
       <c r="B22" s="24" t="inlineStr">
         <is>
-          <t>180089.48366015987</t>
+          <t>165471.11047208743</t>
         </is>
       </c>
     </row>
@@ -48386,7 +48386,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-05T16:17:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49382,7 +49382,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CNavigation&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-05T16:17:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -49432,7 +49432,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-05T16:17:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -49905,7 +49905,7 @@
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Debt Service</t>
+          <t>Senior Debt / Opening Balance</t>
         </is>
       </c>
       <c r="B31" s="41" t="inlineStr">
@@ -49915,19 +49915,19 @@
       </c>
       <c r="C31" s="21" t="inlineStr">
         <is>
-          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
+          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
         <is>
-          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
+          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Opening Balance</t>
+          <t>Senior Debt / Closing Balance</t>
         </is>
       </c>
       <c r="B32" s="41" t="inlineStr">
@@ -49937,12 +49937,12 @@
       </c>
       <c r="C32" s="21" t="inlineStr">
         <is>
-          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
+          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
-          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
+          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
         </is>
       </c>
     </row>
@@ -49990,7 +49990,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Dashboard&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-05T16:17:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -50039,7 +50039,7 @@
     <row r="3">
       <c r="A3" s="28" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-02T08:48:06+00:00 | Workbook version: Phase 11 institutional export polish</t>
+          <t>Generated: 2026-07-05T16:17:08+00:00 | Workbook version: Phase 11 institutional export polish</t>
         </is>
       </c>
     </row>
@@ -50129,7 +50129,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.11587734289563015</t>
+          <t>0.11321363695747841</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -50399,7 +50399,7 @@
     <row r="22">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Debt Service</t>
+          <t>Senior Debt / Opening Balance</t>
         </is>
       </c>
       <c r="B22" s="41" t="inlineStr">
@@ -50409,12 +50409,12 @@
       </c>
       <c r="C22" s="21" t="inlineStr">
         <is>
-          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
+          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
         <is>
-          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
+          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -50426,7 +50426,7 @@
     <row r="23">
       <c r="A23" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Opening Balance</t>
+          <t>Senior Debt / Closing Balance</t>
         </is>
       </c>
       <c r="B23" s="41" t="inlineStr">
@@ -50436,12 +50436,12 @@
       </c>
       <c r="C23" s="21" t="inlineStr">
         <is>
-          <t>The committed Excel bridge and runtime schedule do not share the same opening-balance cut point for the operational horizon.</t>
+          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
         </is>
       </c>
       <c r="D23" s="21" t="inlineStr">
         <is>
-          <t>Keep the opening balance row as a reconciliation aid and rely on principal, interest, and closing rows for authoritative debt behavior.</t>
+          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -50453,7 +50453,7 @@
     <row r="24">
       <c r="A24" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Closing Balance</t>
+          <t>SHL / Principal Repaid</t>
         </is>
       </c>
       <c r="B24" s="41" t="inlineStr">
@@ -50463,12 +50463,12 @@
       </c>
       <c r="C24" s="21" t="inlineStr">
         <is>
-          <t>Closing balance drift follows from the opening-balance cut-point difference carried through the operational bridge.</t>
+          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
         </is>
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>Use this row for reviewer traceability only; core runtime debt outputs remain unchanged.</t>
+          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -50485,7 +50485,7 @@
     <row r="25">
       <c r="A25" s="21" t="inlineStr">
         <is>
-          <t>SHL / Principal Repaid</t>
+          <t>SHL / Gross Accrued Interest</t>
         </is>
       </c>
       <c r="B25" s="41" t="inlineStr">
@@ -50495,12 +50495,12 @@
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>SHL principal timing moved closer to Excel after the controlled alignment work, but committed bridge totals still reflect a slightly different period framing.</t>
+          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
         <is>
-          <t>Document as a timing reconciliation item and keep the runtime-alignment branch as the authoritative history.</t>
+          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
         </is>
       </c>
       <c r="F25" s="22" t="inlineStr">
@@ -50512,7 +50512,7 @@
     <row r="26">
       <c r="A26" s="21" t="inlineStr">
         <is>
-          <t>SHL / Gross Accrued Interest</t>
+          <t>OPEX / Total OPEX</t>
         </is>
       </c>
       <c r="B26" s="41" t="inlineStr">
@@ -50522,12 +50522,12 @@
       </c>
       <c r="C26" s="21" t="inlineStr">
         <is>
-          <t>The remaining SHL gross-interest delta reflects timing and presentation differences between the committed bridge and the runtime accrued-interest schedule.</t>
+          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
         </is>
       </c>
       <c r="D26" s="21" t="inlineStr">
         <is>
-          <t>Keep the row visible for reviewer scrutiny, but do not redesign SHL mechanics in this branch.</t>
+          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -50544,7 +50544,7 @@
     <row r="27">
       <c r="A27" s="21" t="inlineStr">
         <is>
-          <t>OPEX / Total OPEX</t>
+          <t>Senior Debt / Interest</t>
         </is>
       </c>
       <c r="B27" s="41" t="inlineStr">
@@ -50554,12 +50554,12 @@
       </c>
       <c r="C27" s="21" t="inlineStr">
         <is>
-          <t>Known local-tax and minor-row grouping residual from prior calibration review.</t>
+          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
         <is>
-          <t>Keep grouped unless a dedicated OPEX sub-line evidence branch is requested.</t>
+          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -50576,7 +50576,7 @@
     <row r="28">
       <c r="A28" s="21" t="inlineStr">
         <is>
-          <t>Senior Debt / Interest</t>
+          <t>Senior Debt / Debt Service</t>
         </is>
       </c>
       <c r="B28" s="41" t="inlineStr">
@@ -50586,12 +50586,12 @@
       </c>
       <c r="C28" s="21" t="inlineStr">
         <is>
-          <t>A small timing and day-count residual remains between the committed Excel extract and runtime debt schedule.</t>
+          <t>Debt service inherits the same minor interest timing residual visible in the senior interest row.</t>
         </is>
       </c>
       <c r="D28" s="21" t="inlineStr">
         <is>
-          <t>Document as a minor review residual unless lenders ask for a debt-source extraction refresh.</t>
+          <t>Keep this as a transparent review delta rather than a model-fix candidate.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -50638,7 +50638,7 @@
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;LTUHO Wind 1&amp;CExecutive Summary&amp;RPhase 11 institutional export polish</oddHeader>
-    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-02T08:48:06+00:00</oddFooter>
+    <oddFooter>&amp;LTUHO Wind 1 | institutional review pack&amp;Creview&amp;R2026-07-05T16:17:08+00:00</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>